<commit_message>
RPA datasets push 2024-08-10
</commit_message>
<xml_diff>
--- a/datasets/ib-strategy-data.xlsx
+++ b/datasets/ib-strategy-data.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="235">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="237">
   <si>
     <t>수요예측(시작일)</t>
   </si>
@@ -614,6 +614,12 @@
     <t>2000</t>
   </si>
   <si>
+    <t>15300</t>
+  </si>
+  <si>
+    <t>16000</t>
+  </si>
+  <si>
     <t>13000</t>
   </si>
   <si>
@@ -629,9 +635,6 @@
     <t>21000</t>
   </si>
   <si>
-    <t>16000</t>
-  </si>
-  <si>
     <t>10000</t>
   </si>
   <si>
@@ -653,7 +656,10 @@
     <t>78720</t>
   </si>
   <si>
-    <t>21308</t>
+    <t>23972</t>
+  </si>
+  <si>
+    <t>24000</t>
   </si>
   <si>
     <t>21700</t>
@@ -2818,10 +2824,10 @@
         <v>117</v>
       </c>
       <c r="E2" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="F2" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -2841,7 +2847,7 @@
         <v>117</v>
       </c>
       <c r="F3" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -2858,10 +2864,10 @@
         <v>117</v>
       </c>
       <c r="E4" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="F4" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -2878,10 +2884,10 @@
         <v>117</v>
       </c>
       <c r="E5" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="F5" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -2898,10 +2904,10 @@
         <v>117</v>
       </c>
       <c r="E6" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="F6" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -2918,10 +2924,10 @@
         <v>198</v>
       </c>
       <c r="E7" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="F7" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -2935,13 +2941,13 @@
         <v>188</v>
       </c>
       <c r="D8" t="s">
-        <v>117</v>
+        <v>199</v>
       </c>
       <c r="E8" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="F8" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -2955,13 +2961,13 @@
         <v>189</v>
       </c>
       <c r="D9" t="s">
-        <v>117</v>
+        <v>200</v>
       </c>
       <c r="E9" t="s">
-        <v>201</v>
+        <v>214</v>
       </c>
       <c r="F9" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -2975,13 +2981,13 @@
         <v>190</v>
       </c>
       <c r="D10" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="E10" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="F10" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -2995,13 +3001,13 @@
         <v>191</v>
       </c>
       <c r="D11" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="E11" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="F11" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -3015,13 +3021,13 @@
         <v>192</v>
       </c>
       <c r="D12" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="E12" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="F12" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -3038,10 +3044,10 @@
         <v>198</v>
       </c>
       <c r="E13" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="F13" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -3055,13 +3061,13 @@
         <v>193</v>
       </c>
       <c r="D14" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="E14" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="F14" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -3075,13 +3081,13 @@
         <v>184</v>
       </c>
       <c r="D15" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="E15" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="F15" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -3095,13 +3101,13 @@
         <v>194</v>
       </c>
       <c r="D16" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="E16" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="F16" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -3115,13 +3121,13 @@
         <v>195</v>
       </c>
       <c r="D17" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="E17" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="F17" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
     </row>
     <row r="18" spans="1:6">
@@ -3135,13 +3141,13 @@
         <v>196</v>
       </c>
       <c r="D18" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="E18" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="F18" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
     </row>
     <row r="19" spans="1:6">
@@ -3158,10 +3164,10 @@
         <v>198</v>
       </c>
       <c r="E19" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="F19" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -3178,10 +3184,10 @@
         <v>198</v>
       </c>
       <c r="E20" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="F20" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -3195,13 +3201,13 @@
         <v>197</v>
       </c>
       <c r="D21" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="E21" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="F21" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
RPA datasets push 2024-08-12
</commit_message>
<xml_diff>
--- a/datasets/ib-strategy-data.xlsx
+++ b/datasets/ib-strategy-data.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="237">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="242">
   <si>
     <t>수요예측(시작일)</t>
   </si>
@@ -92,6 +92,9 @@
     <t>주요제품</t>
   </si>
   <si>
+    <t>2024-07-23</t>
+  </si>
+  <si>
     <t>2024-07-15</t>
   </si>
   <si>
@@ -140,6 +143,9 @@
     <t>2024-05-23</t>
   </si>
   <si>
+    <t>2024-07-29</t>
+  </si>
+  <si>
     <t>2024-07-19</t>
   </si>
   <si>
@@ -164,15 +170,15 @@
     <t>2024-05-29</t>
   </si>
   <si>
+    <t>2024-07-25</t>
+  </si>
+  <si>
     <t>2024-08-06</t>
   </si>
   <si>
     <t>2024-07-26</t>
   </si>
   <si>
-    <t>2024-07-25</t>
-  </si>
-  <si>
     <t>2024-07-12</t>
   </si>
   <si>
@@ -200,6 +206,9 @@
     <t>2024-07-01</t>
   </si>
   <si>
+    <t>미래</t>
+  </si>
+  <si>
     <t>삼성</t>
   </si>
   <si>
@@ -218,9 +227,6 @@
     <t>엘에스</t>
   </si>
   <si>
-    <t>미래</t>
-  </si>
-  <si>
     <t>한국</t>
   </si>
   <si>
@@ -236,6 +242,9 @@
     <t>신한, 한국</t>
   </si>
   <si>
+    <t>뱅크웨어글로벌</t>
+  </si>
+  <si>
     <t>아이빔테크놀로지</t>
   </si>
   <si>
@@ -299,6 +308,9 @@
     <t>신한글로벌액티브리츠</t>
   </si>
   <si>
+    <t>155.74:1</t>
+  </si>
+  <si>
     <t>1011.50:1</t>
   </si>
   <si>
@@ -362,6 +374,9 @@
     <t>38.7:1</t>
   </si>
   <si>
+    <t>1.52%</t>
+  </si>
+  <si>
     <t>0.49%</t>
   </si>
   <si>
@@ -398,6 +413,9 @@
     <t>0.95%</t>
   </si>
   <si>
+    <t>국내외 은행 및 금융기업 대상 코어뱅킹 소프트웨어</t>
+  </si>
+  <si>
     <t>생체현미경, CRO 서비스</t>
   </si>
   <si>
@@ -504,9 +522,6 @@
   </si>
   <si>
     <t>유라클</t>
-  </si>
-  <si>
-    <t>뱅크웨어글로벌</t>
   </si>
   <si>
     <t>NH스팩31호</t>
@@ -1083,7 +1098,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Y22"/>
+  <dimension ref="A1:Y23"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:25">
@@ -1168,76 +1183,76 @@
         <v>25</v>
       </c>
       <c r="B2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="E2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F2">
-        <v>2234000</v>
+        <v>1400000</v>
       </c>
       <c r="G2">
-        <v>2234000</v>
+        <v>1400000</v>
       </c>
       <c r="H2">
         <v>0</v>
       </c>
       <c r="I2">
-        <v>7300</v>
+        <v>16000</v>
       </c>
       <c r="J2">
-        <v>8500</v>
+        <v>19000</v>
       </c>
       <c r="K2">
-        <v>14965620</v>
+        <v>10000988</v>
       </c>
       <c r="L2">
         <v>0</v>
       </c>
       <c r="M2">
-        <v>10000</v>
+        <v>16000</v>
       </c>
       <c r="N2" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="O2" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="P2">
-        <v>1337894447</v>
+        <v>72895458363</v>
       </c>
       <c r="Q2">
-        <v>4495088983</v>
+        <v>72913766913</v>
       </c>
       <c r="R2">
-        <v>99398351</v>
+        <v>11230711680</v>
       </c>
       <c r="S2">
-        <v>-3330678562</v>
+        <v>-6524077412</v>
       </c>
       <c r="T2">
-        <v>-2905069801</v>
+        <v>-4556157069</v>
       </c>
       <c r="U2">
-        <v>-1314068310</v>
+        <v>-3633759729</v>
       </c>
       <c r="V2">
-        <v>-9735376868</v>
+        <v>-11528915410</v>
       </c>
       <c r="W2">
-        <v>-5043515600</v>
+        <v>-7978634776</v>
       </c>
       <c r="X2">
-        <v>-1257080998</v>
+        <v>-3801868433</v>
       </c>
       <c r="Y2" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
     </row>
     <row r="3" spans="1:25">
@@ -1245,76 +1260,76 @@
         <v>26</v>
       </c>
       <c r="B3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C3" t="s">
-        <v>42</v>
+        <v>52</v>
       </c>
       <c r="D3" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F3">
-        <v>1350000</v>
+        <v>2234000</v>
       </c>
       <c r="G3">
-        <v>1350000</v>
+        <v>2234000</v>
       </c>
       <c r="H3">
         <v>0</v>
       </c>
       <c r="I3">
-        <v>14000</v>
+        <v>7300</v>
       </c>
       <c r="J3">
-        <v>17000</v>
+        <v>8500</v>
       </c>
       <c r="K3">
-        <v>6471740</v>
+        <v>14965620</v>
       </c>
       <c r="L3">
         <v>0</v>
       </c>
       <c r="M3">
-        <v>22000</v>
+        <v>10000</v>
       </c>
       <c r="N3" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="O3" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="P3">
-        <v>5214628820</v>
+        <v>1337894447</v>
       </c>
       <c r="Q3">
-        <v>6009352447</v>
+        <v>4495088983</v>
       </c>
       <c r="R3">
-        <v>965797975</v>
+        <v>99398351</v>
       </c>
       <c r="S3">
-        <v>2015081728</v>
+        <v>-3330678562</v>
       </c>
       <c r="T3">
-        <v>1319755337</v>
+        <v>-2905069801</v>
       </c>
       <c r="U3">
-        <v>-44547594</v>
+        <v>-1314068310</v>
       </c>
       <c r="V3">
-        <v>1503069100</v>
+        <v>-9735376868</v>
       </c>
       <c r="W3">
-        <v>1410469786</v>
+        <v>-5043515600</v>
       </c>
       <c r="X3">
-        <v>24178632</v>
+        <v>-1257080998</v>
       </c>
       <c r="Y3" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
     </row>
     <row r="4" spans="1:25">
@@ -1322,99 +1337,99 @@
         <v>27</v>
       </c>
       <c r="B4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C4" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="D4" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="E4" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="F4">
-        <v>6000000</v>
+        <v>1350000</v>
       </c>
       <c r="G4">
-        <v>6000000</v>
+        <v>1350000</v>
       </c>
       <c r="H4">
         <v>0</v>
       </c>
       <c r="I4">
-        <v>2000</v>
+        <v>14000</v>
       </c>
       <c r="J4">
-        <v>2000</v>
+        <v>17000</v>
       </c>
       <c r="K4">
-        <v>6345000</v>
+        <v>6471740</v>
       </c>
       <c r="L4">
         <v>0</v>
       </c>
       <c r="M4">
-        <v>2000</v>
+        <v>22000</v>
       </c>
       <c r="N4" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="O4" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="P4">
-        <v>0</v>
+        <v>5214628820</v>
       </c>
       <c r="Q4">
-        <v>0</v>
+        <v>6009352447</v>
       </c>
       <c r="R4">
-        <v>0</v>
+        <v>965797975</v>
       </c>
       <c r="S4">
-        <v>0</v>
+        <v>2015081728</v>
       </c>
       <c r="T4">
-        <v>0</v>
+        <v>1319755337</v>
       </c>
       <c r="U4">
-        <v>0</v>
+        <v>-44547594</v>
       </c>
       <c r="V4">
-        <v>0</v>
+        <v>1503069100</v>
       </c>
       <c r="W4">
-        <v>0</v>
+        <v>1410469786</v>
       </c>
       <c r="X4">
-        <v>0</v>
+        <v>24178632</v>
       </c>
       <c r="Y4" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
     </row>
     <row r="5" spans="1:25">
       <c r="A5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B5" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C5" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D5" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E5" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="F5">
-        <v>4000000</v>
+        <v>6000000</v>
       </c>
       <c r="G5">
-        <v>4000000</v>
+        <v>6000000</v>
       </c>
       <c r="H5">
         <v>0</v>
@@ -1426,7 +1441,7 @@
         <v>2000</v>
       </c>
       <c r="K5">
-        <v>4420000</v>
+        <v>6345000</v>
       </c>
       <c r="L5">
         <v>0</v>
@@ -1435,10 +1450,10 @@
         <v>2000</v>
       </c>
       <c r="N5" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="O5" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="P5">
         <v>0</v>
@@ -1468,7 +1483,7 @@
         <v>0</v>
       </c>
       <c r="Y5" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
     </row>
     <row r="6" spans="1:25">
@@ -1476,46 +1491,46 @@
         <v>28</v>
       </c>
       <c r="B6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C6" t="s">
-        <v>25</v>
+        <v>51</v>
       </c>
       <c r="D6" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E6" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="F6">
-        <v>1618000</v>
+        <v>4000000</v>
       </c>
       <c r="G6">
-        <v>1618000</v>
+        <v>4000000</v>
       </c>
       <c r="H6">
         <v>0</v>
       </c>
       <c r="I6">
-        <v>6200</v>
+        <v>2000</v>
       </c>
       <c r="J6">
-        <v>7700</v>
+        <v>2000</v>
       </c>
       <c r="K6">
-        <v>10830212</v>
+        <v>4420000</v>
       </c>
       <c r="L6">
         <v>0</v>
       </c>
       <c r="M6">
-        <v>10000</v>
+        <v>2000</v>
       </c>
       <c r="N6" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="O6" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="P6">
         <v>0</v>
@@ -1545,7 +1560,7 @@
         <v>0</v>
       </c>
       <c r="Y6" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
     </row>
     <row r="7" spans="1:25">
@@ -1553,46 +1568,46 @@
         <v>29</v>
       </c>
       <c r="B7" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C7" t="s">
-        <v>52</v>
+        <v>26</v>
       </c>
       <c r="D7" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E7" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="F7">
-        <v>4000000</v>
+        <v>1618000</v>
       </c>
       <c r="G7">
-        <v>4000000</v>
+        <v>1618000</v>
       </c>
       <c r="H7">
         <v>0</v>
       </c>
       <c r="I7">
-        <v>2000</v>
+        <v>6200</v>
       </c>
       <c r="J7">
-        <v>2000</v>
+        <v>7700</v>
       </c>
       <c r="K7">
-        <v>5020000</v>
+        <v>10830212</v>
       </c>
       <c r="L7">
         <v>0</v>
       </c>
       <c r="M7">
-        <v>2000</v>
+        <v>10000</v>
       </c>
       <c r="N7" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="O7" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="P7">
         <v>0</v>
@@ -1622,7 +1637,7 @@
         <v>0</v>
       </c>
       <c r="Y7" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
     </row>
     <row r="8" spans="1:25">
@@ -1630,76 +1645,76 @@
         <v>30</v>
       </c>
       <c r="B8" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C8" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D8" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="E8" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="F8">
-        <v>1810000</v>
+        <v>4000000</v>
       </c>
       <c r="G8">
-        <v>1810000</v>
+        <v>4000000</v>
       </c>
       <c r="H8">
         <v>0</v>
       </c>
       <c r="I8">
-        <v>9000</v>
+        <v>2000</v>
       </c>
       <c r="J8">
-        <v>12000</v>
+        <v>2000</v>
       </c>
       <c r="K8">
-        <v>7836009</v>
+        <v>5020000</v>
       </c>
       <c r="L8">
         <v>0</v>
       </c>
       <c r="M8">
-        <v>16000</v>
+        <v>2000</v>
       </c>
       <c r="N8" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="O8" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="P8">
-        <v>12596039842</v>
+        <v>0</v>
       </c>
       <c r="Q8">
-        <v>14910346438</v>
+        <v>0</v>
       </c>
       <c r="R8">
-        <v>16039074617</v>
+        <v>0</v>
       </c>
       <c r="S8">
-        <v>1732604466</v>
+        <v>0</v>
       </c>
       <c r="T8">
-        <v>2893667787</v>
+        <v>0</v>
       </c>
       <c r="U8">
-        <v>1613779678</v>
+        <v>0</v>
       </c>
       <c r="V8">
-        <v>1558081149</v>
+        <v>0</v>
       </c>
       <c r="W8">
-        <v>2643467726</v>
+        <v>0</v>
       </c>
       <c r="X8">
-        <v>1795726428</v>
+        <v>0</v>
       </c>
       <c r="Y8" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
     </row>
     <row r="9" spans="1:25">
@@ -1707,76 +1722,76 @@
         <v>31</v>
       </c>
       <c r="B9" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C9" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D9" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="E9" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="F9">
-        <v>1330000</v>
+        <v>1810000</v>
       </c>
       <c r="G9">
-        <v>1330000</v>
+        <v>1810000</v>
       </c>
       <c r="H9">
         <v>0</v>
       </c>
       <c r="I9">
-        <v>36400</v>
+        <v>9000</v>
       </c>
       <c r="J9">
-        <v>43300</v>
+        <v>12000</v>
       </c>
       <c r="K9">
-        <v>9375694</v>
+        <v>7836009</v>
       </c>
       <c r="L9">
         <v>0</v>
       </c>
       <c r="M9">
-        <v>43300</v>
+        <v>16000</v>
       </c>
       <c r="N9" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="O9" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="P9">
-        <v>103267682</v>
+        <v>12596039842</v>
       </c>
       <c r="Q9">
-        <v>342201581</v>
+        <v>14910346438</v>
       </c>
       <c r="R9">
-        <v>231425455</v>
+        <v>16039074617</v>
       </c>
       <c r="S9">
-        <v>-7598692896</v>
+        <v>1732604466</v>
       </c>
       <c r="T9">
-        <v>-25822444575</v>
+        <v>2893667787</v>
       </c>
       <c r="U9">
-        <v>-15929213281</v>
+        <v>1613779678</v>
       </c>
       <c r="V9">
-        <v>-6973258680</v>
+        <v>1558081149</v>
       </c>
       <c r="W9">
-        <v>-48433907514</v>
+        <v>2643467726</v>
       </c>
       <c r="X9">
-        <v>-83246975113</v>
+        <v>1795726428</v>
       </c>
       <c r="Y9" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
     </row>
     <row r="10" spans="1:25">
@@ -1784,76 +1799,76 @@
         <v>32</v>
       </c>
       <c r="B10" t="s">
-        <v>30</v>
+        <v>48</v>
       </c>
       <c r="C10" t="s">
-        <v>29</v>
+        <v>56</v>
       </c>
       <c r="D10" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="E10" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="F10">
-        <v>3400000</v>
+        <v>1330000</v>
       </c>
       <c r="G10">
-        <v>3400000</v>
+        <v>1330000</v>
       </c>
       <c r="H10">
         <v>0</v>
       </c>
       <c r="I10">
-        <v>4500</v>
+        <v>36400</v>
       </c>
       <c r="J10">
-        <v>5500</v>
+        <v>43300</v>
       </c>
       <c r="K10">
-        <v>30888000</v>
+        <v>9375694</v>
       </c>
       <c r="L10">
         <v>0</v>
       </c>
       <c r="M10">
-        <v>7000</v>
+        <v>43300</v>
       </c>
       <c r="N10" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="O10" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="P10">
-        <v>85187882584</v>
+        <v>103267682</v>
       </c>
       <c r="Q10">
-        <v>87525689695</v>
+        <v>342201581</v>
       </c>
       <c r="R10">
-        <v>77247394706</v>
+        <v>231425455</v>
       </c>
       <c r="S10">
-        <v>2205797752</v>
+        <v>-7598692896</v>
       </c>
       <c r="T10">
-        <v>4920387020</v>
+        <v>-25822444575</v>
       </c>
       <c r="U10">
-        <v>4336496285</v>
+        <v>-15929213281</v>
       </c>
       <c r="V10">
-        <v>1613954566</v>
+        <v>-6973258680</v>
       </c>
       <c r="W10">
-        <v>3980493669</v>
+        <v>-48433907514</v>
       </c>
       <c r="X10">
-        <v>2646634321</v>
+        <v>-83246975113</v>
       </c>
       <c r="Y10" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
     </row>
     <row r="11" spans="1:25">
@@ -1864,73 +1879,73 @@
         <v>31</v>
       </c>
       <c r="C11" t="s">
-        <v>55</v>
+        <v>30</v>
       </c>
       <c r="D11" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E11" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F11">
-        <v>6250000</v>
+        <v>3400000</v>
       </c>
       <c r="G11">
-        <v>6250000</v>
+        <v>3400000</v>
       </c>
       <c r="H11">
         <v>0</v>
       </c>
       <c r="I11">
-        <v>2000</v>
+        <v>4500</v>
       </c>
       <c r="J11">
-        <v>2000</v>
+        <v>5500</v>
       </c>
       <c r="K11">
-        <v>6870000</v>
+        <v>30888000</v>
       </c>
       <c r="L11">
         <v>0</v>
       </c>
       <c r="M11">
-        <v>2000</v>
+        <v>7000</v>
       </c>
       <c r="N11" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="O11" t="s">
-        <v>117</v>
+        <v>126</v>
       </c>
       <c r="P11">
-        <v>0</v>
+        <v>85187882584</v>
       </c>
       <c r="Q11">
-        <v>0</v>
+        <v>87525689695</v>
       </c>
       <c r="R11">
-        <v>0</v>
+        <v>77247394706</v>
       </c>
       <c r="S11">
-        <v>0</v>
+        <v>2205797752</v>
       </c>
       <c r="T11">
-        <v>0</v>
+        <v>4920387020</v>
       </c>
       <c r="U11">
-        <v>0</v>
+        <v>4336496285</v>
       </c>
       <c r="V11">
-        <v>0</v>
+        <v>1613954566</v>
       </c>
       <c r="W11">
-        <v>0</v>
+        <v>3980493669</v>
       </c>
       <c r="X11">
-        <v>0</v>
+        <v>2646634321</v>
       </c>
       <c r="Y11" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
     </row>
     <row r="12" spans="1:25">
@@ -1938,43 +1953,43 @@
         <v>34</v>
       </c>
       <c r="B12" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C12" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D12" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E12" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F12">
-        <v>2000000</v>
+        <v>6250000</v>
       </c>
       <c r="G12">
-        <v>2000000</v>
+        <v>6250000</v>
       </c>
       <c r="H12">
         <v>0</v>
       </c>
       <c r="I12">
-        <v>7500</v>
+        <v>2000</v>
       </c>
       <c r="J12">
-        <v>9000</v>
+        <v>2000</v>
       </c>
       <c r="K12">
-        <v>17529140</v>
+        <v>6870000</v>
       </c>
       <c r="L12">
         <v>0</v>
       </c>
       <c r="M12">
-        <v>11500</v>
+        <v>2000</v>
       </c>
       <c r="N12" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="O12" t="s">
         <v>122</v>
@@ -2007,7 +2022,7 @@
         <v>0</v>
       </c>
       <c r="Y12" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
     </row>
     <row r="13" spans="1:25">
@@ -2015,46 +2030,46 @@
         <v>35</v>
       </c>
       <c r="B13" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C13" t="s">
-        <v>28</v>
+        <v>58</v>
       </c>
       <c r="D13" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="E13" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="F13">
-        <v>6450000</v>
+        <v>2000000</v>
       </c>
       <c r="G13">
-        <v>6450000</v>
+        <v>2000000</v>
       </c>
       <c r="H13">
         <v>0</v>
       </c>
       <c r="I13">
-        <v>2000</v>
+        <v>7500</v>
       </c>
       <c r="J13">
-        <v>2000</v>
+        <v>9000</v>
       </c>
       <c r="K13">
-        <v>6930000</v>
+        <v>17529140</v>
       </c>
       <c r="L13">
         <v>0</v>
       </c>
       <c r="M13">
-        <v>2000</v>
+        <v>11500</v>
       </c>
       <c r="N13" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="O13" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
       <c r="P13">
         <v>0</v>
@@ -2084,7 +2099,7 @@
         <v>0</v>
       </c>
       <c r="Y13" t="s">
-        <v>135</v>
+        <v>142</v>
       </c>
     </row>
     <row r="14" spans="1:25">
@@ -2092,22 +2107,22 @@
         <v>36</v>
       </c>
       <c r="B14" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C14" t="s">
-        <v>57</v>
+        <v>29</v>
       </c>
       <c r="D14" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="E14" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="F14">
-        <v>6000000</v>
+        <v>6450000</v>
       </c>
       <c r="G14">
-        <v>6000000</v>
+        <v>6450000</v>
       </c>
       <c r="H14">
         <v>0</v>
@@ -2119,7 +2134,7 @@
         <v>2000</v>
       </c>
       <c r="K14">
-        <v>6220000</v>
+        <v>6930000</v>
       </c>
       <c r="L14">
         <v>0</v>
@@ -2128,10 +2143,10 @@
         <v>2000</v>
       </c>
       <c r="N14" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="O14" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="P14">
         <v>0</v>
@@ -2161,30 +2176,30 @@
         <v>0</v>
       </c>
       <c r="Y14" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
     </row>
     <row r="15" spans="1:25">
       <c r="A15" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="B15" t="s">
         <v>36</v>
       </c>
       <c r="C15" t="s">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="D15" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="E15" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="F15">
-        <v>4000000</v>
+        <v>6000000</v>
       </c>
       <c r="G15">
-        <v>4000000</v>
+        <v>6000000</v>
       </c>
       <c r="H15">
         <v>0</v>
@@ -2196,7 +2211,7 @@
         <v>2000</v>
       </c>
       <c r="K15">
-        <v>4810000</v>
+        <v>6220000</v>
       </c>
       <c r="L15">
         <v>0</v>
@@ -2205,10 +2220,10 @@
         <v>2000</v>
       </c>
       <c r="N15" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="O15" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="P15">
         <v>0</v>
@@ -2238,30 +2253,30 @@
         <v>0</v>
       </c>
       <c r="Y15" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
     </row>
     <row r="16" spans="1:25">
       <c r="A16" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B16" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C16" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D16" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="E16" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="F16">
-        <v>4750000</v>
+        <v>4000000</v>
       </c>
       <c r="G16">
-        <v>4750000</v>
+        <v>4000000</v>
       </c>
       <c r="H16">
         <v>0</v>
@@ -2273,7 +2288,7 @@
         <v>2000</v>
       </c>
       <c r="K16">
-        <v>5480000</v>
+        <v>4810000</v>
       </c>
       <c r="L16">
         <v>0</v>
@@ -2282,10 +2297,10 @@
         <v>2000</v>
       </c>
       <c r="N16" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="O16" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="P16">
         <v>0</v>
@@ -2315,84 +2330,84 @@
         <v>0</v>
       </c>
       <c r="Y16" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
     </row>
     <row r="17" spans="1:25">
       <c r="A17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17" t="s">
         <v>37</v>
       </c>
-      <c r="B17" t="s">
+      <c r="C17" t="s">
         <v>47</v>
       </c>
-      <c r="C17" t="s">
-        <v>45</v>
-      </c>
       <c r="D17" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="E17" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F17">
-        <v>1300000</v>
+        <v>4750000</v>
       </c>
       <c r="G17">
-        <v>1300000</v>
+        <v>4750000</v>
       </c>
       <c r="H17">
         <v>0</v>
       </c>
       <c r="I17">
-        <v>10500</v>
+        <v>2000</v>
       </c>
       <c r="J17">
-        <v>14000</v>
+        <v>2000</v>
       </c>
       <c r="K17">
-        <v>12293880</v>
+        <v>5480000</v>
       </c>
       <c r="L17">
         <v>0</v>
       </c>
       <c r="M17">
-        <v>17000</v>
+        <v>2000</v>
       </c>
       <c r="N17" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="O17" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="P17">
-        <v>1386123525</v>
+        <v>0</v>
       </c>
       <c r="Q17">
-        <v>1152944128</v>
+        <v>0</v>
       </c>
       <c r="R17">
-        <v>1885010467</v>
+        <v>0</v>
       </c>
       <c r="S17">
-        <v>-4388824706</v>
+        <v>0</v>
       </c>
       <c r="T17">
-        <v>-7990287699</v>
+        <v>0</v>
       </c>
       <c r="U17">
-        <v>-9803411085</v>
+        <v>0</v>
       </c>
       <c r="V17">
-        <v>-4430563401</v>
+        <v>0</v>
       </c>
       <c r="W17">
-        <v>-7988275689</v>
+        <v>0</v>
       </c>
       <c r="X17">
-        <v>-9916946238</v>
+        <v>0</v>
       </c>
       <c r="Y17" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
     </row>
     <row r="18" spans="1:25">
@@ -2400,230 +2415,230 @@
         <v>38</v>
       </c>
       <c r="B18" t="s">
-        <v>35</v>
+        <v>49</v>
       </c>
       <c r="C18" t="s">
-        <v>28</v>
+        <v>47</v>
       </c>
       <c r="D18" t="s">
         <v>70</v>
       </c>
       <c r="E18" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="F18">
-        <v>1600000</v>
+        <v>1300000</v>
       </c>
       <c r="G18">
-        <v>1600000</v>
+        <v>1300000</v>
       </c>
       <c r="H18">
         <v>0</v>
       </c>
       <c r="I18">
-        <v>20000</v>
+        <v>10500</v>
       </c>
       <c r="J18">
-        <v>23500</v>
+        <v>14000</v>
       </c>
       <c r="K18">
-        <v>8751446</v>
+        <v>12293880</v>
       </c>
       <c r="L18">
         <v>0</v>
       </c>
       <c r="M18">
-        <v>30000</v>
+        <v>17000</v>
       </c>
       <c r="N18" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="O18" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="P18">
-        <v>0</v>
+        <v>1386123525</v>
       </c>
       <c r="Q18">
-        <v>0</v>
+        <v>1152944128</v>
       </c>
       <c r="R18">
-        <v>0</v>
+        <v>1885010467</v>
       </c>
       <c r="S18">
-        <v>0</v>
+        <v>-4388824706</v>
       </c>
       <c r="T18">
-        <v>0</v>
+        <v>-7990287699</v>
       </c>
       <c r="U18">
-        <v>0</v>
+        <v>-9803411085</v>
       </c>
       <c r="V18">
-        <v>0</v>
+        <v>-4430563401</v>
       </c>
       <c r="W18">
-        <v>0</v>
+        <v>-7988275689</v>
       </c>
       <c r="X18">
-        <v>0</v>
+        <v>-9916946238</v>
       </c>
       <c r="Y18" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
     </row>
     <row r="19" spans="1:25">
       <c r="A19" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B19" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="C19" t="s">
-        <v>46</v>
+        <v>29</v>
       </c>
       <c r="D19" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="E19" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F19">
-        <v>1298000</v>
+        <v>1600000</v>
       </c>
       <c r="G19">
-        <v>1298000</v>
+        <v>1600000</v>
       </c>
       <c r="H19">
         <v>0</v>
       </c>
       <c r="I19">
-        <v>10400</v>
+        <v>20000</v>
       </c>
       <c r="J19">
-        <v>12700</v>
+        <v>23500</v>
       </c>
       <c r="K19">
-        <v>8650735</v>
+        <v>8751446</v>
       </c>
       <c r="L19">
         <v>0</v>
       </c>
       <c r="M19">
-        <v>16000</v>
+        <v>30000</v>
       </c>
       <c r="N19" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="O19" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="P19">
-        <v>2055746777</v>
+        <v>0</v>
       </c>
       <c r="Q19">
-        <v>2918221978</v>
+        <v>0</v>
       </c>
       <c r="R19">
-        <v>979078233</v>
+        <v>0</v>
       </c>
       <c r="S19">
-        <v>-3343774083</v>
+        <v>0</v>
       </c>
       <c r="T19">
-        <v>-3525649863</v>
+        <v>0</v>
       </c>
       <c r="U19">
-        <v>-1713494359</v>
+        <v>0</v>
       </c>
       <c r="V19">
-        <v>-4430074915</v>
+        <v>0</v>
       </c>
       <c r="W19">
-        <v>-8304699942</v>
+        <v>0</v>
       </c>
       <c r="X19">
-        <v>-1627684107</v>
+        <v>0</v>
       </c>
       <c r="Y19" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
     </row>
     <row r="20" spans="1:25">
       <c r="A20" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B20" t="s">
+        <v>49</v>
+      </c>
+      <c r="C20" t="s">
         <v>48</v>
       </c>
-      <c r="C20" t="s">
-        <v>58</v>
-      </c>
       <c r="D20" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="E20" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="F20">
-        <v>5000000</v>
+        <v>1298000</v>
       </c>
       <c r="G20">
-        <v>5000000</v>
+        <v>1298000</v>
       </c>
       <c r="H20">
         <v>0</v>
       </c>
       <c r="I20">
-        <v>2000</v>
+        <v>10400</v>
       </c>
       <c r="J20">
-        <v>2000</v>
+        <v>12700</v>
       </c>
       <c r="K20">
-        <v>5840000</v>
+        <v>8650735</v>
       </c>
       <c r="L20">
         <v>0</v>
       </c>
       <c r="M20">
-        <v>2000</v>
+        <v>16000</v>
       </c>
       <c r="N20" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="O20" t="s">
-        <v>117</v>
+        <v>130</v>
       </c>
       <c r="P20">
-        <v>0</v>
+        <v>2055746777</v>
       </c>
       <c r="Q20">
-        <v>0</v>
+        <v>2918221978</v>
       </c>
       <c r="R20">
-        <v>0</v>
+        <v>979078233</v>
       </c>
       <c r="S20">
-        <v>0</v>
+        <v>-3343774083</v>
       </c>
       <c r="T20">
-        <v>0</v>
+        <v>-3525649863</v>
       </c>
       <c r="U20">
-        <v>0</v>
+        <v>-1713494359</v>
       </c>
       <c r="V20">
-        <v>0</v>
+        <v>-4430074915</v>
       </c>
       <c r="W20">
-        <v>0</v>
+        <v>-8304699942</v>
       </c>
       <c r="X20">
-        <v>0</v>
+        <v>-1627684107</v>
       </c>
       <c r="Y20" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
     </row>
     <row r="21" spans="1:25">
@@ -2631,46 +2646,46 @@
         <v>40</v>
       </c>
       <c r="B21" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C21" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D21" t="s">
-        <v>61</v>
+        <v>73</v>
       </c>
       <c r="E21" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="F21">
-        <v>1400000</v>
+        <v>5000000</v>
       </c>
       <c r="G21">
-        <v>1400000</v>
+        <v>5000000</v>
       </c>
       <c r="H21">
         <v>0</v>
       </c>
       <c r="I21">
-        <v>34000</v>
+        <v>2000</v>
       </c>
       <c r="J21">
-        <v>40000</v>
+        <v>2000</v>
       </c>
       <c r="K21">
-        <v>7942750</v>
+        <v>5840000</v>
       </c>
       <c r="L21">
         <v>0</v>
       </c>
       <c r="M21">
-        <v>40000</v>
+        <v>2000</v>
       </c>
       <c r="N21" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="O21" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="P21">
         <v>0</v>
@@ -2700,84 +2715,161 @@
         <v>0</v>
       </c>
       <c r="Y21" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
     </row>
     <row r="22" spans="1:25">
       <c r="A22" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="B22" t="s">
+        <v>50</v>
+      </c>
+      <c r="C22" t="s">
+        <v>61</v>
+      </c>
+      <c r="D22" t="s">
+        <v>64</v>
+      </c>
+      <c r="E22" t="s">
+        <v>95</v>
+      </c>
+      <c r="F22">
+        <v>1400000</v>
+      </c>
+      <c r="G22">
+        <v>1400000</v>
+      </c>
+      <c r="H22">
+        <v>0</v>
+      </c>
+      <c r="I22">
+        <v>34000</v>
+      </c>
+      <c r="J22">
+        <v>40000</v>
+      </c>
+      <c r="K22">
+        <v>7942750</v>
+      </c>
+      <c r="L22">
+        <v>0</v>
+      </c>
+      <c r="M22">
+        <v>40000</v>
+      </c>
+      <c r="N22" t="s">
+        <v>117</v>
+      </c>
+      <c r="O22" t="s">
+        <v>131</v>
+      </c>
+      <c r="P22">
+        <v>0</v>
+      </c>
+      <c r="Q22">
+        <v>0</v>
+      </c>
+      <c r="R22">
+        <v>0</v>
+      </c>
+      <c r="S22">
+        <v>0</v>
+      </c>
+      <c r="T22">
+        <v>0</v>
+      </c>
+      <c r="U22">
+        <v>0</v>
+      </c>
+      <c r="V22">
+        <v>0</v>
+      </c>
+      <c r="W22">
+        <v>0</v>
+      </c>
+      <c r="X22">
+        <v>0</v>
+      </c>
+      <c r="Y22" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="23" spans="1:25">
+      <c r="A23" t="s">
         <v>35</v>
       </c>
-      <c r="C22" t="s">
-        <v>60</v>
-      </c>
-      <c r="D22" t="s">
-        <v>72</v>
-      </c>
-      <c r="E22" t="s">
-        <v>93</v>
-      </c>
-      <c r="F22">
+      <c r="B23" t="s">
+        <v>36</v>
+      </c>
+      <c r="C23" t="s">
+        <v>62</v>
+      </c>
+      <c r="D23" t="s">
+        <v>74</v>
+      </c>
+      <c r="E23" t="s">
+        <v>96</v>
+      </c>
+      <c r="F23">
         <v>23333334</v>
       </c>
-      <c r="G22">
+      <c r="G23">
         <v>23333334</v>
       </c>
-      <c r="H22">
-        <v>0</v>
-      </c>
-      <c r="I22">
+      <c r="H23">
+        <v>0</v>
+      </c>
+      <c r="I23">
         <v>3000</v>
       </c>
-      <c r="J22">
+      <c r="J23">
         <v>3800</v>
       </c>
-      <c r="K22">
+      <c r="K23">
         <v>43477664</v>
       </c>
-      <c r="L22">
-        <v>0</v>
-      </c>
-      <c r="M22">
+      <c r="L23">
+        <v>0</v>
+      </c>
+      <c r="M23">
         <v>3000</v>
       </c>
-      <c r="N22" t="s">
-        <v>114</v>
-      </c>
-      <c r="O22" t="s">
-        <v>117</v>
-      </c>
-      <c r="P22">
-        <v>0</v>
-      </c>
-      <c r="Q22">
-        <v>0</v>
-      </c>
-      <c r="R22">
-        <v>0</v>
-      </c>
-      <c r="S22">
-        <v>0</v>
-      </c>
-      <c r="T22">
-        <v>0</v>
-      </c>
-      <c r="U22">
-        <v>0</v>
-      </c>
-      <c r="V22">
-        <v>0</v>
-      </c>
-      <c r="W22">
-        <v>0</v>
-      </c>
-      <c r="X22">
-        <v>0</v>
-      </c>
-      <c r="Y22" t="s">
-        <v>142</v>
+      <c r="N23" t="s">
+        <v>118</v>
+      </c>
+      <c r="O23" t="s">
+        <v>122</v>
+      </c>
+      <c r="P23">
+        <v>0</v>
+      </c>
+      <c r="Q23">
+        <v>0</v>
+      </c>
+      <c r="R23">
+        <v>0</v>
+      </c>
+      <c r="S23">
+        <v>0</v>
+      </c>
+      <c r="T23">
+        <v>0</v>
+      </c>
+      <c r="U23">
+        <v>0</v>
+      </c>
+      <c r="V23">
+        <v>0</v>
+      </c>
+      <c r="W23">
+        <v>0</v>
+      </c>
+      <c r="X23">
+        <v>0</v>
+      </c>
+      <c r="Y23" t="s">
+        <v>148</v>
       </c>
     </row>
   </sheetData>
@@ -2792,422 +2884,422 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="B2" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="C2" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="D2" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="E2" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="F2" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="B3" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="C3" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="D3" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="E3" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="F3" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="B4" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="C4" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="D4" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="E4" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="F4" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="B5" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="C5" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="D5" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="E5" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="F5" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="B6" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="C6" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="D6" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="E6" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="F6" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="B7" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="C7" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="D7" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
       <c r="E7" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="F7" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="B8" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="C8" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="D8" t="s">
-        <v>199</v>
+        <v>204</v>
       </c>
       <c r="E8" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
       <c r="F8" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="B9" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="C9" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
       <c r="D9" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="E9" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
       <c r="F9" t="s">
-        <v>231</v>
+        <v>236</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="B10" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="C10" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="D10" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="E10" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="F10" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="B11" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="C11" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="D11" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="E11" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="F11" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="B12" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="C12" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
       <c r="D12" t="s">
-        <v>203</v>
+        <v>208</v>
       </c>
       <c r="E12" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
       <c r="F12" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="B13" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="C13" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="D13" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
       <c r="E13" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="F13" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="B14" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="C14" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="D14" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="E14" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="F14" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="B15" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="C15" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="D15" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="E15" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="F15" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" t="s">
-        <v>163</v>
+        <v>75</v>
       </c>
       <c r="B16" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="C16" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="D16" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="E16" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="F16" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B17" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="C17" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="D17" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="E17" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="F17" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B18" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="C18" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
       <c r="D18" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="E18" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="F18" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="B19" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="C19" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="D19" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
       <c r="E19" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
       <c r="F19" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
     </row>
     <row r="20" spans="1:6">
       <c r="A20" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="B20" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="C20" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="D20" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
       <c r="E20" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
       <c r="F20" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="B21" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="C21" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="D21" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="E21" t="s">
-        <v>224</v>
+        <v>229</v>
       </c>
       <c r="F21" t="s">
-        <v>236</v>
+        <v>241</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
RPA datasets push 2024-08-15
</commit_message>
<xml_diff>
--- a/datasets/ib-strategy-data.xlsx
+++ b/datasets/ib-strategy-data.xlsx
@@ -479,15 +479,15 @@
     <t>주간사</t>
   </si>
   <si>
+    <t>아이언디바이스</t>
+  </si>
+  <si>
     <t>에이치이엠파마(구.에이치이엠)</t>
   </si>
   <si>
     <t>미래에셋비전스팩7호</t>
   </si>
   <si>
-    <t>아이언디바이스</t>
-  </si>
-  <si>
     <t>키움스팩9호</t>
   </si>
   <si>
@@ -530,15 +530,15 @@
     <t>산일전기(유가)</t>
   </si>
   <si>
+    <t>2024.08.30~09.05</t>
+  </si>
+  <si>
     <t>2024.08.26~08.30</t>
   </si>
   <si>
     <t>2024.08.26~08.27</t>
   </si>
   <si>
-    <t>2024.08.19~08.23</t>
-  </si>
-  <si>
     <t>2024.08.13~08.14</t>
   </si>
   <si>
@@ -581,15 +581,15 @@
     <t>2024.07.09~07.15</t>
   </si>
   <si>
+    <t>4,900~5,700</t>
+  </si>
+  <si>
     <t>18,000~21,000</t>
   </si>
   <si>
     <t>2,000~2,000</t>
   </si>
   <si>
-    <t>4,900~5,700</t>
-  </si>
-  <si>
     <t>32,000~40,200</t>
   </si>
   <si>
@@ -656,12 +656,12 @@
     <t>35000</t>
   </si>
   <si>
+    <t>14700</t>
+  </si>
+  <si>
     <t>12546</t>
   </si>
   <si>
-    <t>14700</t>
-  </si>
-  <si>
     <t>6000</t>
   </si>
   <si>
@@ -704,13 +704,13 @@
     <t>266000</t>
   </si>
   <si>
+    <t>대신증권</t>
+  </si>
+  <si>
     <t>신한투자증권</t>
   </si>
   <si>
     <t>미래에셋증권</t>
-  </si>
-  <si>
-    <t>대신증권</t>
   </si>
   <si>
     <t>키움증권</t>
@@ -2933,7 +2933,7 @@
         <v>120</v>
       </c>
       <c r="E3" t="s">
-        <v>120</v>
+        <v>214</v>
       </c>
       <c r="F3" t="s">
         <v>230</v>
@@ -2953,7 +2953,7 @@
         <v>120</v>
       </c>
       <c r="E4" t="s">
-        <v>214</v>
+        <v>120</v>
       </c>
       <c r="F4" t="s">
         <v>231</v>
@@ -2967,7 +2967,7 @@
         <v>174</v>
       </c>
       <c r="C5" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D5" t="s">
         <v>120</v>
@@ -3007,7 +3007,7 @@
         <v>176</v>
       </c>
       <c r="C7" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D7" t="s">
         <v>202</v>
@@ -3016,7 +3016,7 @@
         <v>205</v>
       </c>
       <c r="F7" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -3116,7 +3116,7 @@
         <v>220</v>
       </c>
       <c r="F12" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -3127,7 +3127,7 @@
         <v>181</v>
       </c>
       <c r="C13" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D13" t="s">
         <v>202</v>
@@ -3167,7 +3167,7 @@
         <v>182</v>
       </c>
       <c r="C15" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D15" t="s">
         <v>209</v>
@@ -3196,7 +3196,7 @@
         <v>223</v>
       </c>
       <c r="F16" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -3247,7 +3247,7 @@
         <v>186</v>
       </c>
       <c r="C19" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D19" t="s">
         <v>202</v>
@@ -3267,7 +3267,7 @@
         <v>186</v>
       </c>
       <c r="C20" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D20" t="s">
         <v>202</v>

</xml_diff>

<commit_message>
RPA datasets push 2024-08-16
</commit_message>
<xml_diff>
--- a/datasets/ib-strategy-data.xlsx
+++ b/datasets/ib-strategy-data.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="241">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="335" uniqueCount="246">
   <si>
     <t>수요예측(시작일)</t>
   </si>
@@ -143,6 +143,9 @@
     <t>2024-05-28</t>
   </si>
   <si>
+    <t>2024-08-02</t>
+  </si>
+  <si>
     <t>2024-07-30</t>
   </si>
   <si>
@@ -170,6 +173,9 @@
     <t>2024-05-29</t>
   </si>
   <si>
+    <t>2024-08-16</t>
+  </si>
+  <si>
     <t>2024-08-13</t>
   </si>
   <si>
@@ -206,6 +212,9 @@
     <t>2024-07-01</t>
   </si>
   <si>
+    <t>키움</t>
+  </si>
+  <si>
     <t>교보</t>
   </si>
   <si>
@@ -215,9 +224,6 @@
     <t>삼성</t>
   </si>
   <si>
-    <t>키움</t>
-  </si>
-  <si>
     <t>NH</t>
   </si>
   <si>
@@ -245,6 +251,9 @@
     <t>신한, 한국</t>
   </si>
   <si>
+    <t>유라클</t>
+  </si>
+  <si>
     <t>교보16호스팩</t>
   </si>
   <si>
@@ -311,6 +320,9 @@
     <t>신한글로벌액티브리츠</t>
   </si>
   <si>
+    <t>1065.86:1</t>
+  </si>
+  <si>
     <t>1085.71:1</t>
   </si>
   <si>
@@ -377,6 +389,9 @@
     <t>38.7:1</t>
   </si>
   <si>
+    <t>0.55%</t>
+  </si>
+  <si>
     <t>-</t>
   </si>
   <si>
@@ -413,6 +428,9 @@
     <t>9.93%</t>
   </si>
   <si>
+    <t>모바일 앱 개발 플랫폼</t>
+  </si>
+  <si>
     <t>기업인수합병</t>
   </si>
   <si>
@@ -516,9 +534,6 @@
   </si>
   <si>
     <t>넥스트바이오메디컬</t>
-  </si>
-  <si>
-    <t>유라클</t>
   </si>
   <si>
     <t>NH스팩31호</t>
@@ -1095,7 +1110,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Y23"/>
+  <dimension ref="A1:Y24"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:25">
@@ -1183,43 +1198,43 @@
         <v>42</v>
       </c>
       <c r="C2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="E2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="F2">
-        <v>5800000</v>
+        <v>751000</v>
       </c>
       <c r="G2">
-        <v>5800000</v>
+        <v>203700</v>
       </c>
       <c r="H2">
-        <v>0</v>
+        <v>547300</v>
       </c>
       <c r="I2">
-        <v>2000</v>
+        <v>18000</v>
       </c>
       <c r="J2">
-        <v>2000</v>
+        <v>21000</v>
       </c>
       <c r="K2">
-        <v>6100000</v>
+        <v>4330068</v>
       </c>
       <c r="L2">
         <v>0</v>
       </c>
       <c r="M2">
-        <v>2000</v>
+        <v>21000</v>
       </c>
       <c r="N2" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="O2" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="P2">
         <v>0</v>
@@ -1249,315 +1264,315 @@
         <v>0</v>
       </c>
       <c r="Y2" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
     </row>
     <row r="3" spans="1:25">
       <c r="A3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B3" t="s">
-        <v>25</v>
+        <v>43</v>
       </c>
       <c r="C3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D3" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="F3">
-        <v>1400000</v>
+        <v>5800000</v>
       </c>
       <c r="G3">
-        <v>1400000</v>
+        <v>5800000</v>
       </c>
       <c r="H3">
         <v>0</v>
       </c>
       <c r="I3">
-        <v>16000</v>
+        <v>2000</v>
       </c>
       <c r="J3">
-        <v>19000</v>
+        <v>2000</v>
       </c>
       <c r="K3">
-        <v>10000988</v>
+        <v>6100000</v>
       </c>
       <c r="L3">
         <v>0</v>
       </c>
       <c r="M3">
-        <v>16000</v>
+        <v>2000</v>
       </c>
       <c r="N3" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="O3" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="P3">
-        <v>72895458363</v>
+        <v>0</v>
       </c>
       <c r="Q3">
-        <v>72913766913</v>
+        <v>0</v>
       </c>
       <c r="R3">
-        <v>11230711680</v>
+        <v>0</v>
       </c>
       <c r="S3">
-        <v>-6524077412</v>
+        <v>0</v>
       </c>
       <c r="T3">
-        <v>-4556157069</v>
+        <v>0</v>
       </c>
       <c r="U3">
-        <v>-3633759729</v>
+        <v>0</v>
       </c>
       <c r="V3">
-        <v>-11528915410</v>
+        <v>0</v>
       </c>
       <c r="W3">
-        <v>-7978634776</v>
+        <v>0</v>
       </c>
       <c r="X3">
-        <v>-3801868433</v>
+        <v>0</v>
       </c>
       <c r="Y3" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
     </row>
     <row r="4" spans="1:25">
       <c r="A4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B4" t="s">
-        <v>43</v>
+        <v>25</v>
       </c>
       <c r="C4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D4" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E4" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="F4">
-        <v>2234000</v>
+        <v>1400000</v>
       </c>
       <c r="G4">
-        <v>2234000</v>
+        <v>1400000</v>
       </c>
       <c r="H4">
         <v>0</v>
       </c>
       <c r="I4">
-        <v>7300</v>
+        <v>16000</v>
       </c>
       <c r="J4">
-        <v>8500</v>
+        <v>19000</v>
       </c>
       <c r="K4">
-        <v>14965620</v>
+        <v>10000988</v>
       </c>
       <c r="L4">
         <v>0</v>
       </c>
       <c r="M4">
-        <v>10000</v>
+        <v>16000</v>
       </c>
       <c r="N4" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="O4" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="P4">
-        <v>1337894447</v>
+        <v>72895458363</v>
       </c>
       <c r="Q4">
-        <v>4495088983</v>
+        <v>72913766913</v>
       </c>
       <c r="R4">
-        <v>99398351</v>
+        <v>11230711680</v>
       </c>
       <c r="S4">
-        <v>-3330678562</v>
+        <v>-6524077412</v>
       </c>
       <c r="T4">
-        <v>-2905069801</v>
+        <v>-4556157069</v>
       </c>
       <c r="U4">
-        <v>-1314068310</v>
+        <v>-3633759729</v>
       </c>
       <c r="V4">
-        <v>-9735376868</v>
+        <v>-11528915410</v>
       </c>
       <c r="W4">
-        <v>-5043515600</v>
+        <v>-7978634776</v>
       </c>
       <c r="X4">
-        <v>-1257080998</v>
+        <v>-3801868433</v>
       </c>
       <c r="Y4" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
     </row>
     <row r="5" spans="1:25">
       <c r="A5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B5" t="s">
         <v>44</v>
       </c>
       <c r="C5" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="D5" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E5" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="F5">
-        <v>1350000</v>
+        <v>2234000</v>
       </c>
       <c r="G5">
-        <v>1350000</v>
+        <v>2234000</v>
       </c>
       <c r="H5">
         <v>0</v>
       </c>
       <c r="I5">
-        <v>14000</v>
+        <v>7300</v>
       </c>
       <c r="J5">
-        <v>17000</v>
+        <v>8500</v>
       </c>
       <c r="K5">
-        <v>6471740</v>
+        <v>14965620</v>
       </c>
       <c r="L5">
         <v>0</v>
       </c>
       <c r="M5">
-        <v>22000</v>
+        <v>10000</v>
       </c>
       <c r="N5" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="O5" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="P5">
-        <v>5214628820</v>
+        <v>1337894447</v>
       </c>
       <c r="Q5">
-        <v>6009352447</v>
+        <v>4495088983</v>
       </c>
       <c r="R5">
-        <v>965797975</v>
+        <v>99398351</v>
       </c>
       <c r="S5">
-        <v>2015081728</v>
+        <v>-3330678562</v>
       </c>
       <c r="T5">
-        <v>1319755337</v>
+        <v>-2905069801</v>
       </c>
       <c r="U5">
-        <v>-44547594</v>
+        <v>-1314068310</v>
       </c>
       <c r="V5">
-        <v>1503069100</v>
+        <v>-9735376868</v>
       </c>
       <c r="W5">
-        <v>1410469786</v>
+        <v>-5043515600</v>
       </c>
       <c r="X5">
-        <v>24178632</v>
+        <v>-1257080998</v>
       </c>
       <c r="Y5" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
     </row>
     <row r="6" spans="1:25">
       <c r="A6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B6" t="s">
         <v>45</v>
       </c>
       <c r="C6" t="s">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="D6" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E6" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="F6">
-        <v>6000000</v>
+        <v>1350000</v>
       </c>
       <c r="G6">
-        <v>6000000</v>
+        <v>1350000</v>
       </c>
       <c r="H6">
         <v>0</v>
       </c>
       <c r="I6">
-        <v>2000</v>
+        <v>14000</v>
       </c>
       <c r="J6">
-        <v>2000</v>
+        <v>17000</v>
       </c>
       <c r="K6">
-        <v>6345000</v>
+        <v>6471740</v>
       </c>
       <c r="L6">
         <v>0</v>
       </c>
       <c r="M6">
-        <v>2000</v>
+        <v>22000</v>
       </c>
       <c r="N6" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="O6" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="P6">
-        <v>0</v>
+        <v>5214628820</v>
       </c>
       <c r="Q6">
-        <v>0</v>
+        <v>6009352447</v>
       </c>
       <c r="R6">
-        <v>0</v>
+        <v>965797975</v>
       </c>
       <c r="S6">
-        <v>0</v>
+        <v>2015081728</v>
       </c>
       <c r="T6">
-        <v>0</v>
+        <v>1319755337</v>
       </c>
       <c r="U6">
-        <v>0</v>
+        <v>-44547594</v>
       </c>
       <c r="V6">
-        <v>0</v>
+        <v>1503069100</v>
       </c>
       <c r="W6">
-        <v>0</v>
+        <v>1410469786</v>
       </c>
       <c r="X6">
-        <v>0</v>
+        <v>24178632</v>
       </c>
       <c r="Y6" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
     </row>
     <row r="7" spans="1:25">
@@ -1565,22 +1580,22 @@
         <v>29</v>
       </c>
       <c r="B7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C7" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="D7" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E7" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="F7">
-        <v>4000000</v>
+        <v>6000000</v>
       </c>
       <c r="G7">
-        <v>4000000</v>
+        <v>6000000</v>
       </c>
       <c r="H7">
         <v>0</v>
@@ -1592,7 +1607,7 @@
         <v>2000</v>
       </c>
       <c r="K7">
-        <v>4420000</v>
+        <v>6345000</v>
       </c>
       <c r="L7">
         <v>0</v>
@@ -1601,10 +1616,10 @@
         <v>2000</v>
       </c>
       <c r="N7" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="O7" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="P7">
         <v>0</v>
@@ -1634,54 +1649,54 @@
         <v>0</v>
       </c>
       <c r="Y7" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
     </row>
     <row r="8" spans="1:25">
       <c r="A8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B8" t="s">
         <v>46</v>
       </c>
       <c r="C8" t="s">
-        <v>27</v>
+        <v>54</v>
       </c>
       <c r="D8" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F8">
-        <v>1618000</v>
+        <v>4000000</v>
       </c>
       <c r="G8">
-        <v>1618000</v>
+        <v>4000000</v>
       </c>
       <c r="H8">
         <v>0</v>
       </c>
       <c r="I8">
-        <v>6200</v>
+        <v>2000</v>
       </c>
       <c r="J8">
-        <v>7700</v>
+        <v>2000</v>
       </c>
       <c r="K8">
-        <v>10830212</v>
+        <v>4420000</v>
       </c>
       <c r="L8">
         <v>0</v>
       </c>
       <c r="M8">
-        <v>10000</v>
+        <v>2000</v>
       </c>
       <c r="N8" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="O8" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="P8">
         <v>0</v>
@@ -1711,54 +1726,54 @@
         <v>0</v>
       </c>
       <c r="Y8" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
     </row>
     <row r="9" spans="1:25">
       <c r="A9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B9" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C9" t="s">
-        <v>55</v>
+        <v>27</v>
       </c>
       <c r="D9" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E9" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F9">
-        <v>4000000</v>
+        <v>1618000</v>
       </c>
       <c r="G9">
-        <v>4000000</v>
+        <v>1618000</v>
       </c>
       <c r="H9">
         <v>0</v>
       </c>
       <c r="I9">
-        <v>2000</v>
+        <v>6200</v>
       </c>
       <c r="J9">
-        <v>2000</v>
+        <v>7700</v>
       </c>
       <c r="K9">
-        <v>5020000</v>
+        <v>10830212</v>
       </c>
       <c r="L9">
         <v>0</v>
       </c>
       <c r="M9">
-        <v>2000</v>
+        <v>10000</v>
       </c>
       <c r="N9" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="O9" t="s">
-        <v>120</v>
+        <v>129</v>
       </c>
       <c r="P9">
         <v>0</v>
@@ -1788,362 +1803,362 @@
         <v>0</v>
       </c>
       <c r="Y9" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
     </row>
     <row r="10" spans="1:25">
       <c r="A10" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B10" t="s">
         <v>47</v>
       </c>
       <c r="C10" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D10" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="E10" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="F10">
-        <v>1810000</v>
+        <v>4000000</v>
       </c>
       <c r="G10">
-        <v>1810000</v>
+        <v>4000000</v>
       </c>
       <c r="H10">
         <v>0</v>
       </c>
       <c r="I10">
-        <v>9000</v>
+        <v>2000</v>
       </c>
       <c r="J10">
-        <v>12000</v>
+        <v>2000</v>
       </c>
       <c r="K10">
-        <v>7836009</v>
+        <v>5020000</v>
       </c>
       <c r="L10">
         <v>0</v>
       </c>
       <c r="M10">
-        <v>16000</v>
+        <v>2000</v>
       </c>
       <c r="N10" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="O10" t="s">
         <v>125</v>
       </c>
       <c r="P10">
-        <v>12596039842</v>
+        <v>0</v>
       </c>
       <c r="Q10">
-        <v>14910346438</v>
+        <v>0</v>
       </c>
       <c r="R10">
-        <v>16039074617</v>
+        <v>0</v>
       </c>
       <c r="S10">
-        <v>1732604466</v>
+        <v>0</v>
       </c>
       <c r="T10">
-        <v>2893667787</v>
+        <v>0</v>
       </c>
       <c r="U10">
-        <v>1613779678</v>
+        <v>0</v>
       </c>
       <c r="V10">
-        <v>1558081149</v>
+        <v>0</v>
       </c>
       <c r="W10">
-        <v>2643467726</v>
+        <v>0</v>
       </c>
       <c r="X10">
-        <v>1795726428</v>
+        <v>0</v>
       </c>
       <c r="Y10" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
     </row>
     <row r="11" spans="1:25">
       <c r="A11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B11" t="s">
         <v>48</v>
       </c>
       <c r="C11" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D11" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E11" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="F11">
-        <v>1330000</v>
+        <v>1810000</v>
       </c>
       <c r="G11">
-        <v>1330000</v>
+        <v>1810000</v>
       </c>
       <c r="H11">
         <v>0</v>
       </c>
       <c r="I11">
-        <v>36400</v>
+        <v>9000</v>
       </c>
       <c r="J11">
-        <v>43300</v>
+        <v>12000</v>
       </c>
       <c r="K11">
-        <v>9375694</v>
+        <v>7836009</v>
       </c>
       <c r="L11">
         <v>0</v>
       </c>
       <c r="M11">
-        <v>43300</v>
+        <v>16000</v>
       </c>
       <c r="N11" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="O11" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="P11">
-        <v>103267682</v>
+        <v>12596039842</v>
       </c>
       <c r="Q11">
-        <v>342201581</v>
+        <v>14910346438</v>
       </c>
       <c r="R11">
-        <v>231425455</v>
+        <v>16039074617</v>
       </c>
       <c r="S11">
-        <v>-7598692896</v>
+        <v>1732604466</v>
       </c>
       <c r="T11">
-        <v>-25822444575</v>
+        <v>2893667787</v>
       </c>
       <c r="U11">
-        <v>-15929213281</v>
+        <v>1613779678</v>
       </c>
       <c r="V11">
-        <v>-6973258680</v>
+        <v>1558081149</v>
       </c>
       <c r="W11">
-        <v>-48433907514</v>
+        <v>2643467726</v>
       </c>
       <c r="X11">
-        <v>-83246975113</v>
+        <v>1795726428</v>
       </c>
       <c r="Y11" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
     </row>
     <row r="12" spans="1:25">
       <c r="A12" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B12" t="s">
-        <v>32</v>
+        <v>49</v>
       </c>
       <c r="C12" t="s">
-        <v>31</v>
+        <v>59</v>
       </c>
       <c r="D12" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="E12" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="F12">
-        <v>3400000</v>
+        <v>1330000</v>
       </c>
       <c r="G12">
-        <v>3400000</v>
+        <v>1330000</v>
       </c>
       <c r="H12">
         <v>0</v>
       </c>
       <c r="I12">
-        <v>4500</v>
+        <v>36400</v>
       </c>
       <c r="J12">
-        <v>5500</v>
+        <v>43300</v>
       </c>
       <c r="K12">
-        <v>30888000</v>
+        <v>9375694</v>
       </c>
       <c r="L12">
         <v>0</v>
       </c>
       <c r="M12">
-        <v>7000</v>
+        <v>43300</v>
       </c>
       <c r="N12" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="O12" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="P12">
-        <v>85187882584</v>
+        <v>103267682</v>
       </c>
       <c r="Q12">
-        <v>87525689695</v>
+        <v>342201581</v>
       </c>
       <c r="R12">
-        <v>77247394706</v>
+        <v>231425455</v>
       </c>
       <c r="S12">
-        <v>2205797752</v>
+        <v>-7598692896</v>
       </c>
       <c r="T12">
-        <v>4920387020</v>
+        <v>-25822444575</v>
       </c>
       <c r="U12">
-        <v>4336496285</v>
+        <v>-15929213281</v>
       </c>
       <c r="V12">
-        <v>1613954566</v>
+        <v>-6973258680</v>
       </c>
       <c r="W12">
-        <v>3980493669</v>
+        <v>-48433907514</v>
       </c>
       <c r="X12">
-        <v>2646634321</v>
+        <v>-83246975113</v>
       </c>
       <c r="Y12" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
     </row>
     <row r="13" spans="1:25">
       <c r="A13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B13" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C13" t="s">
-        <v>58</v>
+        <v>31</v>
       </c>
       <c r="D13" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="E13" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="F13">
-        <v>6250000</v>
+        <v>3400000</v>
       </c>
       <c r="G13">
-        <v>6250000</v>
+        <v>3400000</v>
       </c>
       <c r="H13">
         <v>0</v>
       </c>
       <c r="I13">
-        <v>2000</v>
+        <v>4500</v>
       </c>
       <c r="J13">
-        <v>2000</v>
+        <v>5500</v>
       </c>
       <c r="K13">
-        <v>6870000</v>
+        <v>30888000</v>
       </c>
       <c r="L13">
         <v>0</v>
       </c>
       <c r="M13">
-        <v>2000</v>
+        <v>7000</v>
       </c>
       <c r="N13" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="O13" t="s">
-        <v>120</v>
+        <v>132</v>
       </c>
       <c r="P13">
-        <v>0</v>
+        <v>85187882584</v>
       </c>
       <c r="Q13">
-        <v>0</v>
+        <v>87525689695</v>
       </c>
       <c r="R13">
-        <v>0</v>
+        <v>77247394706</v>
       </c>
       <c r="S13">
-        <v>0</v>
+        <v>2205797752</v>
       </c>
       <c r="T13">
-        <v>0</v>
+        <v>4920387020</v>
       </c>
       <c r="U13">
-        <v>0</v>
+        <v>4336496285</v>
       </c>
       <c r="V13">
-        <v>0</v>
+        <v>1613954566</v>
       </c>
       <c r="W13">
-        <v>0</v>
+        <v>3980493669</v>
       </c>
       <c r="X13">
-        <v>0</v>
+        <v>2646634321</v>
       </c>
       <c r="Y13" t="s">
-        <v>132</v>
+        <v>147</v>
       </c>
     </row>
     <row r="14" spans="1:25">
       <c r="A14" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B14" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C14" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D14" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="E14" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F14">
-        <v>2000000</v>
+        <v>6250000</v>
       </c>
       <c r="G14">
-        <v>2000000</v>
+        <v>6250000</v>
       </c>
       <c r="H14">
         <v>0</v>
       </c>
       <c r="I14">
-        <v>7500</v>
+        <v>2000</v>
       </c>
       <c r="J14">
-        <v>9000</v>
+        <v>2000</v>
       </c>
       <c r="K14">
-        <v>17529140</v>
+        <v>6870000</v>
       </c>
       <c r="L14">
         <v>0</v>
       </c>
       <c r="M14">
-        <v>11500</v>
+        <v>2000</v>
       </c>
       <c r="N14" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="O14" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="P14">
         <v>0</v>
@@ -2173,54 +2188,54 @@
         <v>0</v>
       </c>
       <c r="Y14" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
     </row>
     <row r="15" spans="1:25">
       <c r="A15" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B15" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C15" t="s">
-        <v>30</v>
+        <v>61</v>
       </c>
       <c r="D15" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="E15" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="F15">
-        <v>6450000</v>
+        <v>2000000</v>
       </c>
       <c r="G15">
-        <v>6450000</v>
+        <v>2000000</v>
       </c>
       <c r="H15">
         <v>0</v>
       </c>
       <c r="I15">
-        <v>2000</v>
+        <v>7500</v>
       </c>
       <c r="J15">
-        <v>2000</v>
+        <v>9000</v>
       </c>
       <c r="K15">
-        <v>6930000</v>
+        <v>17529140</v>
       </c>
       <c r="L15">
         <v>0</v>
       </c>
       <c r="M15">
-        <v>2000</v>
+        <v>11500</v>
       </c>
       <c r="N15" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="O15" t="s">
-        <v>120</v>
+        <v>133</v>
       </c>
       <c r="P15">
         <v>0</v>
@@ -2250,30 +2265,30 @@
         <v>0</v>
       </c>
       <c r="Y15" t="s">
-        <v>132</v>
+        <v>148</v>
       </c>
     </row>
     <row r="16" spans="1:25">
       <c r="A16" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B16" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C16" t="s">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="D16" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="E16" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F16">
-        <v>6000000</v>
+        <v>6450000</v>
       </c>
       <c r="G16">
-        <v>6000000</v>
+        <v>6450000</v>
       </c>
       <c r="H16">
         <v>0</v>
@@ -2285,7 +2300,7 @@
         <v>2000</v>
       </c>
       <c r="K16">
-        <v>6220000</v>
+        <v>6930000</v>
       </c>
       <c r="L16">
         <v>0</v>
@@ -2294,10 +2309,10 @@
         <v>2000</v>
       </c>
       <c r="N16" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="O16" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="P16">
         <v>0</v>
@@ -2327,30 +2342,30 @@
         <v>0</v>
       </c>
       <c r="Y16" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
     </row>
     <row r="17" spans="1:25">
       <c r="A17" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B17" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C17" t="s">
-        <v>47</v>
+        <v>62</v>
       </c>
       <c r="D17" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="E17" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="F17">
-        <v>4000000</v>
+        <v>6000000</v>
       </c>
       <c r="G17">
-        <v>4000000</v>
+        <v>6000000</v>
       </c>
       <c r="H17">
         <v>0</v>
@@ -2362,7 +2377,7 @@
         <v>2000</v>
       </c>
       <c r="K17">
-        <v>4810000</v>
+        <v>6220000</v>
       </c>
       <c r="L17">
         <v>0</v>
@@ -2371,10 +2386,10 @@
         <v>2000</v>
       </c>
       <c r="N17" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="O17" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="P17">
         <v>0</v>
@@ -2404,7 +2419,7 @@
         <v>0</v>
       </c>
       <c r="Y17" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
     </row>
     <row r="18" spans="1:25">
@@ -2415,19 +2430,19 @@
         <v>38</v>
       </c>
       <c r="C18" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D18" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="E18" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="F18">
-        <v>4750000</v>
+        <v>4000000</v>
       </c>
       <c r="G18">
-        <v>4750000</v>
+        <v>4000000</v>
       </c>
       <c r="H18">
         <v>0</v>
@@ -2439,7 +2454,7 @@
         <v>2000</v>
       </c>
       <c r="K18">
-        <v>5480000</v>
+        <v>4810000</v>
       </c>
       <c r="L18">
         <v>0</v>
@@ -2448,10 +2463,10 @@
         <v>2000</v>
       </c>
       <c r="N18" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="O18" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="P18">
         <v>0</v>
@@ -2481,392 +2496,469 @@
         <v>0</v>
       </c>
       <c r="Y18" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
     </row>
     <row r="19" spans="1:25">
       <c r="A19" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B19" t="s">
-        <v>49</v>
+        <v>38</v>
       </c>
       <c r="C19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D19" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="E19" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="F19">
-        <v>1300000</v>
+        <v>4750000</v>
       </c>
       <c r="G19">
-        <v>1300000</v>
+        <v>4750000</v>
       </c>
       <c r="H19">
         <v>0</v>
       </c>
       <c r="I19">
-        <v>10500</v>
+        <v>2000</v>
       </c>
       <c r="J19">
-        <v>14000</v>
+        <v>2000</v>
       </c>
       <c r="K19">
-        <v>12293880</v>
+        <v>5480000</v>
       </c>
       <c r="L19">
         <v>0</v>
       </c>
       <c r="M19">
-        <v>17000</v>
+        <v>2000</v>
       </c>
       <c r="N19" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="O19" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="P19">
-        <v>1386123525</v>
+        <v>0</v>
       </c>
       <c r="Q19">
-        <v>1152944128</v>
+        <v>0</v>
       </c>
       <c r="R19">
-        <v>1885010467</v>
+        <v>0</v>
       </c>
       <c r="S19">
-        <v>-4388824706</v>
+        <v>0</v>
       </c>
       <c r="T19">
-        <v>-7990287699</v>
+        <v>0</v>
       </c>
       <c r="U19">
-        <v>-9803411085</v>
+        <v>0</v>
       </c>
       <c r="V19">
-        <v>-4430563401</v>
+        <v>0</v>
       </c>
       <c r="W19">
-        <v>-7988275689</v>
+        <v>0</v>
       </c>
       <c r="X19">
-        <v>-9916946238</v>
+        <v>0</v>
       </c>
       <c r="Y19" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
     </row>
     <row r="20" spans="1:25">
       <c r="A20" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B20" t="s">
-        <v>37</v>
+        <v>50</v>
       </c>
       <c r="C20" t="s">
-        <v>30</v>
+        <v>48</v>
       </c>
       <c r="D20" t="s">
         <v>73</v>
       </c>
       <c r="E20" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="F20">
-        <v>1600000</v>
+        <v>1300000</v>
       </c>
       <c r="G20">
-        <v>1600000</v>
+        <v>1300000</v>
       </c>
       <c r="H20">
         <v>0</v>
       </c>
       <c r="I20">
-        <v>20000</v>
+        <v>10500</v>
       </c>
       <c r="J20">
-        <v>23500</v>
+        <v>14000</v>
       </c>
       <c r="K20">
-        <v>8751446</v>
+        <v>12293880</v>
       </c>
       <c r="L20">
         <v>0</v>
       </c>
       <c r="M20">
-        <v>30000</v>
+        <v>17000</v>
       </c>
       <c r="N20" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="O20" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="P20">
-        <v>0</v>
+        <v>1386123525</v>
       </c>
       <c r="Q20">
-        <v>0</v>
+        <v>1152944128</v>
       </c>
       <c r="R20">
-        <v>0</v>
+        <v>1885010467</v>
       </c>
       <c r="S20">
-        <v>0</v>
+        <v>-4388824706</v>
       </c>
       <c r="T20">
-        <v>0</v>
+        <v>-7990287699</v>
       </c>
       <c r="U20">
-        <v>0</v>
+        <v>-9803411085</v>
       </c>
       <c r="V20">
-        <v>0</v>
+        <v>-4430563401</v>
       </c>
       <c r="W20">
-        <v>0</v>
+        <v>-7988275689</v>
       </c>
       <c r="X20">
-        <v>0</v>
+        <v>-9916946238</v>
       </c>
       <c r="Y20" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
     </row>
     <row r="21" spans="1:25">
       <c r="A21" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B21" t="s">
-        <v>49</v>
+        <v>37</v>
       </c>
       <c r="C21" t="s">
-        <v>48</v>
+        <v>30</v>
       </c>
       <c r="D21" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="E21" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="F21">
-        <v>1298000</v>
+        <v>1600000</v>
       </c>
       <c r="G21">
-        <v>1298000</v>
+        <v>1600000</v>
       </c>
       <c r="H21">
         <v>0</v>
       </c>
       <c r="I21">
-        <v>10400</v>
+        <v>20000</v>
       </c>
       <c r="J21">
-        <v>12700</v>
+        <v>23500</v>
       </c>
       <c r="K21">
-        <v>8650735</v>
+        <v>8751446</v>
       </c>
       <c r="L21">
         <v>0</v>
       </c>
       <c r="M21">
-        <v>16000</v>
+        <v>30000</v>
       </c>
       <c r="N21" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="O21" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="P21">
-        <v>2055746777</v>
+        <v>0</v>
       </c>
       <c r="Q21">
-        <v>2918221978</v>
+        <v>0</v>
       </c>
       <c r="R21">
-        <v>979078233</v>
+        <v>0</v>
       </c>
       <c r="S21">
-        <v>-3343774083</v>
+        <v>0</v>
       </c>
       <c r="T21">
-        <v>-3525649863</v>
+        <v>0</v>
       </c>
       <c r="U21">
-        <v>-1713494359</v>
+        <v>0</v>
       </c>
       <c r="V21">
-        <v>-4430074915</v>
+        <v>0</v>
       </c>
       <c r="W21">
-        <v>-8304699942</v>
+        <v>0</v>
       </c>
       <c r="X21">
-        <v>-1627684107</v>
+        <v>0</v>
       </c>
       <c r="Y21" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
     </row>
     <row r="22" spans="1:25">
       <c r="A22" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B22" t="s">
         <v>50</v>
       </c>
       <c r="C22" t="s">
-        <v>61</v>
+        <v>49</v>
       </c>
       <c r="D22" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="E22" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="F22">
-        <v>5000000</v>
+        <v>1298000</v>
       </c>
       <c r="G22">
-        <v>5000000</v>
+        <v>1298000</v>
       </c>
       <c r="H22">
         <v>0</v>
       </c>
       <c r="I22">
-        <v>2000</v>
+        <v>10400</v>
       </c>
       <c r="J22">
-        <v>2000</v>
+        <v>12700</v>
       </c>
       <c r="K22">
-        <v>5840000</v>
+        <v>8650735</v>
       </c>
       <c r="L22">
         <v>0</v>
       </c>
       <c r="M22">
-        <v>2000</v>
+        <v>16000</v>
       </c>
       <c r="N22" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="O22" t="s">
-        <v>120</v>
+        <v>136</v>
       </c>
       <c r="P22">
-        <v>0</v>
+        <v>2055746777</v>
       </c>
       <c r="Q22">
-        <v>0</v>
+        <v>2918221978</v>
       </c>
       <c r="R22">
-        <v>0</v>
+        <v>979078233</v>
       </c>
       <c r="S22">
-        <v>0</v>
+        <v>-3343774083</v>
       </c>
       <c r="T22">
-        <v>0</v>
+        <v>-3525649863</v>
       </c>
       <c r="U22">
-        <v>0</v>
+        <v>-1713494359</v>
       </c>
       <c r="V22">
-        <v>0</v>
+        <v>-4430074915</v>
       </c>
       <c r="W22">
-        <v>0</v>
+        <v>-8304699942</v>
       </c>
       <c r="X22">
-        <v>0</v>
+        <v>-1627684107</v>
       </c>
       <c r="Y22" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
     </row>
     <row r="23" spans="1:25">
       <c r="A23" t="s">
+        <v>41</v>
+      </c>
+      <c r="B23" t="s">
+        <v>51</v>
+      </c>
+      <c r="C23" t="s">
+        <v>63</v>
+      </c>
+      <c r="D23" t="s">
+        <v>76</v>
+      </c>
+      <c r="E23" t="s">
+        <v>99</v>
+      </c>
+      <c r="F23">
+        <v>5000000</v>
+      </c>
+      <c r="G23">
+        <v>5000000</v>
+      </c>
+      <c r="H23">
+        <v>0</v>
+      </c>
+      <c r="I23">
+        <v>2000</v>
+      </c>
+      <c r="J23">
+        <v>2000</v>
+      </c>
+      <c r="K23">
+        <v>5840000</v>
+      </c>
+      <c r="L23">
+        <v>0</v>
+      </c>
+      <c r="M23">
+        <v>2000</v>
+      </c>
+      <c r="N23" t="s">
+        <v>122</v>
+      </c>
+      <c r="O23" t="s">
+        <v>125</v>
+      </c>
+      <c r="P23">
+        <v>0</v>
+      </c>
+      <c r="Q23">
+        <v>0</v>
+      </c>
+      <c r="R23">
+        <v>0</v>
+      </c>
+      <c r="S23">
+        <v>0</v>
+      </c>
+      <c r="T23">
+        <v>0</v>
+      </c>
+      <c r="U23">
+        <v>0</v>
+      </c>
+      <c r="V23">
+        <v>0</v>
+      </c>
+      <c r="W23">
+        <v>0</v>
+      </c>
+      <c r="X23">
+        <v>0</v>
+      </c>
+      <c r="Y23" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="24" spans="1:25">
+      <c r="A24" t="s">
         <v>36</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B24" t="s">
         <v>37</v>
       </c>
-      <c r="C23" t="s">
-        <v>62</v>
-      </c>
-      <c r="D23" t="s">
-        <v>75</v>
-      </c>
-      <c r="E23" t="s">
-        <v>97</v>
-      </c>
-      <c r="F23">
+      <c r="C24" t="s">
+        <v>64</v>
+      </c>
+      <c r="D24" t="s">
+        <v>77</v>
+      </c>
+      <c r="E24" t="s">
+        <v>100</v>
+      </c>
+      <c r="F24">
         <v>23333334</v>
       </c>
-      <c r="G23">
+      <c r="G24">
         <v>23333334</v>
       </c>
-      <c r="H23">
-        <v>0</v>
-      </c>
-      <c r="I23">
+      <c r="H24">
+        <v>0</v>
+      </c>
+      <c r="I24">
         <v>3000</v>
       </c>
-      <c r="J23">
+      <c r="J24">
         <v>3800</v>
       </c>
-      <c r="K23">
+      <c r="K24">
         <v>43477664</v>
       </c>
-      <c r="L23">
-        <v>0</v>
-      </c>
-      <c r="M23">
+      <c r="L24">
+        <v>0</v>
+      </c>
+      <c r="M24">
         <v>3000</v>
       </c>
-      <c r="N23" t="s">
-        <v>119</v>
-      </c>
-      <c r="O23" t="s">
-        <v>120</v>
-      </c>
-      <c r="P23">
-        <v>0</v>
-      </c>
-      <c r="Q23">
-        <v>0</v>
-      </c>
-      <c r="R23">
-        <v>0</v>
-      </c>
-      <c r="S23">
-        <v>0</v>
-      </c>
-      <c r="T23">
-        <v>0</v>
-      </c>
-      <c r="U23">
-        <v>0</v>
-      </c>
-      <c r="V23">
-        <v>0</v>
-      </c>
-      <c r="W23">
-        <v>0</v>
-      </c>
-      <c r="X23">
-        <v>0</v>
-      </c>
-      <c r="Y23" t="s">
-        <v>147</v>
+      <c r="N24" t="s">
+        <v>123</v>
+      </c>
+      <c r="O24" t="s">
+        <v>125</v>
+      </c>
+      <c r="P24">
+        <v>0</v>
+      </c>
+      <c r="Q24">
+        <v>0</v>
+      </c>
+      <c r="R24">
+        <v>0</v>
+      </c>
+      <c r="S24">
+        <v>0</v>
+      </c>
+      <c r="T24">
+        <v>0</v>
+      </c>
+      <c r="U24">
+        <v>0</v>
+      </c>
+      <c r="V24">
+        <v>0</v>
+      </c>
+      <c r="W24">
+        <v>0</v>
+      </c>
+      <c r="X24">
+        <v>0</v>
+      </c>
+      <c r="Y24" t="s">
+        <v>153</v>
       </c>
     </row>
   </sheetData>
@@ -2881,422 +2973,422 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="B2" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="C2" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="D2" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="E2" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
       <c r="F2" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="B3" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="C3" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
       <c r="D3" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="E3" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
       <c r="F3" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="B4" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="C4" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="D4" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="E4" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="F4" t="s">
-        <v>231</v>
+        <v>236</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="B5" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="C5" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="D5" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="E5" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="F5" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="B6" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="C6" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="D6" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="E6" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
       <c r="F6" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="B7" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="C7" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="D7" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="E7" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="F7" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="B8" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="C8" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
       <c r="D8" t="s">
-        <v>203</v>
+        <v>208</v>
       </c>
       <c r="E8" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="F8" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="B9" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="C9" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="D9" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="E9" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="F9" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="B10" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="C10" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="D10" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="E10" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="F10" t="s">
-        <v>236</v>
+        <v>241</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="B11" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="C11" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="D11" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="E11" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="F11" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="B12" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="C12" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
       <c r="D12" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="E12" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="F12" t="s">
-        <v>231</v>
+        <v>236</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="B13" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="C13" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="D13" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="E13" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="F13" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="B14" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="C14" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="D14" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="E14" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="F14" t="s">
-        <v>236</v>
+        <v>241</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" t="s">
-        <v>167</v>
+        <v>78</v>
       </c>
       <c r="B15" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="C15" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
       <c r="D15" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="E15" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
       <c r="F15" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="B16" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="C16" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
       <c r="D16" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="E16" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
       <c r="F16" t="s">
-        <v>231</v>
+        <v>236</v>
       </c>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="B17" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="C17" t="s">
-        <v>199</v>
+        <v>204</v>
       </c>
       <c r="D17" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="E17" t="s">
-        <v>224</v>
+        <v>229</v>
       </c>
       <c r="F17" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="B18" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="C18" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="D18" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="E18" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="F18" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="B19" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="C19" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="D19" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="E19" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="F19" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
     </row>
     <row r="20" spans="1:6">
       <c r="A20" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="B20" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="C20" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="D20" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="E20" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="F20" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="B21" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="C21" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="D21" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="E21" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="F21" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
RPA datasets push 2024-08-26
</commit_message>
<xml_diff>
--- a/datasets/ib-strategy-data.xlsx
+++ b/datasets/ib-strategy-data.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="229">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="225">
   <si>
     <t>수요예측(시작일)</t>
   </si>
@@ -134,9 +134,6 @@
     <t>2024-06-07</t>
   </si>
   <si>
-    <t>2024-06-10</t>
-  </si>
-  <si>
     <t>2024-06-03</t>
   </si>
   <si>
@@ -200,9 +197,6 @@
     <t>2024-07-02</t>
   </si>
   <si>
-    <t>2024-06-26</t>
-  </si>
-  <si>
     <t>2024-07-01</t>
   </si>
   <si>
@@ -290,9 +284,6 @@
     <t>하이젠알앤엠</t>
   </si>
   <si>
-    <t>한국제15호스팩</t>
-  </si>
-  <si>
     <t>신한글로벌액티브리츠</t>
   </si>
   <si>
@@ -345,9 +336,6 @@
   </si>
   <si>
     <t>1099.21:1</t>
-  </si>
-  <si>
-    <t>1,073.31:1</t>
   </si>
   <si>
     <t>38.7:1</t>
@@ -1059,7 +1047,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Y20"/>
+  <dimension ref="A1:Y19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:25">
@@ -1144,16 +1132,16 @@
         <v>25</v>
       </c>
       <c r="B2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E2" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="F2">
         <v>1566800</v>
@@ -1180,10 +1168,10 @@
         <v>15300</v>
       </c>
       <c r="N2" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="O2" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="P2">
         <v>7367362</v>
@@ -1213,7 +1201,7 @@
         <v>-2903334</v>
       </c>
       <c r="Y2" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
     </row>
     <row r="3" spans="1:25">
@@ -1221,16 +1209,16 @@
         <v>26</v>
       </c>
       <c r="B3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D3" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E3" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="F3">
         <v>1000000</v>
@@ -1257,10 +1245,10 @@
         <v>13000</v>
       </c>
       <c r="N3" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="O3" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="P3">
         <v>25588</v>
@@ -1290,7 +1278,7 @@
         <v>809</v>
       </c>
       <c r="Y3" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
     </row>
     <row r="4" spans="1:25">
@@ -1298,16 +1286,16 @@
         <v>27</v>
       </c>
       <c r="B4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D4" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="E4" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="F4">
         <v>6500000</v>
@@ -1334,10 +1322,10 @@
         <v>2000</v>
       </c>
       <c r="N4" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="O4" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="P4">
         <v>0</v>
@@ -1367,7 +1355,7 @@
         <v>0</v>
       </c>
       <c r="Y4" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
     </row>
     <row r="5" spans="1:25">
@@ -1378,13 +1366,13 @@
         <v>27</v>
       </c>
       <c r="C5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D5" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="E5" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="F5">
         <v>1400000</v>
@@ -1411,10 +1399,10 @@
         <v>15500</v>
       </c>
       <c r="N5" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="O5" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="P5">
         <v>10740898602</v>
@@ -1444,7 +1432,7 @@
         <v>219774608</v>
       </c>
       <c r="Y5" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
     </row>
     <row r="6" spans="1:25">
@@ -1455,13 +1443,13 @@
         <v>25</v>
       </c>
       <c r="C6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D6" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E6" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="F6">
         <v>1000000</v>
@@ -1488,10 +1476,10 @@
         <v>29000</v>
       </c>
       <c r="N6" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="O6" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="P6">
         <v>0</v>
@@ -1521,7 +1509,7 @@
         <v>0</v>
       </c>
       <c r="Y6" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
     </row>
     <row r="7" spans="1:25">
@@ -1532,13 +1520,13 @@
         <v>25</v>
       </c>
       <c r="C7" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D7" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E7" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="F7">
         <v>751000</v>
@@ -1565,10 +1553,10 @@
         <v>21000</v>
       </c>
       <c r="N7" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="O7" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="P7">
         <v>0</v>
@@ -1598,7 +1586,7 @@
         <v>0</v>
       </c>
       <c r="Y7" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
     </row>
     <row r="8" spans="1:25">
@@ -1609,13 +1597,13 @@
         <v>28</v>
       </c>
       <c r="C8" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D8" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E8" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F8">
         <v>5800000</v>
@@ -1642,10 +1630,10 @@
         <v>2000</v>
       </c>
       <c r="N8" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="O8" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="P8">
         <v>0</v>
@@ -1675,7 +1663,7 @@
         <v>0</v>
       </c>
       <c r="Y8" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
     </row>
     <row r="9" spans="1:25">
@@ -1686,13 +1674,13 @@
         <v>29</v>
       </c>
       <c r="C9" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D9" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="E9" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="F9">
         <v>1400000</v>
@@ -1719,10 +1707,10 @@
         <v>16000</v>
       </c>
       <c r="N9" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="O9" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="P9">
         <v>72895458363</v>
@@ -1752,7 +1740,7 @@
         <v>-3801868433</v>
       </c>
       <c r="Y9" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
     </row>
     <row r="10" spans="1:25">
@@ -1760,16 +1748,16 @@
         <v>31</v>
       </c>
       <c r="B10" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C10" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D10" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="E10" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="F10">
         <v>2234000</v>
@@ -1796,10 +1784,10 @@
         <v>10000</v>
       </c>
       <c r="N10" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="O10" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="P10">
         <v>1337894447</v>
@@ -1829,7 +1817,7 @@
         <v>-1257080998</v>
       </c>
       <c r="Y10" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
     </row>
     <row r="11" spans="1:25">
@@ -1837,16 +1825,16 @@
         <v>32</v>
       </c>
       <c r="B11" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C11" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D11" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E11" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="F11">
         <v>1350000</v>
@@ -1873,10 +1861,10 @@
         <v>22000</v>
       </c>
       <c r="N11" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="O11" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="P11">
         <v>5214628820</v>
@@ -1906,7 +1894,7 @@
         <v>24178632</v>
       </c>
       <c r="Y11" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
     </row>
     <row r="12" spans="1:25">
@@ -1914,16 +1902,16 @@
         <v>33</v>
       </c>
       <c r="B12" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C12" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D12" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E12" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="F12">
         <v>6000000</v>
@@ -1950,10 +1938,10 @@
         <v>2000</v>
       </c>
       <c r="N12" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="O12" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="P12">
         <v>0</v>
@@ -1983,7 +1971,7 @@
         <v>0</v>
       </c>
       <c r="Y12" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
     </row>
     <row r="13" spans="1:25">
@@ -1991,16 +1979,16 @@
         <v>33</v>
       </c>
       <c r="B13" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C13" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D13" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E13" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="F13">
         <v>4000000</v>
@@ -2027,10 +2015,10 @@
         <v>2000</v>
       </c>
       <c r="N13" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="O13" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="P13">
         <v>0</v>
@@ -2060,7 +2048,7 @@
         <v>0</v>
       </c>
       <c r="Y13" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
     </row>
     <row r="14" spans="1:25">
@@ -2068,16 +2056,16 @@
         <v>34</v>
       </c>
       <c r="B14" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C14" t="s">
         <v>31</v>
       </c>
       <c r="D14" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="E14" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F14">
         <v>1618000</v>
@@ -2104,10 +2092,10 @@
         <v>10000</v>
       </c>
       <c r="N14" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="O14" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="P14">
         <v>0</v>
@@ -2137,7 +2125,7 @@
         <v>0</v>
       </c>
       <c r="Y14" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
     </row>
     <row r="15" spans="1:25">
@@ -2145,16 +2133,16 @@
         <v>35</v>
       </c>
       <c r="B15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C15" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D15" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="E15" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="F15">
         <v>4000000</v>
@@ -2181,10 +2169,10 @@
         <v>2000</v>
       </c>
       <c r="N15" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="O15" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="P15">
         <v>0</v>
@@ -2214,7 +2202,7 @@
         <v>0</v>
       </c>
       <c r="Y15" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
     </row>
     <row r="16" spans="1:25">
@@ -2222,16 +2210,16 @@
         <v>36</v>
       </c>
       <c r="B16" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C16" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D16" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="E16" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="F16">
         <v>1810000</v>
@@ -2258,10 +2246,10 @@
         <v>16000</v>
       </c>
       <c r="N16" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="O16" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="P16">
         <v>12596039842</v>
@@ -2291,7 +2279,7 @@
         <v>1795726428</v>
       </c>
       <c r="Y16" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
     </row>
     <row r="17" spans="1:25">
@@ -2299,16 +2287,16 @@
         <v>37</v>
       </c>
       <c r="B17" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C17" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D17" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="E17" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="F17">
         <v>1330000</v>
@@ -2335,10 +2323,10 @@
         <v>43300</v>
       </c>
       <c r="N17" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="O17" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="P17">
         <v>103267682</v>
@@ -2368,7 +2356,7 @@
         <v>-83246975113</v>
       </c>
       <c r="Y17" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
     </row>
     <row r="18" spans="1:25">
@@ -2382,10 +2370,10 @@
         <v>35</v>
       </c>
       <c r="D18" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E18" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="F18">
         <v>3400000</v>
@@ -2412,10 +2400,10 @@
         <v>7000</v>
       </c>
       <c r="N18" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="O18" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="P18">
         <v>85187882584</v>
@@ -2445,7 +2433,7 @@
         <v>2646634321</v>
       </c>
       <c r="Y18" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
     </row>
     <row r="19" spans="1:25">
@@ -2453,47 +2441,47 @@
         <v>39</v>
       </c>
       <c r="B19" t="s">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="C19" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D19" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="E19" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="F19">
-        <v>6250000</v>
+        <v>23333334</v>
       </c>
       <c r="G19">
-        <v>6250000</v>
+        <v>23333334</v>
       </c>
       <c r="H19">
         <v>0</v>
       </c>
       <c r="I19">
-        <v>2000</v>
+        <v>3000</v>
       </c>
       <c r="J19">
-        <v>2000</v>
+        <v>3800</v>
       </c>
       <c r="K19">
-        <v>6870000</v>
+        <v>43477664</v>
       </c>
       <c r="L19">
         <v>0</v>
       </c>
       <c r="M19">
-        <v>2000</v>
+        <v>3000</v>
       </c>
       <c r="N19" t="s">
+        <v>107</v>
+      </c>
+      <c r="O19" t="s">
         <v>110</v>
       </c>
-      <c r="O19" t="s">
-        <v>114</v>
-      </c>
       <c r="P19">
         <v>0</v>
       </c>
@@ -2522,84 +2510,7 @@
         <v>0</v>
       </c>
       <c r="Y19" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="20" spans="1:25">
-      <c r="A20" t="s">
-        <v>40</v>
-      </c>
-      <c r="B20" t="s">
-        <v>49</v>
-      </c>
-      <c r="C20" t="s">
-        <v>62</v>
-      </c>
-      <c r="D20" t="s">
-        <v>73</v>
-      </c>
-      <c r="E20" t="s">
-        <v>92</v>
-      </c>
-      <c r="F20">
-        <v>23333334</v>
-      </c>
-      <c r="G20">
-        <v>23333334</v>
-      </c>
-      <c r="H20">
-        <v>0</v>
-      </c>
-      <c r="I20">
-        <v>3000</v>
-      </c>
-      <c r="J20">
-        <v>3800</v>
-      </c>
-      <c r="K20">
-        <v>43477664</v>
-      </c>
-      <c r="L20">
-        <v>0</v>
-      </c>
-      <c r="M20">
-        <v>3000</v>
-      </c>
-      <c r="N20" t="s">
-        <v>111</v>
-      </c>
-      <c r="O20" t="s">
-        <v>114</v>
-      </c>
-      <c r="P20">
-        <v>0</v>
-      </c>
-      <c r="Q20">
-        <v>0</v>
-      </c>
-      <c r="R20">
-        <v>0</v>
-      </c>
-      <c r="S20">
-        <v>0</v>
-      </c>
-      <c r="T20">
-        <v>0</v>
-      </c>
-      <c r="U20">
-        <v>0</v>
-      </c>
-      <c r="V20">
-        <v>0</v>
-      </c>
-      <c r="W20">
-        <v>0</v>
-      </c>
-      <c r="X20">
-        <v>0</v>
-      </c>
-      <c r="Y20" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
     </row>
   </sheetData>
@@ -2614,422 +2525,422 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>143</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>146</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>147</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="B2" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="C2" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="D2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="E2" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="F2" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="B3" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="C3" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="D3" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="E3" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="F3" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="B4" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="C4" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="D4" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="E4" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="F4" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="B5" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="C5" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="D5" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="E5" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="F5" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="B6" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="C6" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="D6" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="E6" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="F6" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="B7" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="C7" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="D7" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="E7" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="F7" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="B8" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="C8" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="D8" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="E8" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="F8" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="B9" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="C9" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="D9" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="E9" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="F9" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="B10" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="C10" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="D10" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="E10" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="F10" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="B11" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="C11" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="D11" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="E11" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="F11" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="B12" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="C12" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="D12" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="E12" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="F12" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="B13" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="C13" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="D13" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="E13" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="F13" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="B14" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C14" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="D14" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="E14" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="F14" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="B15" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="C15" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="D15" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="E15" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="F15" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="B16" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="C16" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="D16" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="E16" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="F16" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="B17" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="C17" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="D17" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="E17" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="F17" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B18" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="C18" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="D18" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="E18" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="F18" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="B19" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="C19" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="D19" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="E19" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="F19" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
     </row>
     <row r="20" spans="1:6">
       <c r="A20" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B20" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="C20" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="D20" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="E20" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="F20" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B21" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="C21" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="D21" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="E21" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="F21" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
RPA datasets push 2024-08-28
</commit_message>
<xml_diff>
--- a/datasets/ib-strategy-data.xlsx
+++ b/datasets/ib-strategy-data.xlsx
@@ -437,6 +437,9 @@
     <t>신한스팩14호</t>
   </si>
   <si>
+    <t>클로봇</t>
+  </si>
+  <si>
     <t>씨메스</t>
   </si>
   <si>
@@ -488,6 +491,9 @@
     <t>2024.10.01~10.02</t>
   </si>
   <si>
+    <t>2024.09.23~09.27</t>
+  </si>
+  <si>
     <t>2024.09.19~09.25</t>
   </si>
   <si>
@@ -530,12 +536,12 @@
     <t>2024.07.31~08.06</t>
   </si>
   <si>
-    <t>2024.07.30~08.05</t>
-  </si>
-  <si>
     <t>2,000~2,000</t>
   </si>
   <si>
+    <t>9,400~10,900</t>
+  </si>
+  <si>
     <t>20,000~24,000</t>
   </si>
   <si>
@@ -578,9 +584,6 @@
     <t>9,500~10,700</t>
   </si>
   <si>
-    <t>12,500~15,500</t>
-  </si>
-  <si>
     <t>32000</t>
   </si>
   <si>
@@ -596,12 +599,12 @@
     <t>13000</t>
   </si>
   <si>
-    <t>15500</t>
-  </si>
-  <si>
     <t>10000</t>
   </si>
   <si>
+    <t>28200</t>
+  </si>
+  <si>
     <t>52000</t>
   </si>
   <si>
@@ -635,12 +638,12 @@
     <t>24000</t>
   </si>
   <si>
-    <t>21700</t>
-  </si>
-  <si>
     <t>신한투자증권</t>
   </si>
   <si>
+    <t>미래에셋증권,신영증권</t>
+  </si>
+  <si>
     <t>삼성증권,유진투자증권,유안타증권</t>
   </si>
   <si>
@@ -672,9 +675,6 @@
   </si>
   <si>
     <t>신영증권,유진투자증권</t>
-  </si>
-  <si>
-    <t>하나증권</t>
   </si>
 </sst>
 </file>
@@ -2456,10 +2456,10 @@
         <v>139</v>
       </c>
       <c r="B2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C2" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D2" t="s">
         <v>107</v>
@@ -2476,10 +2476,10 @@
         <v>140</v>
       </c>
       <c r="B3" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C3" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D3" t="s">
         <v>107</v>
@@ -2496,10 +2496,10 @@
         <v>141</v>
       </c>
       <c r="B4" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C4" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D4" t="s">
         <v>107</v>
@@ -2516,16 +2516,16 @@
         <v>142</v>
       </c>
       <c r="B5" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="C5" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D5" t="s">
         <v>107</v>
       </c>
       <c r="E5" t="s">
-        <v>107</v>
+        <v>197</v>
       </c>
       <c r="F5" t="s">
         <v>210</v>
@@ -2536,19 +2536,19 @@
         <v>143</v>
       </c>
       <c r="B6" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C6" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="D6" t="s">
         <v>107</v>
       </c>
       <c r="E6" t="s">
-        <v>197</v>
+        <v>107</v>
       </c>
       <c r="F6" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -2556,19 +2556,19 @@
         <v>144</v>
       </c>
       <c r="B7" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C7" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="D7" t="s">
         <v>107</v>
       </c>
       <c r="E7" t="s">
-        <v>107</v>
+        <v>198</v>
       </c>
       <c r="F7" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -2576,16 +2576,16 @@
         <v>145</v>
       </c>
       <c r="B8" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C8" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="D8" t="s">
         <v>107</v>
       </c>
       <c r="E8" t="s">
-        <v>198</v>
+        <v>107</v>
       </c>
       <c r="F8" t="s">
         <v>212</v>
@@ -2596,19 +2596,19 @@
         <v>146</v>
       </c>
       <c r="B9" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C9" t="s">
-        <v>172</v>
+        <v>180</v>
       </c>
       <c r="D9" t="s">
         <v>107</v>
       </c>
       <c r="E9" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="F9" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -2616,16 +2616,16 @@
         <v>147</v>
       </c>
       <c r="B10" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C10" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="D10" t="s">
         <v>107</v>
       </c>
       <c r="E10" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="F10" t="s">
         <v>213</v>
@@ -2636,19 +2636,19 @@
         <v>148</v>
       </c>
       <c r="B11" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C11" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D11" t="s">
         <v>107</v>
       </c>
       <c r="E11" t="s">
-        <v>107</v>
+        <v>200</v>
       </c>
       <c r="F11" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -2656,19 +2656,19 @@
         <v>149</v>
       </c>
       <c r="B12" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C12" t="s">
-        <v>172</v>
+        <v>182</v>
       </c>
       <c r="D12" t="s">
         <v>107</v>
       </c>
       <c r="E12" t="s">
-        <v>200</v>
+        <v>107</v>
       </c>
       <c r="F12" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -2676,10 +2676,10 @@
         <v>150</v>
       </c>
       <c r="B13" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C13" t="s">
-        <v>181</v>
+        <v>173</v>
       </c>
       <c r="D13" t="s">
         <v>107</v>
@@ -2696,10 +2696,10 @@
         <v>151</v>
       </c>
       <c r="B14" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C14" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D14" t="s">
         <v>107</v>
@@ -2708,7 +2708,7 @@
         <v>202</v>
       </c>
       <c r="F14" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -2716,19 +2716,19 @@
         <v>152</v>
       </c>
       <c r="B15" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C15" t="s">
-        <v>172</v>
+        <v>184</v>
       </c>
       <c r="D15" t="s">
         <v>107</v>
       </c>
       <c r="E15" t="s">
-        <v>107</v>
+        <v>203</v>
       </c>
       <c r="F15" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -2736,16 +2736,16 @@
         <v>153</v>
       </c>
       <c r="B16" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C16" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="D16" t="s">
-        <v>188</v>
+        <v>107</v>
       </c>
       <c r="E16" t="s">
-        <v>203</v>
+        <v>107</v>
       </c>
       <c r="F16" t="s">
         <v>217</v>
@@ -2756,50 +2756,50 @@
         <v>154</v>
       </c>
       <c r="B17" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C17" t="s">
-        <v>172</v>
+        <v>185</v>
       </c>
       <c r="D17" t="s">
         <v>189</v>
       </c>
       <c r="E17" t="s">
-        <v>192</v>
+        <v>204</v>
       </c>
       <c r="F17" t="s">
-        <v>210</v>
+        <v>218</v>
       </c>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" t="s">
-        <v>71</v>
+        <v>155</v>
       </c>
       <c r="B18" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C18" t="s">
-        <v>184</v>
+        <v>173</v>
       </c>
       <c r="D18" t="s">
         <v>190</v>
       </c>
       <c r="E18" t="s">
-        <v>204</v>
+        <v>193</v>
       </c>
       <c r="F18" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" t="s">
-        <v>155</v>
+        <v>71</v>
       </c>
       <c r="B19" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C19" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D19" t="s">
         <v>191</v>
@@ -2808,47 +2808,47 @@
         <v>205</v>
       </c>
       <c r="F19" t="s">
-        <v>218</v>
+        <v>210</v>
       </c>
     </row>
     <row r="20" spans="1:6">
       <c r="A20" t="s">
-        <v>72</v>
+        <v>156</v>
       </c>
       <c r="B20" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C20" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D20" t="s">
         <v>192</v>
       </c>
       <c r="E20" t="s">
-        <v>192</v>
+        <v>206</v>
       </c>
       <c r="F20" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B21" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C21" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="D21" t="s">
         <v>193</v>
       </c>
       <c r="E21" t="s">
-        <v>206</v>
+        <v>193</v>
       </c>
       <c r="F21" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
RPA datasets push 2024-09-01
</commit_message>
<xml_diff>
--- a/datasets/ib-strategy-data.xlsx
+++ b/datasets/ib-strategy-data.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="203">
   <si>
     <t>수요예측(시작일)</t>
   </si>
@@ -128,9 +128,6 @@
     <t>2024-06-13</t>
   </si>
   <si>
-    <t>2024-06-11</t>
-  </si>
-  <si>
     <t>2024-08-08</t>
   </si>
   <si>
@@ -152,9 +149,6 @@
     <t>2024-06-19</t>
   </si>
   <si>
-    <t>2024-06-17</t>
-  </si>
-  <si>
     <t>2024-08-23</t>
   </si>
   <si>
@@ -185,9 +179,6 @@
     <t>2024-07-03</t>
   </si>
   <si>
-    <t>2024-07-02</t>
-  </si>
-  <si>
     <t>NH</t>
   </si>
   <si>
@@ -263,9 +254,6 @@
     <t>하스</t>
   </si>
   <si>
-    <t>이노스페이스</t>
-  </si>
-  <si>
     <t>949.3:1</t>
   </si>
   <si>
@@ -311,9 +299,6 @@
     <t>946.40:1</t>
   </si>
   <si>
-    <t>598.87:1</t>
-  </si>
-  <si>
     <t>0.24%</t>
   </si>
   <si>
@@ -347,9 +332,6 @@
     <t>6.36%</t>
   </si>
   <si>
-    <t>1.99%</t>
-  </si>
-  <si>
     <t>첨단바이오의약품 위탁개발생산(CDMO) 서비스 / 차세대 세포,유전자 치료제</t>
   </si>
   <si>
@@ -390,9 +372,6 @@
   </si>
   <si>
     <t>리튬디실리케이트 수복소재(Amber block, Amber Ingot 등), 지르코니아 유치관</t>
-  </si>
-  <si>
-    <t>소형발사체, 로켓추진기관, 과학로켓, 시험평가용역</t>
   </si>
   <si>
     <t>종목명</t>
@@ -1002,7 +981,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Y17"/>
+  <dimension ref="A1:Y16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:25">
@@ -1087,16 +1066,16 @@
         <v>25</v>
       </c>
       <c r="B2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C2" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="D2" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="E2" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="F2">
         <v>1566800</v>
@@ -1123,10 +1102,10 @@
         <v>15300</v>
       </c>
       <c r="N2" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="O2" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="P2">
         <v>7367362</v>
@@ -1156,7 +1135,7 @@
         <v>-2903334</v>
       </c>
       <c r="Y2" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
     </row>
     <row r="3" spans="1:25">
@@ -1164,16 +1143,16 @@
         <v>26</v>
       </c>
       <c r="B3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C3" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D3" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="E3" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F3">
         <v>1000000</v>
@@ -1200,10 +1179,10 @@
         <v>13000</v>
       </c>
       <c r="N3" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="O3" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="P3">
         <v>25588</v>
@@ -1233,7 +1212,7 @@
         <v>809</v>
       </c>
       <c r="Y3" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
     </row>
     <row r="4" spans="1:25">
@@ -1241,16 +1220,16 @@
         <v>27</v>
       </c>
       <c r="B4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C4" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="D4" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="E4" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="F4">
         <v>6500000</v>
@@ -1277,10 +1256,10 @@
         <v>2000</v>
       </c>
       <c r="N4" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="O4" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="P4">
         <v>0</v>
@@ -1310,7 +1289,7 @@
         <v>0</v>
       </c>
       <c r="Y4" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
     </row>
     <row r="5" spans="1:25">
@@ -1321,13 +1300,13 @@
         <v>27</v>
       </c>
       <c r="C5" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D5" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="E5" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="F5">
         <v>1400000</v>
@@ -1354,10 +1333,10 @@
         <v>15500</v>
       </c>
       <c r="N5" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="O5" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="P5">
         <v>10740898602</v>
@@ -1387,7 +1366,7 @@
         <v>219774608</v>
       </c>
       <c r="Y5" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="6" spans="1:25">
@@ -1398,13 +1377,13 @@
         <v>25</v>
       </c>
       <c r="C6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D6" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="E6" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="F6">
         <v>1000000</v>
@@ -1431,10 +1410,10 @@
         <v>29000</v>
       </c>
       <c r="N6" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="O6" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="P6">
         <v>0</v>
@@ -1464,7 +1443,7 @@
         <v>0</v>
       </c>
       <c r="Y6" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
     </row>
     <row r="7" spans="1:25">
@@ -1475,13 +1454,13 @@
         <v>25</v>
       </c>
       <c r="C7" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D7" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="E7" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="F7">
         <v>751000</v>
@@ -1508,10 +1487,10 @@
         <v>21000</v>
       </c>
       <c r="N7" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="O7" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="P7">
         <v>0</v>
@@ -1541,7 +1520,7 @@
         <v>0</v>
       </c>
       <c r="Y7" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
     </row>
     <row r="8" spans="1:25">
@@ -1552,13 +1531,13 @@
         <v>28</v>
       </c>
       <c r="C8" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D8" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="E8" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="F8">
         <v>5800000</v>
@@ -1585,10 +1564,10 @@
         <v>2000</v>
       </c>
       <c r="N8" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="O8" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="P8">
         <v>0</v>
@@ -1618,7 +1597,7 @@
         <v>0</v>
       </c>
       <c r="Y8" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
     </row>
     <row r="9" spans="1:25">
@@ -1629,13 +1608,13 @@
         <v>29</v>
       </c>
       <c r="C9" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D9" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="E9" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="F9">
         <v>1400000</v>
@@ -1662,10 +1641,10 @@
         <v>16000</v>
       </c>
       <c r="N9" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="O9" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="P9">
         <v>72895458363</v>
@@ -1695,7 +1674,7 @@
         <v>-3801868433</v>
       </c>
       <c r="Y9" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
     </row>
     <row r="10" spans="1:25">
@@ -1703,16 +1682,16 @@
         <v>31</v>
       </c>
       <c r="B10" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D10" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="E10" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="F10">
         <v>2234000</v>
@@ -1739,10 +1718,10 @@
         <v>10000</v>
       </c>
       <c r="N10" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="O10" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="P10">
         <v>1337894447</v>
@@ -1772,7 +1751,7 @@
         <v>-1257080998</v>
       </c>
       <c r="Y10" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
     </row>
     <row r="11" spans="1:25">
@@ -1780,16 +1759,16 @@
         <v>32</v>
       </c>
       <c r="B11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D11" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="E11" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="F11">
         <v>1350000</v>
@@ -1816,10 +1795,10 @@
         <v>22000</v>
       </c>
       <c r="N11" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="O11" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="P11">
         <v>5214628820</v>
@@ -1849,7 +1828,7 @@
         <v>24178632</v>
       </c>
       <c r="Y11" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
     </row>
     <row r="12" spans="1:25">
@@ -1857,16 +1836,16 @@
         <v>33</v>
       </c>
       <c r="B12" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C12" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D12" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="E12" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="F12">
         <v>6000000</v>
@@ -1893,10 +1872,10 @@
         <v>2000</v>
       </c>
       <c r="N12" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="O12" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="P12">
         <v>0</v>
@@ -1926,7 +1905,7 @@
         <v>0</v>
       </c>
       <c r="Y12" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
     </row>
     <row r="13" spans="1:25">
@@ -1934,16 +1913,16 @@
         <v>33</v>
       </c>
       <c r="B13" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C13" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D13" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="E13" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="F13">
         <v>4000000</v>
@@ -1970,10 +1949,10 @@
         <v>2000</v>
       </c>
       <c r="N13" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="O13" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="P13">
         <v>0</v>
@@ -2003,7 +1982,7 @@
         <v>0</v>
       </c>
       <c r="Y13" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
     </row>
     <row r="14" spans="1:25">
@@ -2011,16 +1990,16 @@
         <v>34</v>
       </c>
       <c r="B14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C14" t="s">
         <v>31</v>
       </c>
       <c r="D14" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="E14" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="F14">
         <v>1618000</v>
@@ -2047,10 +2026,10 @@
         <v>10000</v>
       </c>
       <c r="N14" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="O14" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="P14">
         <v>0</v>
@@ -2080,7 +2059,7 @@
         <v>0</v>
       </c>
       <c r="Y14" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
     </row>
     <row r="15" spans="1:25">
@@ -2088,16 +2067,16 @@
         <v>35</v>
       </c>
       <c r="B15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C15" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D15" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="E15" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="F15">
         <v>4000000</v>
@@ -2124,10 +2103,10 @@
         <v>2000</v>
       </c>
       <c r="N15" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="O15" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="P15">
         <v>0</v>
@@ -2157,7 +2136,7 @@
         <v>0</v>
       </c>
       <c r="Y15" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
     </row>
     <row r="16" spans="1:25">
@@ -2165,16 +2144,16 @@
         <v>36</v>
       </c>
       <c r="B16" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C16" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D16" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="E16" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="F16">
         <v>1810000</v>
@@ -2201,10 +2180,10 @@
         <v>16000</v>
       </c>
       <c r="N16" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="O16" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="P16">
         <v>12596039842</v>
@@ -2234,84 +2213,7 @@
         <v>1795726428</v>
       </c>
       <c r="Y16" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="17" spans="1:25">
-      <c r="A17" t="s">
-        <v>37</v>
-      </c>
-      <c r="B17" t="s">
-        <v>45</v>
-      </c>
-      <c r="C17" t="s">
-        <v>56</v>
-      </c>
-      <c r="D17" t="s">
-        <v>63</v>
-      </c>
-      <c r="E17" t="s">
-        <v>82</v>
-      </c>
-      <c r="F17">
-        <v>1330000</v>
-      </c>
-      <c r="G17">
-        <v>1330000</v>
-      </c>
-      <c r="H17">
-        <v>0</v>
-      </c>
-      <c r="I17">
-        <v>36400</v>
-      </c>
-      <c r="J17">
-        <v>43300</v>
-      </c>
-      <c r="K17">
-        <v>9375694</v>
-      </c>
-      <c r="L17">
-        <v>0</v>
-      </c>
-      <c r="M17">
-        <v>43300</v>
-      </c>
-      <c r="N17" t="s">
-        <v>98</v>
-      </c>
-      <c r="O17" t="s">
-        <v>110</v>
-      </c>
-      <c r="P17">
-        <v>103267682</v>
-      </c>
-      <c r="Q17">
-        <v>342201581</v>
-      </c>
-      <c r="R17">
-        <v>231425455</v>
-      </c>
-      <c r="S17">
-        <v>-7598692896</v>
-      </c>
-      <c r="T17">
-        <v>-25822444575</v>
-      </c>
-      <c r="U17">
-        <v>-15929213281</v>
-      </c>
-      <c r="V17">
-        <v>-6973258680</v>
-      </c>
-      <c r="W17">
-        <v>-48433907514</v>
-      </c>
-      <c r="X17">
-        <v>-83246975113</v>
-      </c>
-      <c r="Y17" t="s">
-        <v>125</v>
+        <v>118</v>
       </c>
     </row>
   </sheetData>
@@ -2326,422 +2228,422 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="B2" t="s">
-        <v>152</v>
+        <v>145</v>
       </c>
       <c r="C2" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
       <c r="D2" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="E2" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="F2" t="s">
-        <v>198</v>
+        <v>191</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="B3" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
       <c r="C3" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
       <c r="D3" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="E3" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="F3" t="s">
-        <v>199</v>
+        <v>192</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="B4" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="C4" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="D4" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="E4" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="F4" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="B5" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
       <c r="C5" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="D5" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="E5" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
       <c r="F5" t="s">
-        <v>198</v>
+        <v>191</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="B6" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
       <c r="C6" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
       <c r="D6" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="E6" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="F6" t="s">
-        <v>201</v>
+        <v>194</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="B7" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
       <c r="C7" t="s">
-        <v>172</v>
+        <v>165</v>
       </c>
       <c r="D7" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="E7" t="s">
-        <v>187</v>
+        <v>180</v>
       </c>
       <c r="F7" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="B8" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="C8" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
       <c r="D8" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="E8" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="F8" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="B9" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="C9" t="s">
-        <v>174</v>
+        <v>167</v>
       </c>
       <c r="D9" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="E9" t="s">
-        <v>188</v>
+        <v>181</v>
       </c>
       <c r="F9" t="s">
-        <v>204</v>
+        <v>197</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="B10" t="s">
-        <v>158</v>
+        <v>151</v>
       </c>
       <c r="C10" t="s">
-        <v>175</v>
+        <v>168</v>
       </c>
       <c r="D10" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="E10" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="F10" t="s">
-        <v>205</v>
+        <v>198</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="B11" t="s">
-        <v>158</v>
+        <v>151</v>
       </c>
       <c r="C11" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
       <c r="D11" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="E11" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="F11" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="B12" t="s">
-        <v>159</v>
+        <v>152</v>
       </c>
       <c r="C12" t="s">
-        <v>177</v>
+        <v>170</v>
       </c>
       <c r="D12" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="E12" t="s">
-        <v>190</v>
+        <v>183</v>
       </c>
       <c r="F12" t="s">
-        <v>199</v>
+        <v>192</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="B13" t="s">
-        <v>159</v>
+        <v>152</v>
       </c>
       <c r="C13" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="D13" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="E13" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
       <c r="F13" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="B14" t="s">
-        <v>160</v>
+        <v>153</v>
       </c>
       <c r="C14" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
       <c r="D14" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="E14" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="F14" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="B15" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="C15" t="s">
-        <v>179</v>
+        <v>172</v>
       </c>
       <c r="D15" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="E15" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="F15" t="s">
-        <v>206</v>
+        <v>199</v>
       </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="B16" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="C16" t="s">
-        <v>180</v>
+        <v>173</v>
       </c>
       <c r="D16" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="E16" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="F16" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="B17" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="C17" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
       <c r="D17" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="E17" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="F17" t="s">
-        <v>207</v>
+        <v>200</v>
       </c>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" t="s">
-        <v>148</v>
+        <v>141</v>
       </c>
       <c r="B18" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
       <c r="C18" t="s">
-        <v>181</v>
+        <v>174</v>
       </c>
       <c r="D18" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="E18" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="F18" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="B19" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="C19" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
       <c r="D19" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
       <c r="E19" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="F19" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
     </row>
     <row r="20" spans="1:6">
       <c r="A20" t="s">
-        <v>150</v>
+        <v>143</v>
       </c>
       <c r="B20" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="C20" t="s">
-        <v>182</v>
+        <v>175</v>
       </c>
       <c r="D20" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="E20" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="F20" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="B21" t="s">
-        <v>166</v>
+        <v>159</v>
       </c>
       <c r="C21" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
       <c r="D21" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
       <c r="E21" t="s">
-        <v>197</v>
+        <v>190</v>
       </c>
       <c r="F21" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
RPA datasets push 2024-09-02
</commit_message>
<xml_diff>
--- a/datasets/ib-strategy-data.xlsx
+++ b/datasets/ib-strategy-data.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="203">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="196">
   <si>
     <t>수요예측(시작일)</t>
   </si>
@@ -125,9 +125,6 @@
     <t>2024-06-27</t>
   </si>
   <si>
-    <t>2024-06-13</t>
-  </si>
-  <si>
     <t>2024-08-08</t>
   </si>
   <si>
@@ -146,9 +143,6 @@
     <t>2024-06-28</t>
   </si>
   <si>
-    <t>2024-06-19</t>
-  </si>
-  <si>
     <t>2024-08-23</t>
   </si>
   <si>
@@ -176,9 +170,6 @@
     <t>2024-07-12</t>
   </si>
   <si>
-    <t>2024-07-03</t>
-  </si>
-  <si>
     <t>NH</t>
   </si>
   <si>
@@ -251,9 +242,6 @@
     <t>이베스트스팩6호</t>
   </si>
   <si>
-    <t>하스</t>
-  </si>
-  <si>
     <t>949.3:1</t>
   </si>
   <si>
@@ -296,9 +284,6 @@
     <t>1131.75:1</t>
   </si>
   <si>
-    <t>946.40:1</t>
-  </si>
-  <si>
     <t>0.24%</t>
   </si>
   <si>
@@ -329,9 +314,6 @@
     <t>4.50%</t>
   </si>
   <si>
-    <t>6.36%</t>
-  </si>
-  <si>
     <t>첨단바이오의약품 위탁개발생산(CDMO) 서비스 / 차세대 세포,유전자 치료제</t>
   </si>
   <si>
@@ -369,9 +351,6 @@
   </si>
   <si>
     <t>CellCor SFD/CD(세포배양배지)</t>
-  </si>
-  <si>
-    <t>리튬디실리케이트 수복소재(Amber block, Amber Ingot 등), 지르코니아 유치관</t>
   </si>
   <si>
     <t>종목명</t>
@@ -981,7 +960,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Y16"/>
+  <dimension ref="A1:Y15"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:25">
@@ -1066,16 +1045,16 @@
         <v>25</v>
       </c>
       <c r="B2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="E2" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="F2">
         <v>1566800</v>
@@ -1102,10 +1081,10 @@
         <v>15300</v>
       </c>
       <c r="N2" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="O2" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="P2">
         <v>7367362</v>
@@ -1135,7 +1114,7 @@
         <v>-2903334</v>
       </c>
       <c r="Y2" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
     </row>
     <row r="3" spans="1:25">
@@ -1143,16 +1122,16 @@
         <v>26</v>
       </c>
       <c r="B3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D3" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="E3" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="F3">
         <v>1000000</v>
@@ -1179,10 +1158,10 @@
         <v>13000</v>
       </c>
       <c r="N3" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="O3" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="P3">
         <v>25588</v>
@@ -1212,7 +1191,7 @@
         <v>809</v>
       </c>
       <c r="Y3" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4" spans="1:25">
@@ -1220,16 +1199,16 @@
         <v>27</v>
       </c>
       <c r="B4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C4" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="D4" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="E4" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="F4">
         <v>6500000</v>
@@ -1256,10 +1235,10 @@
         <v>2000</v>
       </c>
       <c r="N4" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="O4" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="P4">
         <v>0</v>
@@ -1289,7 +1268,7 @@
         <v>0</v>
       </c>
       <c r="Y4" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
     </row>
     <row r="5" spans="1:25">
@@ -1300,13 +1279,13 @@
         <v>27</v>
       </c>
       <c r="C5" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D5" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="E5" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="F5">
         <v>1400000</v>
@@ -1333,10 +1312,10 @@
         <v>15500</v>
       </c>
       <c r="N5" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="O5" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="P5">
         <v>10740898602</v>
@@ -1366,7 +1345,7 @@
         <v>219774608</v>
       </c>
       <c r="Y5" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
     </row>
     <row r="6" spans="1:25">
@@ -1377,13 +1356,13 @@
         <v>25</v>
       </c>
       <c r="C6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D6" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="E6" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F6">
         <v>1000000</v>
@@ -1410,10 +1389,10 @@
         <v>29000</v>
       </c>
       <c r="N6" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="O6" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="P6">
         <v>0</v>
@@ -1443,7 +1422,7 @@
         <v>0</v>
       </c>
       <c r="Y6" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
     </row>
     <row r="7" spans="1:25">
@@ -1454,13 +1433,13 @@
         <v>25</v>
       </c>
       <c r="C7" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="D7" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="E7" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="F7">
         <v>751000</v>
@@ -1487,10 +1466,10 @@
         <v>21000</v>
       </c>
       <c r="N7" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="O7" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="P7">
         <v>0</v>
@@ -1520,7 +1499,7 @@
         <v>0</v>
       </c>
       <c r="Y7" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
     </row>
     <row r="8" spans="1:25">
@@ -1531,13 +1510,13 @@
         <v>28</v>
       </c>
       <c r="C8" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D8" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="E8" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="F8">
         <v>5800000</v>
@@ -1564,10 +1543,10 @@
         <v>2000</v>
       </c>
       <c r="N8" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="O8" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="P8">
         <v>0</v>
@@ -1597,7 +1576,7 @@
         <v>0</v>
       </c>
       <c r="Y8" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
     </row>
     <row r="9" spans="1:25">
@@ -1608,13 +1587,13 @@
         <v>29</v>
       </c>
       <c r="C9" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D9" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="E9" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="F9">
         <v>1400000</v>
@@ -1641,10 +1620,10 @@
         <v>16000</v>
       </c>
       <c r="N9" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="O9" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="P9">
         <v>72895458363</v>
@@ -1674,7 +1653,7 @@
         <v>-3801868433</v>
       </c>
       <c r="Y9" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
     </row>
     <row r="10" spans="1:25">
@@ -1682,16 +1661,16 @@
         <v>31</v>
       </c>
       <c r="B10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D10" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="E10" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="F10">
         <v>2234000</v>
@@ -1718,10 +1697,10 @@
         <v>10000</v>
       </c>
       <c r="N10" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="O10" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="P10">
         <v>1337894447</v>
@@ -1751,7 +1730,7 @@
         <v>-1257080998</v>
       </c>
       <c r="Y10" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
     </row>
     <row r="11" spans="1:25">
@@ -1759,16 +1738,16 @@
         <v>32</v>
       </c>
       <c r="B11" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C11" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D11" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="E11" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="F11">
         <v>1350000</v>
@@ -1795,10 +1774,10 @@
         <v>22000</v>
       </c>
       <c r="N11" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="O11" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="P11">
         <v>5214628820</v>
@@ -1828,7 +1807,7 @@
         <v>24178632</v>
       </c>
       <c r="Y11" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="12" spans="1:25">
@@ -1836,16 +1815,16 @@
         <v>33</v>
       </c>
       <c r="B12" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C12" t="s">
+        <v>49</v>
+      </c>
+      <c r="D12" t="s">
         <v>51</v>
       </c>
-      <c r="D12" t="s">
-        <v>54</v>
-      </c>
       <c r="E12" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="F12">
         <v>6000000</v>
@@ -1872,10 +1851,10 @@
         <v>2000</v>
       </c>
       <c r="N12" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="O12" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="P12">
         <v>0</v>
@@ -1905,7 +1884,7 @@
         <v>0</v>
       </c>
       <c r="Y12" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
     </row>
     <row r="13" spans="1:25">
@@ -1913,16 +1892,16 @@
         <v>33</v>
       </c>
       <c r="B13" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C13" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D13" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="E13" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="F13">
         <v>4000000</v>
@@ -1949,10 +1928,10 @@
         <v>2000</v>
       </c>
       <c r="N13" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="O13" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="P13">
         <v>0</v>
@@ -1982,7 +1961,7 @@
         <v>0</v>
       </c>
       <c r="Y13" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
     </row>
     <row r="14" spans="1:25">
@@ -1990,16 +1969,16 @@
         <v>34</v>
       </c>
       <c r="B14" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C14" t="s">
         <v>31</v>
       </c>
       <c r="D14" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="E14" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="F14">
         <v>1618000</v>
@@ -2026,10 +2005,10 @@
         <v>10000</v>
       </c>
       <c r="N14" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="O14" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="P14">
         <v>0</v>
@@ -2059,7 +2038,7 @@
         <v>0</v>
       </c>
       <c r="Y14" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
     </row>
     <row r="15" spans="1:25">
@@ -2067,16 +2046,16 @@
         <v>35</v>
       </c>
       <c r="B15" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C15" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D15" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="E15" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="F15">
         <v>4000000</v>
@@ -2103,10 +2082,10 @@
         <v>2000</v>
       </c>
       <c r="N15" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="O15" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="P15">
         <v>0</v>
@@ -2136,84 +2115,7 @@
         <v>0</v>
       </c>
       <c r="Y15" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="16" spans="1:25">
-      <c r="A16" t="s">
-        <v>36</v>
-      </c>
-      <c r="B16" t="s">
-        <v>43</v>
-      </c>
-      <c r="C16" t="s">
-        <v>53</v>
-      </c>
-      <c r="D16" t="s">
-        <v>61</v>
-      </c>
-      <c r="E16" t="s">
-        <v>78</v>
-      </c>
-      <c r="F16">
-        <v>1810000</v>
-      </c>
-      <c r="G16">
-        <v>1810000</v>
-      </c>
-      <c r="H16">
-        <v>0</v>
-      </c>
-      <c r="I16">
-        <v>9000</v>
-      </c>
-      <c r="J16">
-        <v>12000</v>
-      </c>
-      <c r="K16">
-        <v>7836009</v>
-      </c>
-      <c r="L16">
-        <v>0</v>
-      </c>
-      <c r="M16">
-        <v>16000</v>
-      </c>
-      <c r="N16" t="s">
-        <v>93</v>
-      </c>
-      <c r="O16" t="s">
-        <v>104</v>
-      </c>
-      <c r="P16">
-        <v>12596039842</v>
-      </c>
-      <c r="Q16">
-        <v>14910346438</v>
-      </c>
-      <c r="R16">
-        <v>16039074617</v>
-      </c>
-      <c r="S16">
-        <v>1732604466</v>
-      </c>
-      <c r="T16">
-        <v>2893667787</v>
-      </c>
-      <c r="U16">
-        <v>1613779678</v>
-      </c>
-      <c r="V16">
-        <v>1558081149</v>
-      </c>
-      <c r="W16">
-        <v>2643467726</v>
-      </c>
-      <c r="X16">
-        <v>1795726428</v>
-      </c>
-      <c r="Y16" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
     </row>
   </sheetData>
@@ -2228,422 +2130,422 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>125</v>
+        <v>118</v>
       </c>
       <c r="B2" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="C2" t="s">
-        <v>160</v>
+        <v>153</v>
       </c>
       <c r="D2" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="E2" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="F2" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="B3" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="C3" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="D3" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="E3" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="F3" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="B4" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="C4" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="D4" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="E4" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="F4" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
       <c r="B5" t="s">
-        <v>148</v>
+        <v>141</v>
       </c>
       <c r="C5" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
       <c r="D5" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="E5" t="s">
-        <v>179</v>
+        <v>172</v>
       </c>
       <c r="F5" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="B6" t="s">
-        <v>148</v>
+        <v>141</v>
       </c>
       <c r="C6" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="D6" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="E6" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="F6" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="B7" t="s">
-        <v>148</v>
+        <v>141</v>
       </c>
       <c r="C7" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="D7" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="E7" t="s">
-        <v>180</v>
+        <v>173</v>
       </c>
       <c r="F7" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="B8" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="C8" t="s">
-        <v>166</v>
+        <v>159</v>
       </c>
       <c r="D8" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="E8" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="F8" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="B9" t="s">
-        <v>150</v>
+        <v>143</v>
       </c>
       <c r="C9" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
       <c r="D9" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="E9" t="s">
-        <v>181</v>
+        <v>174</v>
       </c>
       <c r="F9" t="s">
-        <v>197</v>
+        <v>190</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="B10" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="C10" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
       <c r="D10" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="E10" t="s">
-        <v>182</v>
+        <v>175</v>
       </c>
       <c r="F10" t="s">
-        <v>198</v>
+        <v>191</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="B11" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="C11" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="D11" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="E11" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="F11" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="B12" t="s">
-        <v>152</v>
+        <v>145</v>
       </c>
       <c r="C12" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="D12" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="E12" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
       <c r="F12" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="B13" t="s">
-        <v>152</v>
+        <v>145</v>
       </c>
       <c r="C13" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
       <c r="D13" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="E13" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="F13" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="B14" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
       <c r="C14" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="D14" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="E14" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="F14" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="B15" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="C15" t="s">
-        <v>172</v>
+        <v>165</v>
       </c>
       <c r="D15" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="E15" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="F15" t="s">
-        <v>199</v>
+        <v>192</v>
       </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="B16" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="C16" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
       <c r="D16" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="E16" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="F16" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="B17" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
       <c r="C17" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="D17" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="E17" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
       <c r="F17" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="B18" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="C18" t="s">
-        <v>174</v>
+        <v>167</v>
       </c>
       <c r="D18" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="E18" t="s">
-        <v>187</v>
+        <v>180</v>
       </c>
       <c r="F18" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="B19" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="C19" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="D19" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
       <c r="E19" t="s">
-        <v>188</v>
+        <v>181</v>
       </c>
       <c r="F19" t="s">
-        <v>201</v>
+        <v>194</v>
       </c>
     </row>
     <row r="20" spans="1:6">
       <c r="A20" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="B20" t="s">
-        <v>158</v>
+        <v>151</v>
       </c>
       <c r="C20" t="s">
-        <v>175</v>
+        <v>168</v>
       </c>
       <c r="D20" t="s">
-        <v>177</v>
+        <v>170</v>
       </c>
       <c r="E20" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="F20" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="B21" t="s">
-        <v>159</v>
+        <v>152</v>
       </c>
       <c r="C21" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="D21" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
       <c r="E21" t="s">
-        <v>190</v>
+        <v>183</v>
       </c>
       <c r="F21" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
RPA datasets push 2024-09-03
</commit_message>
<xml_diff>
--- a/datasets/ib-strategy-data.xlsx
+++ b/datasets/ib-strategy-data.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="197">
   <si>
     <t>수요예측(시작일)</t>
   </si>
@@ -377,6 +377,9 @@
     <t>신한스팩14호</t>
   </si>
   <si>
+    <t>와이제이링크</t>
+  </si>
+  <si>
     <t>탑런토탈솔루션</t>
   </si>
   <si>
@@ -404,9 +407,6 @@
     <t>에이치이엠파마(구.에이치이엠)</t>
   </si>
   <si>
-    <t>와이제이링크</t>
-  </si>
-  <si>
     <t>KB스팩30호</t>
   </si>
   <si>
@@ -437,6 +437,9 @@
     <t>2024.09.26~09.27</t>
   </si>
   <si>
+    <t>2024.09.25~10.02</t>
+  </si>
+  <si>
     <t>2024.09.24~09.30</t>
   </si>
   <si>
@@ -482,6 +485,9 @@
     <t>2,000~2,000</t>
   </si>
   <si>
+    <t>8,600~9,800</t>
+  </si>
+  <si>
     <t>12,000~14,000</t>
   </si>
   <si>
@@ -509,9 +515,6 @@
     <t>16,400~19,000</t>
   </si>
   <si>
-    <t>8,600~9,800</t>
-  </si>
-  <si>
     <t>28,000~34,000</t>
   </si>
   <si>
@@ -533,6 +536,9 @@
     <t>10000</t>
   </si>
   <si>
+    <t>30616</t>
+  </si>
+  <si>
     <t>18000</t>
   </si>
   <si>
@@ -546,9 +552,6 @@
   </si>
   <si>
     <t>11430</t>
-  </si>
-  <si>
-    <t>30616</t>
   </si>
   <si>
     <t>18480</t>
@@ -2156,7 +2159,7 @@
         <v>138</v>
       </c>
       <c r="C2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D2" t="s">
         <v>91</v>
@@ -2165,7 +2168,7 @@
         <v>91</v>
       </c>
       <c r="F2" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -2176,16 +2179,16 @@
         <v>139</v>
       </c>
       <c r="C3" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D3" t="s">
         <v>91</v>
       </c>
       <c r="E3" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="F3" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -2196,16 +2199,16 @@
         <v>140</v>
       </c>
       <c r="C4" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D4" t="s">
         <v>91</v>
       </c>
       <c r="E4" t="s">
-        <v>91</v>
+        <v>173</v>
       </c>
       <c r="F4" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -2216,16 +2219,16 @@
         <v>141</v>
       </c>
       <c r="C5" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D5" t="s">
         <v>91</v>
       </c>
       <c r="E5" t="s">
-        <v>172</v>
+        <v>91</v>
       </c>
       <c r="F5" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -2233,19 +2236,19 @@
         <v>122</v>
       </c>
       <c r="B6" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D6" t="s">
         <v>91</v>
       </c>
       <c r="E6" t="s">
-        <v>91</v>
+        <v>174</v>
       </c>
       <c r="F6" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -2253,16 +2256,16 @@
         <v>123</v>
       </c>
       <c r="B7" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C7" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D7" t="s">
         <v>91</v>
       </c>
       <c r="E7" t="s">
-        <v>173</v>
+        <v>91</v>
       </c>
       <c r="F7" t="s">
         <v>188</v>
@@ -2276,13 +2279,13 @@
         <v>142</v>
       </c>
       <c r="C8" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D8" t="s">
         <v>91</v>
       </c>
       <c r="E8" t="s">
-        <v>91</v>
+        <v>175</v>
       </c>
       <c r="F8" t="s">
         <v>189</v>
@@ -2296,13 +2299,13 @@
         <v>143</v>
       </c>
       <c r="C9" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D9" t="s">
         <v>91</v>
       </c>
       <c r="E9" t="s">
-        <v>174</v>
+        <v>91</v>
       </c>
       <c r="F9" t="s">
         <v>190</v>
@@ -2316,13 +2319,13 @@
         <v>144</v>
       </c>
       <c r="C10" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D10" t="s">
         <v>91</v>
       </c>
       <c r="E10" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F10" t="s">
         <v>191</v>
@@ -2333,19 +2336,19 @@
         <v>127</v>
       </c>
       <c r="B11" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C11" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D11" t="s">
         <v>91</v>
       </c>
       <c r="E11" t="s">
-        <v>91</v>
+        <v>177</v>
       </c>
       <c r="F11" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -2356,16 +2359,16 @@
         <v>145</v>
       </c>
       <c r="C12" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D12" t="s">
         <v>91</v>
       </c>
       <c r="E12" t="s">
-        <v>176</v>
+        <v>91</v>
       </c>
       <c r="F12" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -2373,16 +2376,16 @@
         <v>129</v>
       </c>
       <c r="B13" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C13" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D13" t="s">
         <v>91</v>
       </c>
       <c r="E13" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="F13" t="s">
         <v>186</v>
@@ -2393,19 +2396,19 @@
         <v>130</v>
       </c>
       <c r="B14" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C14" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D14" t="s">
         <v>91</v>
       </c>
       <c r="E14" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="F14" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -2413,19 +2416,19 @@
         <v>131</v>
       </c>
       <c r="B15" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C15" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D15" t="s">
         <v>91</v>
       </c>
       <c r="E15" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="F15" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -2433,10 +2436,10 @@
         <v>132</v>
       </c>
       <c r="B16" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C16" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D16" t="s">
         <v>91</v>
@@ -2445,7 +2448,7 @@
         <v>91</v>
       </c>
       <c r="F16" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -2453,19 +2456,19 @@
         <v>133</v>
       </c>
       <c r="B17" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C17" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D17" t="s">
         <v>91</v>
       </c>
       <c r="E17" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="F17" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="18" spans="1:6">
@@ -2473,19 +2476,19 @@
         <v>134</v>
       </c>
       <c r="B18" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C18" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D18" t="s">
         <v>91</v>
       </c>
       <c r="E18" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="F18" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="19" spans="1:6">
@@ -2493,19 +2496,19 @@
         <v>135</v>
       </c>
       <c r="B19" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C19" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D19" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="E19" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F19" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -2513,19 +2516,19 @@
         <v>136</v>
       </c>
       <c r="B20" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C20" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D20" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="E20" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="F20" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -2533,19 +2536,19 @@
         <v>137</v>
       </c>
       <c r="B21" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C21" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D21" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="E21" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F21" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
RPA datasets push 2024-09-05
</commit_message>
<xml_diff>
--- a/datasets/ib-strategy-data.xlsx
+++ b/datasets/ib-strategy-data.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="197">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="198">
   <si>
     <t>수요예측(시작일)</t>
   </si>
@@ -374,12 +374,18 @@
     <t>쓰리빌리언</t>
   </si>
   <si>
+    <t>루미르</t>
+  </si>
+  <si>
     <t>신한스팩14호</t>
   </si>
   <si>
     <t>와이제이링크</t>
   </si>
   <si>
+    <t>셀비온</t>
+  </si>
+  <si>
     <t>탑런토탈솔루션</t>
   </si>
   <si>
@@ -398,9 +404,6 @@
     <t>씨메스</t>
   </si>
   <si>
-    <t>루미르</t>
-  </si>
-  <si>
     <t>웨이비스</t>
   </si>
   <si>
@@ -413,9 +416,6 @@
     <t>제닉스</t>
   </si>
   <si>
-    <t>셀비온</t>
-  </si>
-  <si>
     <t>키움스팩9호</t>
   </si>
   <si>
@@ -434,6 +434,9 @@
     <t>2024.09.27~10.04</t>
   </si>
   <si>
+    <t>2024.09.26~10.04</t>
+  </si>
+  <si>
     <t>2024.09.26~09.27</t>
   </si>
   <si>
@@ -482,12 +485,18 @@
     <t>4,500~6,500</t>
   </si>
   <si>
+    <t>16,500~20,500</t>
+  </si>
+  <si>
     <t>2,000~2,000</t>
   </si>
   <si>
     <t>8,600~9,800</t>
   </si>
   <si>
+    <t>10,000~12,200</t>
+  </si>
+  <si>
     <t>12,000~14,000</t>
   </si>
   <si>
@@ -506,9 +515,6 @@
     <t>20,000~24,000</t>
   </si>
   <si>
-    <t>16,500~20,500</t>
-  </si>
-  <si>
     <t>11,000~12,500</t>
   </si>
   <si>
@@ -518,9 +524,6 @@
     <t>28,000~34,000</t>
   </si>
   <si>
-    <t>10,000~12,200</t>
-  </si>
-  <si>
     <t>4,900~5,700</t>
   </si>
   <si>
@@ -533,6 +536,9 @@
     <t>32000</t>
   </si>
   <si>
+    <t>49500</t>
+  </si>
+  <si>
     <t>10000</t>
   </si>
   <si>
@@ -548,9 +554,6 @@
     <t>52000</t>
   </si>
   <si>
-    <t>49500</t>
-  </si>
-  <si>
     <t>11430</t>
   </si>
   <si>
@@ -575,28 +578,28 @@
     <t>한국투자증권</t>
   </si>
   <si>
+    <t>NH투자증권</t>
+  </si>
+  <si>
     <t>신한투자증권</t>
   </si>
   <si>
     <t>KB증권</t>
   </si>
   <si>
+    <t>대신증권</t>
+  </si>
+  <si>
     <t>신영증권,유진증권</t>
   </si>
   <si>
     <t>미래에셋증권,신영증권</t>
   </si>
   <si>
-    <t>대신증권</t>
-  </si>
-  <si>
     <t>삼성증권,유진투자증권,유안타증권</t>
   </si>
   <si>
-    <t>NH투자증권</t>
-  </si>
-  <si>
-    <t>신영증권,케이비증권</t>
+    <t>신영증권,KB증권</t>
   </si>
   <si>
     <t>키움증권</t>
@@ -2159,7 +2162,7 @@
         <v>138</v>
       </c>
       <c r="C2" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D2" t="s">
         <v>91</v>
@@ -2168,7 +2171,7 @@
         <v>91</v>
       </c>
       <c r="F2" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -2179,16 +2182,16 @@
         <v>139</v>
       </c>
       <c r="C3" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D3" t="s">
         <v>91</v>
       </c>
       <c r="E3" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F3" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -2199,16 +2202,16 @@
         <v>140</v>
       </c>
       <c r="C4" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D4" t="s">
         <v>91</v>
       </c>
       <c r="E4" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="F4" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -2219,16 +2222,16 @@
         <v>141</v>
       </c>
       <c r="C5" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D5" t="s">
         <v>91</v>
       </c>
       <c r="E5" t="s">
-        <v>91</v>
+        <v>175</v>
       </c>
       <c r="F5" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -2239,16 +2242,16 @@
         <v>142</v>
       </c>
       <c r="C6" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D6" t="s">
         <v>91</v>
       </c>
       <c r="E6" t="s">
-        <v>174</v>
+        <v>91</v>
       </c>
       <c r="F6" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -2259,7 +2262,7 @@
         <v>142</v>
       </c>
       <c r="C7" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D7" t="s">
         <v>91</v>
@@ -2268,7 +2271,7 @@
         <v>91</v>
       </c>
       <c r="F7" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -2276,19 +2279,19 @@
         <v>124</v>
       </c>
       <c r="B8" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C8" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D8" t="s">
         <v>91</v>
       </c>
       <c r="E8" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F8" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -2299,7 +2302,7 @@
         <v>143</v>
       </c>
       <c r="C9" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D9" t="s">
         <v>91</v>
@@ -2308,7 +2311,7 @@
         <v>91</v>
       </c>
       <c r="F9" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -2316,19 +2319,19 @@
         <v>126</v>
       </c>
       <c r="B10" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C10" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D10" t="s">
         <v>91</v>
       </c>
       <c r="E10" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -2336,19 +2339,19 @@
         <v>127</v>
       </c>
       <c r="B11" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C11" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D11" t="s">
         <v>91</v>
       </c>
       <c r="E11" t="s">
-        <v>177</v>
+        <v>91</v>
       </c>
       <c r="F11" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -2359,16 +2362,16 @@
         <v>145</v>
       </c>
       <c r="C12" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D12" t="s">
         <v>91</v>
       </c>
       <c r="E12" t="s">
-        <v>91</v>
+        <v>178</v>
       </c>
       <c r="F12" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -2379,16 +2382,16 @@
         <v>146</v>
       </c>
       <c r="C13" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D13" t="s">
         <v>91</v>
       </c>
       <c r="E13" t="s">
-        <v>178</v>
+        <v>91</v>
       </c>
       <c r="F13" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -2399,16 +2402,16 @@
         <v>147</v>
       </c>
       <c r="C14" t="s">
-        <v>155</v>
+        <v>167</v>
       </c>
       <c r="D14" t="s">
         <v>91</v>
       </c>
       <c r="E14" t="s">
-        <v>172</v>
+        <v>179</v>
       </c>
       <c r="F14" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -2419,16 +2422,16 @@
         <v>148</v>
       </c>
       <c r="C15" t="s">
-        <v>166</v>
+        <v>157</v>
       </c>
       <c r="D15" t="s">
         <v>91</v>
       </c>
       <c r="E15" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="F15" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -2436,19 +2439,19 @@
         <v>132</v>
       </c>
       <c r="B16" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C16" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D16" t="s">
         <v>91</v>
       </c>
       <c r="E16" t="s">
-        <v>91</v>
+        <v>180</v>
       </c>
       <c r="F16" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -2456,19 +2459,19 @@
         <v>133</v>
       </c>
       <c r="B17" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C17" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D17" t="s">
         <v>91</v>
       </c>
       <c r="E17" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="F17" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="18" spans="1:6">
@@ -2476,16 +2479,16 @@
         <v>134</v>
       </c>
       <c r="B18" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C18" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D18" t="s">
         <v>91</v>
       </c>
       <c r="E18" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F18" t="s">
         <v>190</v>
@@ -2496,19 +2499,19 @@
         <v>135</v>
       </c>
       <c r="B19" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C19" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D19" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="E19" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="F19" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -2516,19 +2519,19 @@
         <v>136</v>
       </c>
       <c r="B20" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C20" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D20" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="E20" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F20" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -2536,16 +2539,16 @@
         <v>137</v>
       </c>
       <c r="B21" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C21" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D21" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="E21" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F21" t="s">
         <v>190</v>

</xml_diff>

<commit_message>
RPA datasets push 2024-09-06
</commit_message>
<xml_diff>
--- a/datasets/ib-strategy-data.xlsx
+++ b/datasets/ib-strategy-data.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="198">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="200">
   <si>
     <t>수요예측(시작일)</t>
   </si>
@@ -371,6 +371,9 @@
     <t>주간사</t>
   </si>
   <si>
+    <t>더본코리아(유가)</t>
+  </si>
+  <si>
     <t>쓰리빌리언</t>
   </si>
   <si>
@@ -428,7 +431,7 @@
     <t>아이스크림미디어(구.시공미디어)</t>
   </si>
   <si>
-    <t>대신밸런스스팩18호</t>
+    <t>2024.10.15~10.21</t>
   </si>
   <si>
     <t>2024.09.27~10.04</t>
@@ -479,7 +482,7 @@
     <t>2024.08.09~08.16</t>
   </si>
   <si>
-    <t>2024.08.05~08.06</t>
+    <t>23,000~28,000</t>
   </si>
   <si>
     <t>4,500~6,500</t>
@@ -536,6 +539,9 @@
     <t>32000</t>
   </si>
   <si>
+    <t>69000</t>
+  </si>
+  <si>
     <t>49500</t>
   </si>
   <si>
@@ -572,7 +578,7 @@
     <t>78720</t>
   </si>
   <si>
-    <t>13000</t>
+    <t>한국투자증권,NH투자증권</t>
   </si>
   <si>
     <t>한국투자증권</t>
@@ -2168,10 +2174,10 @@
         <v>91</v>
       </c>
       <c r="E2" t="s">
-        <v>91</v>
+        <v>174</v>
       </c>
       <c r="F2" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -2188,10 +2194,10 @@
         <v>91</v>
       </c>
       <c r="E3" t="s">
-        <v>173</v>
+        <v>91</v>
       </c>
       <c r="F3" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -2208,10 +2214,10 @@
         <v>91</v>
       </c>
       <c r="E4" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="F4" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -2228,10 +2234,10 @@
         <v>91</v>
       </c>
       <c r="E5" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F5" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -2248,10 +2254,10 @@
         <v>91</v>
       </c>
       <c r="E6" t="s">
-        <v>91</v>
+        <v>177</v>
       </c>
       <c r="F6" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -2259,7 +2265,7 @@
         <v>123</v>
       </c>
       <c r="B7" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C7" t="s">
         <v>160</v>
@@ -2271,7 +2277,7 @@
         <v>91</v>
       </c>
       <c r="F7" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -2288,10 +2294,10 @@
         <v>91</v>
       </c>
       <c r="E8" t="s">
-        <v>176</v>
+        <v>91</v>
       </c>
       <c r="F8" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -2299,7 +2305,7 @@
         <v>125</v>
       </c>
       <c r="B9" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C9" t="s">
         <v>162</v>
@@ -2308,10 +2314,10 @@
         <v>91</v>
       </c>
       <c r="E9" t="s">
-        <v>91</v>
+        <v>178</v>
       </c>
       <c r="F9" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -2319,7 +2325,7 @@
         <v>126</v>
       </c>
       <c r="B10" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C10" t="s">
         <v>163</v>
@@ -2328,10 +2334,10 @@
         <v>91</v>
       </c>
       <c r="E10" t="s">
-        <v>177</v>
+        <v>91</v>
       </c>
       <c r="F10" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -2348,10 +2354,10 @@
         <v>91</v>
       </c>
       <c r="E11" t="s">
-        <v>91</v>
+        <v>179</v>
       </c>
       <c r="F11" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -2368,10 +2374,10 @@
         <v>91</v>
       </c>
       <c r="E12" t="s">
-        <v>178</v>
+        <v>91</v>
       </c>
       <c r="F12" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -2388,10 +2394,10 @@
         <v>91</v>
       </c>
       <c r="E13" t="s">
-        <v>91</v>
+        <v>180</v>
       </c>
       <c r="F13" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -2408,10 +2414,10 @@
         <v>91</v>
       </c>
       <c r="E14" t="s">
-        <v>179</v>
+        <v>91</v>
       </c>
       <c r="F14" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -2422,16 +2428,16 @@
         <v>148</v>
       </c>
       <c r="C15" t="s">
-        <v>157</v>
+        <v>168</v>
       </c>
       <c r="D15" t="s">
         <v>91</v>
       </c>
       <c r="E15" t="s">
-        <v>174</v>
+        <v>181</v>
       </c>
       <c r="F15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -2442,16 +2448,16 @@
         <v>149</v>
       </c>
       <c r="C16" t="s">
-        <v>168</v>
+        <v>158</v>
       </c>
       <c r="D16" t="s">
         <v>91</v>
       </c>
       <c r="E16" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="F16" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -2462,16 +2468,16 @@
         <v>150</v>
       </c>
       <c r="C17" t="s">
-        <v>157</v>
+        <v>169</v>
       </c>
       <c r="D17" t="s">
         <v>91</v>
       </c>
       <c r="E17" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F17" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="18" spans="1:6">
@@ -2482,16 +2488,16 @@
         <v>151</v>
       </c>
       <c r="C18" t="s">
-        <v>169</v>
+        <v>158</v>
       </c>
       <c r="D18" t="s">
         <v>91</v>
       </c>
       <c r="E18" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="F18" t="s">
-        <v>190</v>
+        <v>197</v>
       </c>
     </row>
     <row r="19" spans="1:6">
@@ -2502,16 +2508,16 @@
         <v>152</v>
       </c>
       <c r="C19" t="s">
-        <v>157</v>
+        <v>170</v>
       </c>
       <c r="D19" t="s">
-        <v>171</v>
+        <v>91</v>
       </c>
       <c r="E19" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F19" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -2522,16 +2528,16 @@
         <v>153</v>
       </c>
       <c r="C20" t="s">
-        <v>170</v>
+        <v>158</v>
       </c>
       <c r="D20" t="s">
         <v>172</v>
       </c>
       <c r="E20" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F20" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -2542,16 +2548,16 @@
         <v>154</v>
       </c>
       <c r="C21" t="s">
-        <v>157</v>
+        <v>171</v>
       </c>
       <c r="D21" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="E21" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="F21" t="s">
-        <v>190</v>
+        <v>199</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
RPA datasets push 2024-09-11
</commit_message>
<xml_diff>
--- a/datasets/ib-strategy-data.xlsx
+++ b/datasets/ib-strategy-data.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="199">
   <si>
     <t>수요예측(시작일)</t>
   </si>
@@ -92,6 +92,9 @@
     <t>주요제품</t>
   </si>
   <si>
+    <t>2024-08-26</t>
+  </si>
+  <si>
     <t>2024-08-02</t>
   </si>
   <si>
@@ -122,7 +125,7 @@
     <t>2024-06-24</t>
   </si>
   <si>
-    <t>2024-06-27</t>
+    <t>2024-08-27</t>
   </si>
   <si>
     <t>2024-08-08</t>
@@ -143,6 +146,9 @@
     <t>2024-06-28</t>
   </si>
   <si>
+    <t>2024-09-11</t>
+  </si>
+  <si>
     <t>2024-08-23</t>
   </si>
   <si>
@@ -167,7 +173,7 @@
     <t>2024-07-26</t>
   </si>
   <si>
-    <t>2024-07-12</t>
+    <t>미래</t>
   </si>
   <si>
     <t>NH</t>
@@ -188,16 +194,13 @@
     <t>교보</t>
   </si>
   <si>
-    <t>미래</t>
-  </si>
-  <si>
     <t>삼성</t>
   </si>
   <si>
     <t>SK</t>
   </si>
   <si>
-    <t>엘에스</t>
+    <t>미래에셋비전스팩7호</t>
   </si>
   <si>
     <t>이엔셀</t>
@@ -239,7 +242,7 @@
     <t>엑셀세라퓨틱스</t>
   </si>
   <si>
-    <t>이베스트스팩6호</t>
+    <t>1051.62 :1</t>
   </si>
   <si>
     <t>949.3:1</t>
@@ -281,7 +284,7 @@
     <t>1233.80:1</t>
   </si>
   <si>
-    <t>1131.75:1</t>
+    <t>-</t>
   </si>
   <si>
     <t>0.24%</t>
@@ -290,9 +293,6 @@
     <t>4.23%</t>
   </si>
   <si>
-    <t>-</t>
-  </si>
-  <si>
     <t>1.03%</t>
   </si>
   <si>
@@ -314,6 +314,9 @@
     <t>4.50%</t>
   </si>
   <si>
+    <t>기업인수합병</t>
+  </si>
+  <si>
     <t>첨단바이오의약품 위탁개발생산(CDMO) 서비스 / 차세대 세포,유전자 치료제</t>
   </si>
   <si>
@@ -332,9 +335,6 @@
     <t>모바일 앱 개발 플랫폼</t>
   </si>
   <si>
-    <t>기업인수합병</t>
-  </si>
-  <si>
     <t>국내외 은행 및 금융기업 대상 코어뱅킹 소프트웨어</t>
   </si>
   <si>
@@ -374,6 +374,9 @@
     <t>더본코리아(유가)</t>
   </si>
   <si>
+    <t>씨메스</t>
+  </si>
+  <si>
     <t>쓰리빌리언</t>
   </si>
   <si>
@@ -404,9 +407,6 @@
     <t>토모큐브</t>
   </si>
   <si>
-    <t>씨메스</t>
-  </si>
-  <si>
     <t>웨이비스</t>
   </si>
   <si>
@@ -422,9 +422,6 @@
     <t>아이언디바이스</t>
   </si>
   <si>
-    <t>미래에셋비전스팩7호</t>
-  </si>
-  <si>
     <t>아이스크림미디어(구.시공미디어)</t>
   </si>
   <si>
@@ -434,6 +431,9 @@
     <t>2024.10.15~10.21</t>
   </si>
   <si>
+    <t>2024.09.30~10.08</t>
+  </si>
+  <si>
     <t>2024.09.27~10.04</t>
   </si>
   <si>
@@ -455,9 +455,6 @@
     <t>2024.09.20~09.26</t>
   </si>
   <si>
-    <t>2024.09.19~09.25</t>
-  </si>
-  <si>
     <t>2024.09.09~09.13</t>
   </si>
   <si>
@@ -485,6 +482,9 @@
     <t>23,000~28,000</t>
   </si>
   <si>
+    <t>20,000~24,000</t>
+  </si>
+  <si>
     <t>4,500~6,500</t>
   </si>
   <si>
@@ -515,9 +515,6 @@
     <t>10,900~13,400</t>
   </si>
   <si>
-    <t>20,000~24,000</t>
-  </si>
-  <si>
     <t>11,000~12,500</t>
   </si>
   <si>
@@ -545,6 +542,9 @@
     <t>69000</t>
   </si>
   <si>
+    <t>52000</t>
+  </si>
+  <si>
     <t>49500</t>
   </si>
   <si>
@@ -560,9 +560,6 @@
     <t>28200</t>
   </si>
   <si>
-    <t>52000</t>
-  </si>
-  <si>
     <t>11430</t>
   </si>
   <si>
@@ -584,6 +581,9 @@
     <t>한국투자증권,NH투자증권</t>
   </si>
   <si>
+    <t>삼성증권,유진투자증권,유안타증권</t>
+  </si>
+  <si>
     <t>한국투자증권</t>
   </si>
   <si>
@@ -603,9 +603,6 @@
   </si>
   <si>
     <t>미래에셋증권,신영증권</t>
-  </si>
-  <si>
-    <t>삼성증권,유진투자증권,유안타증권</t>
   </si>
   <si>
     <t>신영증권,KB증권</t>
@@ -1060,37 +1057,37 @@
         <v>36</v>
       </c>
       <c r="C2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E2" t="s">
         <v>61</v>
       </c>
       <c r="F2">
-        <v>1566800</v>
+        <v>7950000</v>
       </c>
       <c r="G2">
-        <v>1566800</v>
+        <v>7950000</v>
       </c>
       <c r="H2">
         <v>0</v>
       </c>
       <c r="I2">
-        <v>13600</v>
+        <v>2000</v>
       </c>
       <c r="J2">
-        <v>15300</v>
+        <v>2000</v>
       </c>
       <c r="K2">
-        <v>9349954</v>
+        <v>8215000</v>
       </c>
       <c r="L2">
         <v>0</v>
       </c>
       <c r="M2">
-        <v>15300</v>
+        <v>2000</v>
       </c>
       <c r="N2" t="s">
         <v>75</v>
@@ -1099,31 +1096,31 @@
         <v>89</v>
       </c>
       <c r="P2">
-        <v>7367362</v>
+        <v>0</v>
       </c>
       <c r="Q2">
-        <v>10525887</v>
+        <v>0</v>
       </c>
       <c r="R2">
-        <v>1790340</v>
+        <v>0</v>
       </c>
       <c r="S2">
-        <v>-9315442</v>
+        <v>0</v>
       </c>
       <c r="T2">
-        <v>-11755057</v>
+        <v>0</v>
       </c>
       <c r="U2">
-        <v>-2929307</v>
+        <v>0</v>
       </c>
       <c r="V2">
-        <v>-45566953</v>
+        <v>0</v>
       </c>
       <c r="W2">
-        <v>-5053520</v>
+        <v>0</v>
       </c>
       <c r="X2">
-        <v>-2903334</v>
+        <v>0</v>
       </c>
       <c r="Y2" t="s">
         <v>99</v>
@@ -1137,37 +1134,37 @@
         <v>37</v>
       </c>
       <c r="C3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E3" t="s">
         <v>62</v>
       </c>
       <c r="F3">
-        <v>1000000</v>
+        <v>1566800</v>
       </c>
       <c r="G3">
-        <v>500000</v>
+        <v>1566800</v>
       </c>
       <c r="H3">
-        <v>500000</v>
+        <v>0</v>
       </c>
       <c r="I3">
-        <v>9500</v>
+        <v>13600</v>
       </c>
       <c r="J3">
-        <v>10700</v>
+        <v>15300</v>
       </c>
       <c r="K3">
-        <v>5530000</v>
+        <v>9349954</v>
       </c>
       <c r="L3">
         <v>0</v>
       </c>
       <c r="M3">
-        <v>13000</v>
+        <v>15300</v>
       </c>
       <c r="N3" t="s">
         <v>76</v>
@@ -1176,31 +1173,31 @@
         <v>90</v>
       </c>
       <c r="P3">
-        <v>25588</v>
+        <v>7367362</v>
       </c>
       <c r="Q3">
-        <v>30049</v>
+        <v>10525887</v>
       </c>
       <c r="R3">
-        <v>7363</v>
+        <v>1790340</v>
       </c>
       <c r="S3">
-        <v>3780</v>
+        <v>-9315442</v>
       </c>
       <c r="T3">
-        <v>5016</v>
+        <v>-11755057</v>
       </c>
       <c r="U3">
-        <v>938</v>
+        <v>-2929307</v>
       </c>
       <c r="V3">
-        <v>3456</v>
+        <v>-45566953</v>
       </c>
       <c r="W3">
-        <v>4688</v>
+        <v>-5053520</v>
       </c>
       <c r="X3">
-        <v>809</v>
+        <v>-2903334</v>
       </c>
       <c r="Y3" t="s">
         <v>100</v>
@@ -1211,40 +1208,40 @@
         <v>27</v>
       </c>
       <c r="B4" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E4" t="s">
         <v>63</v>
       </c>
       <c r="F4">
-        <v>6500000</v>
+        <v>1000000</v>
       </c>
       <c r="G4">
-        <v>6500000</v>
+        <v>500000</v>
       </c>
       <c r="H4">
-        <v>0</v>
+        <v>500000</v>
       </c>
       <c r="I4">
-        <v>2000</v>
+        <v>9500</v>
       </c>
       <c r="J4">
-        <v>2000</v>
+        <v>10700</v>
       </c>
       <c r="K4">
-        <v>7910000</v>
+        <v>5530000</v>
       </c>
       <c r="L4">
         <v>0</v>
       </c>
       <c r="M4">
-        <v>2000</v>
+        <v>13000</v>
       </c>
       <c r="N4" t="s">
         <v>77</v>
@@ -1253,31 +1250,31 @@
         <v>91</v>
       </c>
       <c r="P4">
-        <v>0</v>
+        <v>25588</v>
       </c>
       <c r="Q4">
-        <v>0</v>
+        <v>30049</v>
       </c>
       <c r="R4">
-        <v>0</v>
+        <v>7363</v>
       </c>
       <c r="S4">
-        <v>0</v>
+        <v>3780</v>
       </c>
       <c r="T4">
-        <v>0</v>
+        <v>5016</v>
       </c>
       <c r="U4">
-        <v>0</v>
+        <v>938</v>
       </c>
       <c r="V4">
-        <v>0</v>
+        <v>3456</v>
       </c>
       <c r="W4">
-        <v>0</v>
+        <v>4688</v>
       </c>
       <c r="X4">
-        <v>0</v>
+        <v>809</v>
       </c>
       <c r="Y4" t="s">
         <v>101</v>
@@ -1288,73 +1285,73 @@
         <v>28</v>
       </c>
       <c r="B5" t="s">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="C5" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D5" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E5" t="s">
         <v>64</v>
       </c>
       <c r="F5">
-        <v>1400000</v>
+        <v>6500000</v>
       </c>
       <c r="G5">
-        <v>1400000</v>
+        <v>6500000</v>
       </c>
       <c r="H5">
         <v>0</v>
       </c>
       <c r="I5">
-        <v>12500</v>
+        <v>2000</v>
       </c>
       <c r="J5">
-        <v>15500</v>
+        <v>2000</v>
       </c>
       <c r="K5">
-        <v>7486442</v>
+        <v>7910000</v>
       </c>
       <c r="L5">
         <v>0</v>
       </c>
       <c r="M5">
-        <v>15500</v>
+        <v>2000</v>
       </c>
       <c r="N5" t="s">
         <v>78</v>
       </c>
       <c r="O5" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="P5">
-        <v>10740898602</v>
+        <v>0</v>
       </c>
       <c r="Q5">
-        <v>13058877126</v>
+        <v>0</v>
       </c>
       <c r="R5">
-        <v>3506428302</v>
+        <v>0</v>
       </c>
       <c r="S5">
-        <v>1748628548</v>
+        <v>0</v>
       </c>
       <c r="T5">
-        <v>1115790858</v>
+        <v>0</v>
       </c>
       <c r="U5">
-        <v>191527654</v>
+        <v>0</v>
       </c>
       <c r="V5">
-        <v>1491084554</v>
+        <v>0</v>
       </c>
       <c r="W5">
-        <v>1185231988</v>
+        <v>0</v>
       </c>
       <c r="X5">
-        <v>219774608</v>
+        <v>0</v>
       </c>
       <c r="Y5" t="s">
         <v>102</v>
@@ -1365,73 +1362,73 @@
         <v>29</v>
       </c>
       <c r="B6" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="C6" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="D6" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="E6" t="s">
         <v>65</v>
       </c>
       <c r="F6">
-        <v>1000000</v>
+        <v>1400000</v>
       </c>
       <c r="G6">
-        <v>1000000</v>
+        <v>1400000</v>
       </c>
       <c r="H6">
         <v>0</v>
       </c>
       <c r="I6">
-        <v>24000</v>
+        <v>12500</v>
       </c>
       <c r="J6">
-        <v>29000</v>
+        <v>15500</v>
       </c>
       <c r="K6">
-        <v>8008066</v>
+        <v>7486442</v>
       </c>
       <c r="L6">
         <v>0</v>
       </c>
       <c r="M6">
-        <v>29000</v>
+        <v>15500</v>
       </c>
       <c r="N6" t="s">
         <v>79</v>
       </c>
       <c r="O6" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="P6">
-        <v>0</v>
+        <v>10740898602</v>
       </c>
       <c r="Q6">
-        <v>0</v>
+        <v>13058877126</v>
       </c>
       <c r="R6">
-        <v>0</v>
+        <v>3506428302</v>
       </c>
       <c r="S6">
-        <v>0</v>
+        <v>1748628548</v>
       </c>
       <c r="T6">
-        <v>0</v>
+        <v>1115790858</v>
       </c>
       <c r="U6">
-        <v>0</v>
+        <v>191527654</v>
       </c>
       <c r="V6">
-        <v>0</v>
+        <v>1491084554</v>
       </c>
       <c r="W6">
-        <v>0</v>
+        <v>1185231988</v>
       </c>
       <c r="X6">
-        <v>0</v>
+        <v>219774608</v>
       </c>
       <c r="Y6" t="s">
         <v>103</v>
@@ -1439,49 +1436,49 @@
     </row>
     <row r="7" spans="1:25">
       <c r="A7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B7" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C7" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="D7" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E7" t="s">
         <v>66</v>
       </c>
       <c r="F7">
-        <v>751000</v>
+        <v>1000000</v>
       </c>
       <c r="G7">
-        <v>203700</v>
+        <v>1000000</v>
       </c>
       <c r="H7">
-        <v>547300</v>
+        <v>0</v>
       </c>
       <c r="I7">
-        <v>18000</v>
+        <v>24000</v>
       </c>
       <c r="J7">
-        <v>21000</v>
+        <v>29000</v>
       </c>
       <c r="K7">
-        <v>4330068</v>
+        <v>8008066</v>
       </c>
       <c r="L7">
         <v>0</v>
       </c>
       <c r="M7">
-        <v>21000</v>
+        <v>29000</v>
       </c>
       <c r="N7" t="s">
         <v>80</v>
       </c>
       <c r="O7" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="P7">
         <v>0</v>
@@ -1516,49 +1513,49 @@
     </row>
     <row r="8" spans="1:25">
       <c r="A8" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B8" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C8" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D8" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E8" t="s">
         <v>67</v>
       </c>
       <c r="F8">
-        <v>5800000</v>
+        <v>751000</v>
       </c>
       <c r="G8">
-        <v>5800000</v>
+        <v>203700</v>
       </c>
       <c r="H8">
-        <v>0</v>
+        <v>547300</v>
       </c>
       <c r="I8">
-        <v>2000</v>
+        <v>18000</v>
       </c>
       <c r="J8">
-        <v>2000</v>
+        <v>21000</v>
       </c>
       <c r="K8">
-        <v>6100000</v>
+        <v>4330068</v>
       </c>
       <c r="L8">
         <v>0</v>
       </c>
       <c r="M8">
-        <v>2000</v>
+        <v>21000</v>
       </c>
       <c r="N8" t="s">
         <v>81</v>
       </c>
       <c r="O8" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="P8">
         <v>0</v>
@@ -1599,73 +1596,73 @@
         <v>29</v>
       </c>
       <c r="C9" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D9" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E9" t="s">
         <v>68</v>
       </c>
       <c r="F9">
-        <v>1400000</v>
+        <v>5800000</v>
       </c>
       <c r="G9">
-        <v>1400000</v>
+        <v>5800000</v>
       </c>
       <c r="H9">
         <v>0</v>
       </c>
       <c r="I9">
-        <v>16000</v>
+        <v>2000</v>
       </c>
       <c r="J9">
-        <v>19000</v>
+        <v>2000</v>
       </c>
       <c r="K9">
-        <v>10000988</v>
+        <v>6100000</v>
       </c>
       <c r="L9">
         <v>0</v>
       </c>
       <c r="M9">
-        <v>16000</v>
+        <v>2000</v>
       </c>
       <c r="N9" t="s">
         <v>82</v>
       </c>
       <c r="O9" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="P9">
-        <v>72895458363</v>
+        <v>0</v>
       </c>
       <c r="Q9">
-        <v>72913766913</v>
+        <v>0</v>
       </c>
       <c r="R9">
-        <v>11230711680</v>
+        <v>0</v>
       </c>
       <c r="S9">
-        <v>-6524077412</v>
+        <v>0</v>
       </c>
       <c r="T9">
-        <v>-4556157069</v>
+        <v>0</v>
       </c>
       <c r="U9">
-        <v>-3633759729</v>
+        <v>0</v>
       </c>
       <c r="V9">
-        <v>-11528915410</v>
+        <v>0</v>
       </c>
       <c r="W9">
-        <v>-7978634776</v>
+        <v>0</v>
       </c>
       <c r="X9">
-        <v>-3801868433</v>
+        <v>0</v>
       </c>
       <c r="Y9" t="s">
-        <v>106</v>
+        <v>99</v>
       </c>
     </row>
     <row r="10" spans="1:25">
@@ -1673,76 +1670,76 @@
         <v>31</v>
       </c>
       <c r="B10" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="C10" t="s">
-        <v>37</v>
+        <v>50</v>
       </c>
       <c r="D10" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="E10" t="s">
         <v>69</v>
       </c>
       <c r="F10">
-        <v>2234000</v>
+        <v>1400000</v>
       </c>
       <c r="G10">
-        <v>2234000</v>
+        <v>1400000</v>
       </c>
       <c r="H10">
         <v>0</v>
       </c>
       <c r="I10">
-        <v>7300</v>
+        <v>16000</v>
       </c>
       <c r="J10">
-        <v>8500</v>
+        <v>19000</v>
       </c>
       <c r="K10">
-        <v>14965620</v>
+        <v>10000988</v>
       </c>
       <c r="L10">
         <v>0</v>
       </c>
       <c r="M10">
-        <v>10000</v>
+        <v>16000</v>
       </c>
       <c r="N10" t="s">
         <v>83</v>
       </c>
       <c r="O10" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="P10">
-        <v>1337894447</v>
+        <v>72895458363</v>
       </c>
       <c r="Q10">
-        <v>4495088983</v>
+        <v>72913766913</v>
       </c>
       <c r="R10">
-        <v>99398351</v>
+        <v>11230711680</v>
       </c>
       <c r="S10">
-        <v>-3330678562</v>
+        <v>-6524077412</v>
       </c>
       <c r="T10">
-        <v>-2905069801</v>
+        <v>-4556157069</v>
       </c>
       <c r="U10">
-        <v>-1314068310</v>
+        <v>-3633759729</v>
       </c>
       <c r="V10">
-        <v>-9735376868</v>
+        <v>-11528915410</v>
       </c>
       <c r="W10">
-        <v>-5043515600</v>
+        <v>-7978634776</v>
       </c>
       <c r="X10">
-        <v>-1257080998</v>
+        <v>-3801868433</v>
       </c>
       <c r="Y10" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="11" spans="1:25">
@@ -1753,73 +1750,73 @@
         <v>39</v>
       </c>
       <c r="C11" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D11" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="E11" t="s">
         <v>70</v>
       </c>
       <c r="F11">
-        <v>1350000</v>
+        <v>2234000</v>
       </c>
       <c r="G11">
-        <v>1350000</v>
+        <v>2234000</v>
       </c>
       <c r="H11">
         <v>0</v>
       </c>
       <c r="I11">
-        <v>14000</v>
+        <v>7300</v>
       </c>
       <c r="J11">
-        <v>17000</v>
+        <v>8500</v>
       </c>
       <c r="K11">
-        <v>6471740</v>
+        <v>14965620</v>
       </c>
       <c r="L11">
         <v>0</v>
       </c>
       <c r="M11">
-        <v>22000</v>
+        <v>10000</v>
       </c>
       <c r="N11" t="s">
         <v>84</v>
       </c>
       <c r="O11" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="P11">
-        <v>5214628820</v>
+        <v>1337894447</v>
       </c>
       <c r="Q11">
-        <v>6009352447</v>
+        <v>4495088983</v>
       </c>
       <c r="R11">
-        <v>965797975</v>
+        <v>99398351</v>
       </c>
       <c r="S11">
-        <v>2015081728</v>
+        <v>-3330678562</v>
       </c>
       <c r="T11">
-        <v>1319755337</v>
+        <v>-2905069801</v>
       </c>
       <c r="U11">
-        <v>-44547594</v>
+        <v>-1314068310</v>
       </c>
       <c r="V11">
-        <v>1503069100</v>
+        <v>-9735376868</v>
       </c>
       <c r="W11">
-        <v>1410469786</v>
+        <v>-5043515600</v>
       </c>
       <c r="X11">
-        <v>24178632</v>
+        <v>-1257080998</v>
       </c>
       <c r="Y11" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="12" spans="1:25">
@@ -1830,96 +1827,96 @@
         <v>40</v>
       </c>
       <c r="C12" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="D12" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="E12" t="s">
         <v>71</v>
       </c>
       <c r="F12">
-        <v>6000000</v>
+        <v>1350000</v>
       </c>
       <c r="G12">
-        <v>6000000</v>
+        <v>1350000</v>
       </c>
       <c r="H12">
         <v>0</v>
       </c>
       <c r="I12">
-        <v>2000</v>
+        <v>14000</v>
       </c>
       <c r="J12">
-        <v>2000</v>
+        <v>17000</v>
       </c>
       <c r="K12">
-        <v>6345000</v>
+        <v>6471740</v>
       </c>
       <c r="L12">
         <v>0</v>
       </c>
       <c r="M12">
-        <v>2000</v>
+        <v>22000</v>
       </c>
       <c r="N12" t="s">
         <v>85</v>
       </c>
       <c r="O12" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="P12">
-        <v>0</v>
+        <v>5214628820</v>
       </c>
       <c r="Q12">
-        <v>0</v>
+        <v>6009352447</v>
       </c>
       <c r="R12">
-        <v>0</v>
+        <v>965797975</v>
       </c>
       <c r="S12">
-        <v>0</v>
+        <v>2015081728</v>
       </c>
       <c r="T12">
-        <v>0</v>
+        <v>1319755337</v>
       </c>
       <c r="U12">
-        <v>0</v>
+        <v>-44547594</v>
       </c>
       <c r="V12">
-        <v>0</v>
+        <v>1503069100</v>
       </c>
       <c r="W12">
-        <v>0</v>
+        <v>1410469786</v>
       </c>
       <c r="X12">
-        <v>0</v>
+        <v>24178632</v>
       </c>
       <c r="Y12" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="13" spans="1:25">
       <c r="A13" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B13" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C13" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="D13" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="E13" t="s">
         <v>72</v>
       </c>
       <c r="F13">
-        <v>4000000</v>
+        <v>6000000</v>
       </c>
       <c r="G13">
-        <v>4000000</v>
+        <v>6000000</v>
       </c>
       <c r="H13">
         <v>0</v>
@@ -1931,7 +1928,7 @@
         <v>2000</v>
       </c>
       <c r="K13">
-        <v>4420000</v>
+        <v>6345000</v>
       </c>
       <c r="L13">
         <v>0</v>
@@ -1943,7 +1940,7 @@
         <v>86</v>
       </c>
       <c r="O13" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="P13">
         <v>0</v>
@@ -1973,7 +1970,7 @@
         <v>0</v>
       </c>
       <c r="Y13" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="14" spans="1:25">
@@ -1984,43 +1981,43 @@
         <v>41</v>
       </c>
       <c r="C14" t="s">
-        <v>31</v>
+        <v>50</v>
       </c>
       <c r="D14" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="E14" t="s">
         <v>73</v>
       </c>
       <c r="F14">
-        <v>1618000</v>
+        <v>4000000</v>
       </c>
       <c r="G14">
-        <v>1618000</v>
+        <v>4000000</v>
       </c>
       <c r="H14">
         <v>0</v>
       </c>
       <c r="I14">
-        <v>6200</v>
+        <v>2000</v>
       </c>
       <c r="J14">
-        <v>7700</v>
+        <v>2000</v>
       </c>
       <c r="K14">
-        <v>10830212</v>
+        <v>4420000</v>
       </c>
       <c r="L14">
         <v>0</v>
       </c>
       <c r="M14">
-        <v>10000</v>
+        <v>2000</v>
       </c>
       <c r="N14" t="s">
         <v>87</v>
       </c>
       <c r="O14" t="s">
-        <v>98</v>
+        <v>89</v>
       </c>
       <c r="P14">
         <v>0</v>
@@ -2050,7 +2047,7 @@
         <v>0</v>
       </c>
       <c r="Y14" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="15" spans="1:25">
@@ -2058,46 +2055,46 @@
         <v>35</v>
       </c>
       <c r="B15" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C15" t="s">
-        <v>50</v>
+        <v>32</v>
       </c>
       <c r="D15" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="E15" t="s">
         <v>74</v>
       </c>
       <c r="F15">
-        <v>4000000</v>
+        <v>1618000</v>
       </c>
       <c r="G15">
-        <v>4000000</v>
+        <v>1618000</v>
       </c>
       <c r="H15">
         <v>0</v>
       </c>
       <c r="I15">
-        <v>2000</v>
+        <v>6200</v>
       </c>
       <c r="J15">
-        <v>2000</v>
+        <v>7700</v>
       </c>
       <c r="K15">
-        <v>5020000</v>
+        <v>10830212</v>
       </c>
       <c r="L15">
         <v>0</v>
       </c>
       <c r="M15">
-        <v>2000</v>
+        <v>10000</v>
       </c>
       <c r="N15" t="s">
         <v>88</v>
       </c>
       <c r="O15" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="P15">
         <v>0</v>
@@ -2127,7 +2124,7 @@
         <v>0</v>
       </c>
       <c r="Y15" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
   </sheetData>
@@ -2165,19 +2162,19 @@
         <v>118</v>
       </c>
       <c r="B2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C2" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E2" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="F2" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -2185,19 +2182,19 @@
         <v>119</v>
       </c>
       <c r="B3" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C3" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D3" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E3" t="s">
-        <v>91</v>
+        <v>175</v>
       </c>
       <c r="F3" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -2205,19 +2202,19 @@
         <v>120</v>
       </c>
       <c r="B4" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C4" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E4" t="s">
-        <v>176</v>
+        <v>89</v>
       </c>
       <c r="F4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -2225,19 +2222,19 @@
         <v>121</v>
       </c>
       <c r="B5" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D5" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E5" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F5" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -2245,19 +2242,19 @@
         <v>122</v>
       </c>
       <c r="B6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C6" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D6" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E6" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F6" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -2265,19 +2262,19 @@
         <v>123</v>
       </c>
       <c r="B7" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C7" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D7" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E7" t="s">
-        <v>91</v>
+        <v>178</v>
       </c>
       <c r="F7" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -2288,16 +2285,16 @@
         <v>143</v>
       </c>
       <c r="C8" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D8" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E8" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="F8" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -2305,19 +2302,19 @@
         <v>125</v>
       </c>
       <c r="B9" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C9" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D9" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E9" t="s">
-        <v>179</v>
+        <v>89</v>
       </c>
       <c r="F9" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -2328,16 +2325,16 @@
         <v>144</v>
       </c>
       <c r="C10" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D10" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E10" t="s">
-        <v>91</v>
+        <v>179</v>
       </c>
       <c r="F10" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -2348,16 +2345,16 @@
         <v>144</v>
       </c>
       <c r="C11" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D11" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E11" t="s">
-        <v>180</v>
+        <v>89</v>
       </c>
       <c r="F11" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -2365,19 +2362,19 @@
         <v>128</v>
       </c>
       <c r="B12" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C12" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D12" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E12" t="s">
-        <v>91</v>
+        <v>180</v>
       </c>
       <c r="F12" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -2385,19 +2382,19 @@
         <v>129</v>
       </c>
       <c r="B13" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C13" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D13" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E13" t="s">
-        <v>181</v>
+        <v>89</v>
       </c>
       <c r="F13" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -2405,16 +2402,16 @@
         <v>130</v>
       </c>
       <c r="B14" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C14" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D14" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E14" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="F14" t="s">
         <v>193</v>
@@ -2425,16 +2422,16 @@
         <v>131</v>
       </c>
       <c r="B15" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C15" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D15" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="F15" t="s">
         <v>191</v>
@@ -2445,13 +2442,13 @@
         <v>132</v>
       </c>
       <c r="B16" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C16" t="s">
         <v>158</v>
       </c>
       <c r="D16" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="E16" t="s">
         <v>177</v>
@@ -2465,19 +2462,19 @@
         <v>133</v>
       </c>
       <c r="B17" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C17" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D17" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E17" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="F17" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="18" spans="1:6">
@@ -2485,16 +2482,16 @@
         <v>134</v>
       </c>
       <c r="B18" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C18" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D18" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E18" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="F18" t="s">
         <v>193</v>
@@ -2502,59 +2499,59 @@
     </row>
     <row r="19" spans="1:6">
       <c r="A19" t="s">
-        <v>135</v>
+        <v>61</v>
       </c>
       <c r="B19" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C19" t="s">
         <v>158</v>
       </c>
       <c r="D19" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="E19" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F19" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="20" spans="1:6">
       <c r="A20" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B20" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C20" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D20" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="E20" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="F20" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B21" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C21" t="s">
         <v>158</v>
       </c>
       <c r="D21" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="E21" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="F21" t="s">
         <v>193</v>

</xml_diff>

<commit_message>
RPA datasets push 2024-09-13
</commit_message>
<xml_diff>
--- a/datasets/ib-strategy-data.xlsx
+++ b/datasets/ib-strategy-data.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="198">
   <si>
     <t>수요예측(시작일)</t>
   </si>
@@ -371,15 +371,24 @@
     <t>주간사</t>
   </si>
   <si>
+    <t>위츠</t>
+  </si>
+  <si>
     <t>더본코리아(유가)</t>
   </si>
   <si>
     <t>닷밀</t>
   </si>
   <si>
+    <t>성우</t>
+  </si>
+  <si>
     <t>웨이비스</t>
   </si>
   <si>
+    <t>클로봇</t>
+  </si>
+  <si>
     <t>씨메스</t>
   </si>
   <si>
@@ -407,9 +416,6 @@
     <t>한켐</t>
   </si>
   <si>
-    <t>클로봇</t>
-  </si>
-  <si>
     <t>토모큐브</t>
   </si>
   <si>
@@ -425,7 +431,7 @@
     <t>아이언디바이스</t>
   </si>
   <si>
-    <t>아이스크림미디어(구.시공미디어)</t>
+    <t>2024.10.28~11.01</t>
   </si>
   <si>
     <t>2024.10.15~10.21</t>
@@ -473,10 +479,7 @@
     <t>2024.08.30~09.05</t>
   </si>
   <si>
-    <t>2024.08.26~08.27</t>
-  </si>
-  <si>
-    <t>2024.08.09~08.16</t>
+    <t>5,300~6,400</t>
   </si>
   <si>
     <t>23,000~28,000</t>
@@ -485,9 +488,15 @@
     <t>11,000~13,000</t>
   </si>
   <si>
+    <t>25,000~29,000</t>
+  </si>
+  <si>
     <t>11,000~12,500</t>
   </si>
   <si>
+    <t>9,400~10,900</t>
+  </si>
+  <si>
     <t>20,000~24,000</t>
   </si>
   <si>
@@ -515,9 +524,6 @@
     <t>12,500~14,500</t>
   </si>
   <si>
-    <t>9,400~10,900</t>
-  </si>
-  <si>
     <t>10,900~13,400</t>
   </si>
   <si>
@@ -530,21 +536,24 @@
     <t>4,900~5,700</t>
   </si>
   <si>
-    <t>32,000~40,200</t>
-  </si>
-  <si>
     <t>2000</t>
   </si>
   <si>
     <t>7000</t>
   </si>
   <si>
-    <t>32000</t>
+    <t>15900</t>
   </si>
   <si>
     <t>69000</t>
   </si>
   <si>
+    <t>75000</t>
+  </si>
+  <si>
+    <t>28200</t>
+  </si>
+  <si>
     <t>52000</t>
   </si>
   <si>
@@ -560,9 +569,6 @@
     <t>18000</t>
   </si>
   <si>
-    <t>28200</t>
-  </si>
-  <si>
     <t>11430</t>
   </si>
   <si>
@@ -572,10 +578,7 @@
     <t>21000</t>
   </si>
   <si>
-    <t>15900</t>
-  </si>
-  <si>
-    <t>78720</t>
+    <t>신한투자증권</t>
   </si>
   <si>
     <t>한국투자증권,NH투자증권</t>
@@ -584,34 +587,28 @@
     <t>미래에셋증권</t>
   </si>
   <si>
+    <t>한국투자증권</t>
+  </si>
+  <si>
     <t>대신증권</t>
   </si>
   <si>
+    <t>미래에셋증권,신영증권</t>
+  </si>
+  <si>
     <t>삼성증권,유진투자증권,유안타증권</t>
   </si>
   <si>
-    <t>한국투자증권</t>
-  </si>
-  <si>
     <t>NH투자증권</t>
   </si>
   <si>
-    <t>신한투자증권</t>
-  </si>
-  <si>
     <t>KB증권</t>
   </si>
   <si>
     <t>신영증권,유진증권</t>
   </si>
   <si>
-    <t>미래에셋증권,신영증권</t>
-  </si>
-  <si>
     <t>신영증권,KB증권</t>
-  </si>
-  <si>
-    <t>삼성증권</t>
   </si>
 </sst>
 </file>
@@ -2162,7 +2159,7 @@
         <v>118</v>
       </c>
       <c r="B2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C2" t="s">
         <v>154</v>
@@ -2182,7 +2179,7 @@
         <v>119</v>
       </c>
       <c r="B3" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C3" t="s">
         <v>155</v>
@@ -2191,7 +2188,7 @@
         <v>89</v>
       </c>
       <c r="E3" t="s">
-        <v>89</v>
+        <v>176</v>
       </c>
       <c r="F3" t="s">
         <v>188</v>
@@ -2202,7 +2199,7 @@
         <v>120</v>
       </c>
       <c r="B4" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C4" t="s">
         <v>156</v>
@@ -2231,7 +2228,7 @@
         <v>89</v>
       </c>
       <c r="E5" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F5" t="s">
         <v>190</v>
@@ -2262,7 +2259,7 @@
         <v>123</v>
       </c>
       <c r="B7" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C7" t="s">
         <v>159</v>
@@ -2271,7 +2268,7 @@
         <v>89</v>
       </c>
       <c r="E7" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="F7" t="s">
         <v>192</v>
@@ -2282,7 +2279,7 @@
         <v>124</v>
       </c>
       <c r="B8" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C8" t="s">
         <v>160</v>
@@ -2291,7 +2288,7 @@
         <v>89</v>
       </c>
       <c r="E8" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="F8" t="s">
         <v>193</v>
@@ -2302,7 +2299,7 @@
         <v>125</v>
       </c>
       <c r="B9" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C9" t="s">
         <v>161</v>
@@ -2311,10 +2308,10 @@
         <v>89</v>
       </c>
       <c r="E9" t="s">
-        <v>179</v>
+        <v>89</v>
       </c>
       <c r="F9" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -2322,7 +2319,7 @@
         <v>126</v>
       </c>
       <c r="B10" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C10" t="s">
         <v>162</v>
@@ -2331,10 +2328,10 @@
         <v>89</v>
       </c>
       <c r="E10" t="s">
-        <v>89</v>
+        <v>180</v>
       </c>
       <c r="F10" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -2351,10 +2348,10 @@
         <v>89</v>
       </c>
       <c r="E11" t="s">
-        <v>89</v>
+        <v>181</v>
       </c>
       <c r="F11" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -2371,10 +2368,10 @@
         <v>89</v>
       </c>
       <c r="E12" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="F12" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -2382,7 +2379,7 @@
         <v>129</v>
       </c>
       <c r="B13" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C13" t="s">
         <v>165</v>
@@ -2394,7 +2391,7 @@
         <v>89</v>
       </c>
       <c r="F13" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -2402,7 +2399,7 @@
         <v>130</v>
       </c>
       <c r="B14" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C14" t="s">
         <v>166</v>
@@ -2411,10 +2408,10 @@
         <v>89</v>
       </c>
       <c r="E14" t="s">
-        <v>181</v>
+        <v>89</v>
       </c>
       <c r="F14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -2422,7 +2419,7 @@
         <v>131</v>
       </c>
       <c r="B15" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C15" t="s">
         <v>167</v>
@@ -2431,10 +2428,10 @@
         <v>89</v>
       </c>
       <c r="E15" t="s">
-        <v>89</v>
+        <v>183</v>
       </c>
       <c r="F15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -2451,10 +2448,10 @@
         <v>89</v>
       </c>
       <c r="E16" t="s">
-        <v>182</v>
+        <v>89</v>
       </c>
       <c r="F16" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -2465,16 +2462,16 @@
         <v>149</v>
       </c>
       <c r="C17" t="s">
-        <v>160</v>
+        <v>169</v>
       </c>
       <c r="D17" t="s">
-        <v>172</v>
+        <v>89</v>
       </c>
       <c r="E17" t="s">
-        <v>178</v>
+        <v>89</v>
       </c>
       <c r="F17" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
     </row>
     <row r="18" spans="1:6">
@@ -2485,16 +2482,16 @@
         <v>150</v>
       </c>
       <c r="C18" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D18" t="s">
         <v>89</v>
       </c>
       <c r="E18" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F18" t="s">
-        <v>197</v>
+        <v>187</v>
       </c>
     </row>
     <row r="19" spans="1:6">
@@ -2505,47 +2502,47 @@
         <v>151</v>
       </c>
       <c r="C19" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="D19" t="s">
         <v>173</v>
       </c>
       <c r="E19" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="F19" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
     </row>
     <row r="20" spans="1:6">
       <c r="A20" t="s">
-        <v>61</v>
+        <v>136</v>
       </c>
       <c r="B20" t="s">
         <v>152</v>
       </c>
       <c r="C20" t="s">
-        <v>160</v>
+        <v>171</v>
       </c>
       <c r="D20" t="s">
-        <v>172</v>
+        <v>89</v>
       </c>
       <c r="E20" t="s">
         <v>185</v>
       </c>
       <c r="F20" t="s">
-        <v>188</v>
+        <v>197</v>
       </c>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B21" t="s">
         <v>153</v>
       </c>
       <c r="C21" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D21" t="s">
         <v>174</v>
@@ -2554,7 +2551,7 @@
         <v>186</v>
       </c>
       <c r="F21" t="s">
-        <v>198</v>
+        <v>191</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
RPA datasets push 2024-09-14
</commit_message>
<xml_diff>
--- a/datasets/ib-strategy-data.xlsx
+++ b/datasets/ib-strategy-data.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="198">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="190">
   <si>
     <t>수요예측(시작일)</t>
   </si>
@@ -122,9 +122,6 @@
     <t>2024-07-09</t>
   </si>
   <si>
-    <t>2024-06-24</t>
-  </si>
-  <si>
     <t>2024-08-27</t>
   </si>
   <si>
@@ -143,9 +140,6 @@
     <t>2024-07-10</t>
   </si>
   <si>
-    <t>2024-06-28</t>
-  </si>
-  <si>
     <t>2024-09-11</t>
   </si>
   <si>
@@ -239,9 +233,6 @@
     <t>SK증권제13호스팩</t>
   </si>
   <si>
-    <t>엑셀세라퓨틱스</t>
-  </si>
-  <si>
     <t>1051.62 :1</t>
   </si>
   <si>
@@ -281,9 +272,6 @@
     <t>1197.45:1</t>
   </si>
   <si>
-    <t>1233.80:1</t>
-  </si>
-  <si>
     <t>-</t>
   </si>
   <si>
@@ -311,9 +299,6 @@
     <t>5.60%</t>
   </si>
   <si>
-    <t>4.50%</t>
-  </si>
-  <si>
     <t>기업인수합병</t>
   </si>
   <si>
@@ -350,9 +335,6 @@
     <t>기업인수목적 주식회사</t>
   </si>
   <si>
-    <t>CellCor SFD/CD(세포배양배지)</t>
-  </si>
-  <si>
     <t>종목명</t>
   </si>
   <si>
@@ -377,12 +359,24 @@
     <t>더본코리아(유가)</t>
   </si>
   <si>
+    <t>유진스팩11호</t>
+  </si>
+  <si>
+    <t>노머스</t>
+  </si>
+  <si>
     <t>닷밀</t>
   </si>
   <si>
+    <t>탑런토탈솔루션</t>
+  </si>
+  <si>
     <t>성우</t>
   </si>
   <si>
+    <t>케이뱅크(유가)</t>
+  </si>
+  <si>
     <t>웨이비스</t>
   </si>
   <si>
@@ -392,6 +386,9 @@
     <t>씨메스</t>
   </si>
   <si>
+    <t>에이치엔에스하이텍</t>
+  </si>
+  <si>
     <t>쓰리빌리언</t>
   </si>
   <si>
@@ -407,9 +404,6 @@
     <t>셀비온</t>
   </si>
   <si>
-    <t>탑런토탈솔루션</t>
-  </si>
-  <si>
     <t>인스피언</t>
   </si>
   <si>
@@ -419,24 +413,18 @@
     <t>토모큐브</t>
   </si>
   <si>
-    <t>에이치이엠파마(구.에이치이엠)</t>
-  </si>
-  <si>
-    <t>KB스팩30호</t>
-  </si>
-  <si>
-    <t>제닉스</t>
-  </si>
-  <si>
-    <t>아이언디바이스</t>
-  </si>
-  <si>
     <t>2024.10.28~11.01</t>
   </si>
   <si>
     <t>2024.10.15~10.21</t>
   </si>
   <si>
+    <t>2024.10.15~10.16</t>
+  </si>
+  <si>
+    <t>2024.10.11~10.17</t>
+  </si>
+  <si>
     <t>2024.10.10~10.16</t>
   </si>
   <si>
@@ -467,30 +455,30 @@
     <t>2024.09.20~09.26</t>
   </si>
   <si>
-    <t>2024.09.06~09.12</t>
-  </si>
-  <si>
-    <t>2024.09.05~09.06</t>
-  </si>
-  <si>
-    <t>2024.09.05~09.11</t>
-  </si>
-  <si>
-    <t>2024.08.30~09.05</t>
-  </si>
-  <si>
     <t>5,300~6,400</t>
   </si>
   <si>
     <t>23,000~28,000</t>
   </si>
   <si>
+    <t>2,000~2,000</t>
+  </si>
+  <si>
+    <t>27,200~30,200</t>
+  </si>
+  <si>
     <t>11,000~13,000</t>
   </si>
   <si>
+    <t>12,000~14,000</t>
+  </si>
+  <si>
     <t>25,000~29,000</t>
   </si>
   <si>
+    <t>9,500~12,000</t>
+  </si>
+  <si>
     <t>11,000~12,500</t>
   </si>
   <si>
@@ -500,24 +488,21 @@
     <t>20,000~24,000</t>
   </si>
   <si>
+    <t>22,000~26,000</t>
+  </si>
+  <si>
     <t>4,500~6,500</t>
   </si>
   <si>
     <t>16,500~20,500</t>
   </si>
   <si>
-    <t>2,000~2,000</t>
-  </si>
-  <si>
     <t>8,600~9,800</t>
   </si>
   <si>
     <t>10,000~12,200</t>
   </si>
   <si>
-    <t>12,000~14,000</t>
-  </si>
-  <si>
     <t>8,000~10,000</t>
   </si>
   <si>
@@ -527,36 +512,33 @@
     <t>10,900~13,400</t>
   </si>
   <si>
-    <t>16,400~19,000</t>
-  </si>
-  <si>
-    <t>28,000~34,000</t>
-  </si>
-  <si>
-    <t>4,900~5,700</t>
-  </si>
-  <si>
-    <t>2000</t>
-  </si>
-  <si>
-    <t>7000</t>
-  </si>
-  <si>
     <t>15900</t>
   </si>
   <si>
     <t>69000</t>
   </si>
   <si>
+    <t>9000</t>
+  </si>
+  <si>
+    <t>30736</t>
+  </si>
+  <si>
     <t>75000</t>
   </si>
   <si>
+    <t>779000</t>
+  </si>
+  <si>
     <t>28200</t>
   </si>
   <si>
     <t>52000</t>
   </si>
   <si>
+    <t>11000</t>
+  </si>
+  <si>
     <t>49500</t>
   </si>
   <si>
@@ -569,28 +551,28 @@
     <t>18000</t>
   </si>
   <si>
-    <t>11430</t>
-  </si>
-  <si>
-    <t>18480</t>
-  </si>
-  <si>
-    <t>21000</t>
-  </si>
-  <si>
     <t>신한투자증권</t>
   </si>
   <si>
     <t>한국투자증권,NH투자증권</t>
   </si>
   <si>
+    <t>유진증권</t>
+  </si>
+  <si>
+    <t>대신증권</t>
+  </si>
+  <si>
     <t>미래에셋증권</t>
   </si>
   <si>
+    <t>KB증권</t>
+  </si>
+  <si>
     <t>한국투자증권</t>
   </si>
   <si>
-    <t>대신증권</t>
+    <t>NH투자증권,KB증권,신한투자증권,키움증권</t>
   </si>
   <si>
     <t>미래에셋증권,신영증권</t>
@@ -602,13 +584,7 @@
     <t>NH투자증권</t>
   </si>
   <si>
-    <t>KB증권</t>
-  </si>
-  <si>
     <t>신영증권,유진증권</t>
-  </si>
-  <si>
-    <t>신영증권,KB증권</t>
   </si>
 </sst>
 </file>
@@ -966,7 +942,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Y15"/>
+  <dimension ref="A1:Y14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:25">
@@ -1051,16 +1027,16 @@
         <v>25</v>
       </c>
       <c r="B2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="F2">
         <v>7950000</v>
@@ -1087,10 +1063,10 @@
         <v>2000</v>
       </c>
       <c r="N2" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="O2" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="P2">
         <v>0</v>
@@ -1120,7 +1096,7 @@
         <v>0</v>
       </c>
       <c r="Y2" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
     </row>
     <row r="3" spans="1:25">
@@ -1128,16 +1104,16 @@
         <v>26</v>
       </c>
       <c r="B3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C3" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E3" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="F3">
         <v>1566800</v>
@@ -1164,10 +1140,10 @@
         <v>15300</v>
       </c>
       <c r="N3" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="O3" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="P3">
         <v>7367362</v>
@@ -1197,7 +1173,7 @@
         <v>-2903334</v>
       </c>
       <c r="Y3" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="4" spans="1:25">
@@ -1205,16 +1181,16 @@
         <v>27</v>
       </c>
       <c r="B4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D4" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E4" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F4">
         <v>1000000</v>
@@ -1241,10 +1217,10 @@
         <v>13000</v>
       </c>
       <c r="N4" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="O4" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="P4">
         <v>25588</v>
@@ -1274,7 +1250,7 @@
         <v>809</v>
       </c>
       <c r="Y4" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
     </row>
     <row r="5" spans="1:25">
@@ -1282,16 +1258,16 @@
         <v>28</v>
       </c>
       <c r="B5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C5" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="D5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="E5" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="F5">
         <v>6500000</v>
@@ -1318,10 +1294,10 @@
         <v>2000</v>
       </c>
       <c r="N5" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="O5" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="P5">
         <v>0</v>
@@ -1351,7 +1327,7 @@
         <v>0</v>
       </c>
       <c r="Y5" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
     </row>
     <row r="6" spans="1:25">
@@ -1362,13 +1338,13 @@
         <v>28</v>
       </c>
       <c r="C6" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D6" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E6" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="F6">
         <v>1400000</v>
@@ -1395,10 +1371,10 @@
         <v>15500</v>
       </c>
       <c r="N6" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="O6" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="P6">
         <v>10740898602</v>
@@ -1428,7 +1404,7 @@
         <v>219774608</v>
       </c>
       <c r="Y6" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
     </row>
     <row r="7" spans="1:25">
@@ -1439,13 +1415,13 @@
         <v>26</v>
       </c>
       <c r="C7" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D7" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E7" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="F7">
         <v>1000000</v>
@@ -1472,10 +1448,10 @@
         <v>29000</v>
       </c>
       <c r="N7" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="O7" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="P7">
         <v>0</v>
@@ -1505,7 +1481,7 @@
         <v>0</v>
       </c>
       <c r="Y7" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
     </row>
     <row r="8" spans="1:25">
@@ -1516,13 +1492,13 @@
         <v>26</v>
       </c>
       <c r="C8" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="D8" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E8" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F8">
         <v>751000</v>
@@ -1549,10 +1525,10 @@
         <v>21000</v>
       </c>
       <c r="N8" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="O8" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="P8">
         <v>0</v>
@@ -1582,7 +1558,7 @@
         <v>0</v>
       </c>
       <c r="Y8" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9" spans="1:25">
@@ -1593,13 +1569,13 @@
         <v>29</v>
       </c>
       <c r="C9" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D9" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E9" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="F9">
         <v>5800000</v>
@@ -1626,10 +1602,10 @@
         <v>2000</v>
       </c>
       <c r="N9" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="O9" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="P9">
         <v>0</v>
@@ -1659,7 +1635,7 @@
         <v>0</v>
       </c>
       <c r="Y9" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
     </row>
     <row r="10" spans="1:25">
@@ -1670,13 +1646,13 @@
         <v>30</v>
       </c>
       <c r="C10" t="s">
+        <v>48</v>
+      </c>
+      <c r="D10" t="s">
         <v>50</v>
       </c>
-      <c r="D10" t="s">
-        <v>52</v>
-      </c>
       <c r="E10" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="F10">
         <v>1400000</v>
@@ -1703,10 +1679,10 @@
         <v>16000</v>
       </c>
       <c r="N10" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="O10" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="P10">
         <v>72895458363</v>
@@ -1736,7 +1712,7 @@
         <v>-3801868433</v>
       </c>
       <c r="Y10" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
     </row>
     <row r="11" spans="1:25">
@@ -1744,16 +1720,16 @@
         <v>32</v>
       </c>
       <c r="B11" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C11" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D11" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E11" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F11">
         <v>2234000</v>
@@ -1780,10 +1756,10 @@
         <v>10000</v>
       </c>
       <c r="N11" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="O11" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="P11">
         <v>1337894447</v>
@@ -1813,7 +1789,7 @@
         <v>-1257080998</v>
       </c>
       <c r="Y11" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
     </row>
     <row r="12" spans="1:25">
@@ -1821,16 +1797,16 @@
         <v>33</v>
       </c>
       <c r="B12" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C12" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D12" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E12" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F12">
         <v>1350000</v>
@@ -1857,10 +1833,10 @@
         <v>22000</v>
       </c>
       <c r="N12" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="O12" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="P12">
         <v>5214628820</v>
@@ -1890,7 +1866,7 @@
         <v>24178632</v>
       </c>
       <c r="Y12" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
     </row>
     <row r="13" spans="1:25">
@@ -1898,16 +1874,16 @@
         <v>34</v>
       </c>
       <c r="B13" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C13" t="s">
+        <v>49</v>
+      </c>
+      <c r="D13" t="s">
         <v>51</v>
       </c>
-      <c r="D13" t="s">
-        <v>53</v>
-      </c>
       <c r="E13" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="F13">
         <v>6000000</v>
@@ -1934,10 +1910,10 @@
         <v>2000</v>
       </c>
       <c r="N13" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="O13" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="P13">
         <v>0</v>
@@ -1967,7 +1943,7 @@
         <v>0</v>
       </c>
       <c r="Y13" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
     </row>
     <row r="14" spans="1:25">
@@ -1975,16 +1951,16 @@
         <v>34</v>
       </c>
       <c r="B14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C14" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D14" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E14" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="F14">
         <v>4000000</v>
@@ -2011,10 +1987,10 @@
         <v>2000</v>
       </c>
       <c r="N14" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="O14" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="P14">
         <v>0</v>
@@ -2044,84 +2020,7 @@
         <v>0</v>
       </c>
       <c r="Y14" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="15" spans="1:25">
-      <c r="A15" t="s">
-        <v>35</v>
-      </c>
-      <c r="B15" t="s">
-        <v>42</v>
-      </c>
-      <c r="C15" t="s">
-        <v>32</v>
-      </c>
-      <c r="D15" t="s">
-        <v>55</v>
-      </c>
-      <c r="E15" t="s">
-        <v>74</v>
-      </c>
-      <c r="F15">
-        <v>1618000</v>
-      </c>
-      <c r="G15">
-        <v>1618000</v>
-      </c>
-      <c r="H15">
-        <v>0</v>
-      </c>
-      <c r="I15">
-        <v>6200</v>
-      </c>
-      <c r="J15">
-        <v>7700</v>
-      </c>
-      <c r="K15">
-        <v>10830212</v>
-      </c>
-      <c r="L15">
-        <v>0</v>
-      </c>
-      <c r="M15">
-        <v>10000</v>
-      </c>
-      <c r="N15" t="s">
-        <v>88</v>
-      </c>
-      <c r="O15" t="s">
-        <v>98</v>
-      </c>
-      <c r="P15">
-        <v>0</v>
-      </c>
-      <c r="Q15">
-        <v>0</v>
-      </c>
-      <c r="R15">
-        <v>0</v>
-      </c>
-      <c r="S15">
-        <v>0</v>
-      </c>
-      <c r="T15">
-        <v>0</v>
-      </c>
-      <c r="U15">
-        <v>0</v>
-      </c>
-      <c r="V15">
-        <v>0</v>
-      </c>
-      <c r="W15">
-        <v>0</v>
-      </c>
-      <c r="X15">
-        <v>0</v>
-      </c>
-      <c r="Y15" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
     </row>
   </sheetData>
@@ -2136,422 +2035,422 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="B2" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="C2" t="s">
-        <v>154</v>
+        <v>146</v>
       </c>
       <c r="D2" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="E2" t="s">
-        <v>175</v>
+        <v>165</v>
       </c>
       <c r="F2" t="s">
-        <v>187</v>
+        <v>178</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="B3" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="C3" t="s">
-        <v>155</v>
+        <v>147</v>
       </c>
       <c r="D3" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="E3" t="s">
-        <v>176</v>
+        <v>166</v>
       </c>
       <c r="F3" t="s">
-        <v>188</v>
+        <v>179</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="B4" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="C4" t="s">
-        <v>156</v>
+        <v>148</v>
       </c>
       <c r="D4" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="E4" t="s">
-        <v>89</v>
+        <v>167</v>
       </c>
       <c r="F4" t="s">
-        <v>189</v>
+        <v>180</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="B5" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="C5" t="s">
-        <v>157</v>
+        <v>149</v>
       </c>
       <c r="D5" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="E5" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="F5" t="s">
-        <v>190</v>
+        <v>181</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="B6" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="C6" t="s">
-        <v>158</v>
+        <v>150</v>
       </c>
       <c r="D6" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="E6" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="F6" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="B7" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="C7" t="s">
-        <v>159</v>
+        <v>151</v>
       </c>
       <c r="D7" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="E7" t="s">
-        <v>178</v>
+        <v>85</v>
       </c>
       <c r="F7" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="B8" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="C8" t="s">
-        <v>160</v>
+        <v>152</v>
       </c>
       <c r="D8" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="E8" t="s">
-        <v>179</v>
+        <v>169</v>
       </c>
       <c r="F8" t="s">
-        <v>193</v>
+        <v>184</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="B9" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="C9" t="s">
-        <v>161</v>
+        <v>153</v>
       </c>
       <c r="D9" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="E9" t="s">
-        <v>89</v>
+        <v>170</v>
       </c>
       <c r="F9" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="B10" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="C10" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="D10" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="E10" t="s">
-        <v>180</v>
+        <v>85</v>
       </c>
       <c r="F10" t="s">
-        <v>194</v>
+        <v>181</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="B11" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="C11" t="s">
-        <v>163</v>
+        <v>155</v>
       </c>
       <c r="D11" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="E11" t="s">
-        <v>181</v>
+        <v>171</v>
       </c>
       <c r="F11" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="B12" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="C12" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
       <c r="D12" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="E12" t="s">
-        <v>182</v>
+        <v>172</v>
       </c>
       <c r="F12" t="s">
-        <v>195</v>
+        <v>187</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="B13" t="s">
-        <v>147</v>
+        <v>138</v>
       </c>
       <c r="C13" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="D13" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="E13" t="s">
-        <v>89</v>
+        <v>173</v>
       </c>
       <c r="F13" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="B14" t="s">
-        <v>147</v>
+        <v>139</v>
       </c>
       <c r="C14" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="D14" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="E14" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="F14" t="s">
-        <v>195</v>
+        <v>184</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="B15" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="C15" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
       <c r="D15" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="E15" t="s">
-        <v>183</v>
+        <v>174</v>
       </c>
       <c r="F15" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="B16" t="s">
+        <v>141</v>
+      </c>
+      <c r="C16" t="s">
         <v>148</v>
       </c>
-      <c r="C16" t="s">
-        <v>168</v>
-      </c>
       <c r="D16" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="E16" t="s">
-        <v>89</v>
+        <v>175</v>
       </c>
       <c r="F16" t="s">
-        <v>196</v>
+        <v>178</v>
       </c>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="B17" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="C17" t="s">
-        <v>169</v>
+        <v>160</v>
       </c>
       <c r="D17" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="E17" t="s">
-        <v>89</v>
+        <v>176</v>
       </c>
       <c r="F17" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="B18" t="s">
-        <v>150</v>
+        <v>143</v>
       </c>
       <c r="C18" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="D18" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="E18" t="s">
-        <v>184</v>
+        <v>85</v>
       </c>
       <c r="F18" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="B19" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="C19" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D19" t="s">
-        <v>173</v>
+        <v>85</v>
       </c>
       <c r="E19" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="F19" t="s">
-        <v>195</v>
+        <v>184</v>
       </c>
     </row>
     <row r="20" spans="1:6">
       <c r="A20" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="B20" t="s">
-        <v>152</v>
+        <v>144</v>
       </c>
       <c r="C20" t="s">
-        <v>171</v>
+        <v>163</v>
       </c>
       <c r="D20" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="E20" t="s">
-        <v>185</v>
+        <v>85</v>
       </c>
       <c r="F20" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="B21" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="C21" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="D21" t="s">
-        <v>174</v>
+        <v>85</v>
       </c>
       <c r="E21" t="s">
-        <v>186</v>
+        <v>85</v>
       </c>
       <c r="F21" t="s">
-        <v>191</v>
+        <v>181</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
RPA datasets push 2024-09-16
</commit_message>
<xml_diff>
--- a/datasets/ib-strategy-data.xlsx
+++ b/datasets/ib-strategy-data.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="190">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="184">
   <si>
     <t>수요예측(시작일)</t>
   </si>
@@ -116,9 +116,6 @@
     <t>2024-07-15</t>
   </si>
   <si>
-    <t>2024-07-11</t>
-  </si>
-  <si>
     <t>2024-07-09</t>
   </si>
   <si>
@@ -134,9 +131,6 @@
     <t>2024-07-19</t>
   </si>
   <si>
-    <t>2024-07-17</t>
-  </si>
-  <si>
     <t>2024-07-10</t>
   </si>
   <si>
@@ -224,9 +218,6 @@
     <t>아이빔테크놀로지</t>
   </si>
   <si>
-    <t>피앤에스미캐닉스</t>
-  </si>
-  <si>
     <t>엔에이치스팩31호</t>
   </si>
   <si>
@@ -263,9 +254,6 @@
     <t>1011.50:1</t>
   </si>
   <si>
-    <t>986.08:1</t>
-  </si>
-  <si>
     <t>1123.43 :1</t>
   </si>
   <si>
@@ -296,9 +284,6 @@
     <t>0.49%</t>
   </si>
   <si>
-    <t>5.60%</t>
-  </si>
-  <si>
     <t>기업인수합병</t>
   </si>
   <si>
@@ -324,9 +309,6 @@
   </si>
   <si>
     <t>생체현미경, CRO 서비스</t>
-  </si>
-  <si>
-    <t>보행재활로봇 시스템</t>
   </si>
   <si>
     <t>금융지원서비스업</t>
@@ -942,7 +924,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Y14"/>
+  <dimension ref="A1:Y13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:25">
@@ -1027,16 +1009,16 @@
         <v>25</v>
       </c>
       <c r="B2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C2" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="D2" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F2">
         <v>7950000</v>
@@ -1063,10 +1045,10 @@
         <v>2000</v>
       </c>
       <c r="N2" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="O2" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="P2">
         <v>0</v>
@@ -1096,7 +1078,7 @@
         <v>0</v>
       </c>
       <c r="Y2" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
     </row>
     <row r="3" spans="1:25">
@@ -1104,16 +1086,16 @@
         <v>26</v>
       </c>
       <c r="B3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C3" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E3" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="F3">
         <v>1566800</v>
@@ -1140,10 +1122,10 @@
         <v>15300</v>
       </c>
       <c r="N3" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="O3" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="P3">
         <v>7367362</v>
@@ -1173,7 +1155,7 @@
         <v>-2903334</v>
       </c>
       <c r="Y3" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
     </row>
     <row r="4" spans="1:25">
@@ -1181,16 +1163,16 @@
         <v>27</v>
       </c>
       <c r="B4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C4" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E4" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="F4">
         <v>1000000</v>
@@ -1217,10 +1199,10 @@
         <v>13000</v>
       </c>
       <c r="N4" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="O4" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="P4">
         <v>25588</v>
@@ -1250,7 +1232,7 @@
         <v>809</v>
       </c>
       <c r="Y4" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
     </row>
     <row r="5" spans="1:25">
@@ -1258,16 +1240,16 @@
         <v>28</v>
       </c>
       <c r="B5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C5" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D5" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E5" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="F5">
         <v>6500000</v>
@@ -1294,10 +1276,10 @@
         <v>2000</v>
       </c>
       <c r="N5" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="O5" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="P5">
         <v>0</v>
@@ -1327,7 +1309,7 @@
         <v>0</v>
       </c>
       <c r="Y5" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
     </row>
     <row r="6" spans="1:25">
@@ -1338,13 +1320,13 @@
         <v>28</v>
       </c>
       <c r="C6" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D6" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E6" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F6">
         <v>1400000</v>
@@ -1371,10 +1353,10 @@
         <v>15500</v>
       </c>
       <c r="N6" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="O6" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="P6">
         <v>10740898602</v>
@@ -1404,7 +1386,7 @@
         <v>219774608</v>
       </c>
       <c r="Y6" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
     </row>
     <row r="7" spans="1:25">
@@ -1415,13 +1397,13 @@
         <v>26</v>
       </c>
       <c r="C7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D7" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E7" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="F7">
         <v>1000000</v>
@@ -1448,10 +1430,10 @@
         <v>29000</v>
       </c>
       <c r="N7" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="O7" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="P7">
         <v>0</v>
@@ -1481,7 +1463,7 @@
         <v>0</v>
       </c>
       <c r="Y7" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
     </row>
     <row r="8" spans="1:25">
@@ -1492,13 +1474,13 @@
         <v>26</v>
       </c>
       <c r="C8" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="D8" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="E8" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="F8">
         <v>751000</v>
@@ -1525,10 +1507,10 @@
         <v>21000</v>
       </c>
       <c r="N8" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="O8" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="P8">
         <v>0</v>
@@ -1558,7 +1540,7 @@
         <v>0</v>
       </c>
       <c r="Y8" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="9" spans="1:25">
@@ -1569,13 +1551,13 @@
         <v>29</v>
       </c>
       <c r="C9" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D9" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E9" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="F9">
         <v>5800000</v>
@@ -1602,10 +1584,10 @@
         <v>2000</v>
       </c>
       <c r="N9" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="O9" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="P9">
         <v>0</v>
@@ -1635,7 +1617,7 @@
         <v>0</v>
       </c>
       <c r="Y9" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
     </row>
     <row r="10" spans="1:25">
@@ -1646,13 +1628,13 @@
         <v>30</v>
       </c>
       <c r="C10" t="s">
+        <v>46</v>
+      </c>
+      <c r="D10" t="s">
         <v>48</v>
       </c>
-      <c r="D10" t="s">
-        <v>50</v>
-      </c>
       <c r="E10" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F10">
         <v>1400000</v>
@@ -1679,10 +1661,10 @@
         <v>16000</v>
       </c>
       <c r="N10" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="O10" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="P10">
         <v>72895458363</v>
@@ -1712,7 +1694,7 @@
         <v>-3801868433</v>
       </c>
       <c r="Y10" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
     </row>
     <row r="11" spans="1:25">
@@ -1720,16 +1702,16 @@
         <v>32</v>
       </c>
       <c r="B11" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D11" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E11" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="F11">
         <v>2234000</v>
@@ -1756,10 +1738,10 @@
         <v>10000</v>
       </c>
       <c r="N11" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="O11" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="P11">
         <v>1337894447</v>
@@ -1789,7 +1771,7 @@
         <v>-1257080998</v>
       </c>
       <c r="Y11" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
     </row>
     <row r="12" spans="1:25">
@@ -1797,99 +1779,99 @@
         <v>33</v>
       </c>
       <c r="B12" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C12" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="D12" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="E12" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="F12">
-        <v>1350000</v>
+        <v>6000000</v>
       </c>
       <c r="G12">
-        <v>1350000</v>
+        <v>6000000</v>
       </c>
       <c r="H12">
         <v>0</v>
       </c>
       <c r="I12">
-        <v>14000</v>
+        <v>2000</v>
       </c>
       <c r="J12">
-        <v>17000</v>
+        <v>2000</v>
       </c>
       <c r="K12">
-        <v>6471740</v>
+        <v>6345000</v>
       </c>
       <c r="L12">
         <v>0</v>
       </c>
       <c r="M12">
-        <v>22000</v>
+        <v>2000</v>
       </c>
       <c r="N12" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="O12" t="s">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="P12">
-        <v>5214628820</v>
+        <v>0</v>
       </c>
       <c r="Q12">
-        <v>6009352447</v>
+        <v>0</v>
       </c>
       <c r="R12">
-        <v>965797975</v>
+        <v>0</v>
       </c>
       <c r="S12">
-        <v>2015081728</v>
+        <v>0</v>
       </c>
       <c r="T12">
-        <v>1319755337</v>
+        <v>0</v>
       </c>
       <c r="U12">
-        <v>-44547594</v>
+        <v>0</v>
       </c>
       <c r="V12">
-        <v>1503069100</v>
+        <v>0</v>
       </c>
       <c r="W12">
-        <v>1410469786</v>
+        <v>0</v>
       </c>
       <c r="X12">
-        <v>24178632</v>
+        <v>0</v>
       </c>
       <c r="Y12" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
     </row>
     <row r="13" spans="1:25">
       <c r="A13" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B13" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C13" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D13" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="E13" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F13">
-        <v>6000000</v>
+        <v>4000000</v>
       </c>
       <c r="G13">
-        <v>6000000</v>
+        <v>4000000</v>
       </c>
       <c r="H13">
         <v>0</v>
@@ -1901,7 +1883,7 @@
         <v>2000</v>
       </c>
       <c r="K13">
-        <v>6345000</v>
+        <v>4420000</v>
       </c>
       <c r="L13">
         <v>0</v>
@@ -1910,10 +1892,10 @@
         <v>2000</v>
       </c>
       <c r="N13" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="O13" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="P13">
         <v>0</v>
@@ -1943,84 +1925,7 @@
         <v>0</v>
       </c>
       <c r="Y13" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="14" spans="1:25">
-      <c r="A14" t="s">
-        <v>34</v>
-      </c>
-      <c r="B14" t="s">
-        <v>40</v>
-      </c>
-      <c r="C14" t="s">
-        <v>48</v>
-      </c>
-      <c r="D14" t="s">
-        <v>58</v>
-      </c>
-      <c r="E14" t="s">
-        <v>71</v>
-      </c>
-      <c r="F14">
-        <v>4000000</v>
-      </c>
-      <c r="G14">
-        <v>4000000</v>
-      </c>
-      <c r="H14">
-        <v>0</v>
-      </c>
-      <c r="I14">
-        <v>2000</v>
-      </c>
-      <c r="J14">
-        <v>2000</v>
-      </c>
-      <c r="K14">
-        <v>4420000</v>
-      </c>
-      <c r="L14">
-        <v>0</v>
-      </c>
-      <c r="M14">
-        <v>2000</v>
-      </c>
-      <c r="N14" t="s">
-        <v>84</v>
-      </c>
-      <c r="O14" t="s">
-        <v>85</v>
-      </c>
-      <c r="P14">
-        <v>0</v>
-      </c>
-      <c r="Q14">
-        <v>0</v>
-      </c>
-      <c r="R14">
-        <v>0</v>
-      </c>
-      <c r="S14">
-        <v>0</v>
-      </c>
-      <c r="T14">
-        <v>0</v>
-      </c>
-      <c r="U14">
-        <v>0</v>
-      </c>
-      <c r="V14">
-        <v>0</v>
-      </c>
-      <c r="W14">
-        <v>0</v>
-      </c>
-      <c r="X14">
-        <v>0</v>
-      </c>
-      <c r="Y14" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
     </row>
   </sheetData>
@@ -2035,422 +1940,422 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="B2" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="C2" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="D2" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="E2" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="F2" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="B3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="C3" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="D3" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="E3" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="F3" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="B4" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="C4" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="D4" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="E4" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="F4" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="B5" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="C5" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="D5" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="E5" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="F5" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="B6" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="C6" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="D6" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="E6" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="F6" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="B7" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="C7" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="D7" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="E7" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="F7" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="B8" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="C8" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="D8" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="E8" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="F8" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="B9" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="C9" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="D9" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="E9" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="F9" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="B10" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="C10" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="D10" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="E10" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="F10" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="B11" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="C11" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="D11" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="E11" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="F11" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="B12" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="C12" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="D12" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="E12" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="F12" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="B13" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="C13" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="D13" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="E13" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="F13" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="B14" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="C14" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="D14" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="E14" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="F14" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="B15" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="C15" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="D15" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="E15" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="F15" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="B16" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="C16" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="D16" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="E16" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="F16" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="B17" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="C17" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="D17" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="E17" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="F17" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="B18" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="C18" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="D18" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="E18" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="F18" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="B19" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="C19" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="D19" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="E19" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="F19" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
     </row>
     <row r="20" spans="1:6">
       <c r="A20" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="B20" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="C20" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="D20" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="E20" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="F20" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="B21" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="C21" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="D21" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="E21" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="F21" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
RPA datasets push 2024-09-20
</commit_message>
<xml_diff>
--- a/datasets/ib-strategy-data.xlsx
+++ b/datasets/ib-strategy-data.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="181">
   <si>
     <t>수요예측(시작일)</t>
   </si>
@@ -326,6 +326,9 @@
     <t>위츠</t>
   </si>
   <si>
+    <t>동방메디컬</t>
+  </si>
+  <si>
     <t>더본코리아(유가)</t>
   </si>
   <si>
@@ -380,12 +383,12 @@
     <t>한켐</t>
   </si>
   <si>
-    <t>토모큐브</t>
-  </si>
-  <si>
     <t>2024.10.28~11.01</t>
   </si>
   <si>
+    <t>2024.10.16~10.22</t>
+  </si>
+  <si>
     <t>2024.10.15~10.21</t>
   </si>
   <si>
@@ -422,12 +425,12 @@
     <t>2024.09.23~09.27</t>
   </si>
   <si>
-    <t>2024.09.20~09.26</t>
-  </si>
-  <si>
     <t>5,300~6,400</t>
   </si>
   <si>
+    <t>9,000~10,500</t>
+  </si>
+  <si>
     <t>23,000~28,000</t>
   </si>
   <si>
@@ -479,12 +482,12 @@
     <t>12,500~14,500</t>
   </si>
   <si>
-    <t>10,900~13,400</t>
-  </si>
-  <si>
     <t>15900</t>
   </si>
   <si>
+    <t>30609</t>
+  </si>
+  <si>
     <t>69000</t>
   </si>
   <si>
@@ -524,6 +527,9 @@
     <t>신한투자증권</t>
   </si>
   <si>
+    <t>NH투자증권</t>
+  </si>
+  <si>
     <t>한국투자증권,NH투자증권</t>
   </si>
   <si>
@@ -549,9 +555,6 @@
   </si>
   <si>
     <t>삼성증권,유진투자증권,유안타증권</t>
-  </si>
-  <si>
-    <t>NH투자증권</t>
   </si>
   <si>
     <t>신영증권,유진증권</t>
@@ -1886,7 +1889,7 @@
         <v>155</v>
       </c>
       <c r="F2" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -1906,7 +1909,7 @@
         <v>156</v>
       </c>
       <c r="F3" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -1926,7 +1929,7 @@
         <v>157</v>
       </c>
       <c r="F4" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -1946,7 +1949,7 @@
         <v>158</v>
       </c>
       <c r="F5" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -1963,10 +1966,10 @@
         <v>79</v>
       </c>
       <c r="E6" t="s">
-        <v>79</v>
+        <v>159</v>
       </c>
       <c r="F6" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -1974,7 +1977,7 @@
         <v>107</v>
       </c>
       <c r="B7" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C7" t="s">
         <v>141</v>
@@ -1986,7 +1989,7 @@
         <v>79</v>
       </c>
       <c r="F7" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -1994,7 +1997,7 @@
         <v>108</v>
       </c>
       <c r="B8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C8" t="s">
         <v>142</v>
@@ -2003,10 +2006,10 @@
         <v>79</v>
       </c>
       <c r="E8" t="s">
-        <v>159</v>
+        <v>79</v>
       </c>
       <c r="F8" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -2014,7 +2017,7 @@
         <v>109</v>
       </c>
       <c r="B9" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C9" t="s">
         <v>143</v>
@@ -2026,7 +2029,7 @@
         <v>160</v>
       </c>
       <c r="F9" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -2043,10 +2046,10 @@
         <v>79</v>
       </c>
       <c r="E10" t="s">
-        <v>79</v>
+        <v>161</v>
       </c>
       <c r="F10" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -2054,7 +2057,7 @@
         <v>111</v>
       </c>
       <c r="B11" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C11" t="s">
         <v>145</v>
@@ -2063,10 +2066,10 @@
         <v>79</v>
       </c>
       <c r="E11" t="s">
-        <v>161</v>
+        <v>79</v>
       </c>
       <c r="F11" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -2086,7 +2089,7 @@
         <v>162</v>
       </c>
       <c r="F12" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -2094,7 +2097,7 @@
         <v>113</v>
       </c>
       <c r="B13" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C13" t="s">
         <v>147</v>
@@ -2106,7 +2109,7 @@
         <v>163</v>
       </c>
       <c r="F13" t="s">
-        <v>172</v>
+        <v>179</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -2123,7 +2126,7 @@
         <v>79</v>
       </c>
       <c r="E14" t="s">
-        <v>79</v>
+        <v>164</v>
       </c>
       <c r="F14" t="s">
         <v>174</v>
@@ -2143,10 +2146,10 @@
         <v>79</v>
       </c>
       <c r="E15" t="s">
-        <v>164</v>
+        <v>79</v>
       </c>
       <c r="F15" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -2157,7 +2160,7 @@
         <v>131</v>
       </c>
       <c r="C16" t="s">
-        <v>138</v>
+        <v>150</v>
       </c>
       <c r="D16" t="s">
         <v>79</v>
@@ -2166,7 +2169,7 @@
         <v>165</v>
       </c>
       <c r="F16" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -2177,7 +2180,7 @@
         <v>132</v>
       </c>
       <c r="C17" t="s">
-        <v>150</v>
+        <v>139</v>
       </c>
       <c r="D17" t="s">
         <v>79</v>
@@ -2186,7 +2189,7 @@
         <v>166</v>
       </c>
       <c r="F17" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
     </row>
     <row r="18" spans="1:6">
@@ -2203,10 +2206,10 @@
         <v>79</v>
       </c>
       <c r="E18" t="s">
-        <v>79</v>
+        <v>167</v>
       </c>
       <c r="F18" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
     </row>
     <row r="19" spans="1:6">
@@ -2223,10 +2226,10 @@
         <v>79</v>
       </c>
       <c r="E19" t="s">
-        <v>167</v>
+        <v>79</v>
       </c>
       <c r="F19" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -2234,7 +2237,7 @@
         <v>120</v>
       </c>
       <c r="B20" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C20" t="s">
         <v>153</v>
@@ -2243,10 +2246,10 @@
         <v>79</v>
       </c>
       <c r="E20" t="s">
-        <v>79</v>
+        <v>168</v>
       </c>
       <c r="F20" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -2266,7 +2269,7 @@
         <v>79</v>
       </c>
       <c r="F21" t="s">
-        <v>171</v>
+        <v>180</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
RPA datasets push 2024-09-21
</commit_message>
<xml_diff>
--- a/datasets/ib-strategy-data.xlsx
+++ b/datasets/ib-strategy-data.xlsx
@@ -326,6 +326,9 @@
     <t>위츠</t>
   </si>
   <si>
+    <t>엠오티</t>
+  </si>
+  <si>
     <t>동방메디컬</t>
   </si>
   <si>
@@ -335,15 +338,21 @@
     <t>유진스팩11호</t>
   </si>
   <si>
+    <t>에이치이엠파마(구.에이치이엠)</t>
+  </si>
+  <si>
+    <t>탑런토탈솔루션</t>
+  </si>
+  <si>
     <t>노머스</t>
   </si>
   <si>
+    <t>에이럭스</t>
+  </si>
+  <si>
     <t>닷밀</t>
   </si>
   <si>
-    <t>탑런토탈솔루션</t>
-  </si>
-  <si>
     <t>성우</t>
   </si>
   <si>
@@ -374,18 +383,12 @@
     <t>와이제이링크</t>
   </si>
   <si>
-    <t>셀비온</t>
-  </si>
-  <si>
-    <t>인스피언</t>
-  </si>
-  <si>
-    <t>한켐</t>
-  </si>
-  <si>
     <t>2024.10.28~11.01</t>
   </si>
   <si>
+    <t>2024.10.17~10.23</t>
+  </si>
+  <si>
     <t>2024.10.16~10.22</t>
   </si>
   <si>
@@ -395,6 +398,9 @@
     <t>2024.10.15~10.16</t>
   </si>
   <si>
+    <t>2024.10.14~10.18</t>
+  </si>
+  <si>
     <t>2024.10.11~10.17</t>
   </si>
   <si>
@@ -419,15 +425,12 @@
     <t>2024.09.25~10.02</t>
   </si>
   <si>
-    <t>2024.09.24~09.30</t>
-  </si>
-  <si>
-    <t>2024.09.23~09.27</t>
-  </si>
-  <si>
     <t>5,300~6,400</t>
   </si>
   <si>
+    <t>12,000~14,000</t>
+  </si>
+  <si>
     <t>9,000~10,500</t>
   </si>
   <si>
@@ -437,15 +440,18 @@
     <t>2,000~2,000</t>
   </si>
   <si>
+    <t>16,400~19,000</t>
+  </si>
+  <si>
     <t>27,200~30,200</t>
   </si>
   <si>
+    <t>11,500~13,500</t>
+  </si>
+  <si>
     <t>11,000~13,000</t>
   </si>
   <si>
-    <t>12,000~14,000</t>
-  </si>
-  <si>
     <t>25,000~29,000</t>
   </si>
   <si>
@@ -473,18 +479,12 @@
     <t>8,600~9,800</t>
   </si>
   <si>
-    <t>10,000~12,200</t>
-  </si>
-  <si>
-    <t>8,000~10,000</t>
-  </si>
-  <si>
-    <t>12,500~14,500</t>
-  </si>
-  <si>
     <t>15900</t>
   </si>
   <si>
+    <t>21000</t>
+  </si>
+  <si>
     <t>30609</t>
   </si>
   <si>
@@ -494,9 +494,15 @@
     <t>9000</t>
   </si>
   <si>
+    <t>11430</t>
+  </si>
+  <si>
     <t>30736</t>
   </si>
   <si>
+    <t>17250</t>
+  </si>
+  <si>
     <t>75000</t>
   </si>
   <si>
@@ -521,12 +527,12 @@
     <t>30616</t>
   </si>
   <si>
-    <t>18000</t>
-  </si>
-  <si>
     <t>신한투자증권</t>
   </si>
   <si>
+    <t>한국투자증권</t>
+  </si>
+  <si>
     <t>NH투자증권</t>
   </si>
   <si>
@@ -536,18 +542,15 @@
     <t>유진증권</t>
   </si>
   <si>
+    <t>KB증권</t>
+  </si>
+  <si>
     <t>대신증권</t>
   </si>
   <si>
     <t>미래에셋증권</t>
   </si>
   <si>
-    <t>KB증권</t>
-  </si>
-  <si>
-    <t>한국투자증권</t>
-  </si>
-  <si>
     <t>NH투자증권,KB증권,신한투자증권,키움증권</t>
   </si>
   <si>
@@ -555,9 +558,6 @@
   </si>
   <si>
     <t>삼성증권,유진투자증권,유안타증권</t>
-  </si>
-  <si>
-    <t>신영증권,유진증권</t>
   </si>
 </sst>
 </file>
@@ -1886,10 +1886,10 @@
         <v>79</v>
       </c>
       <c r="E2" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F2" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -1906,10 +1906,10 @@
         <v>79</v>
       </c>
       <c r="E3" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="F3" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -1926,10 +1926,10 @@
         <v>79</v>
       </c>
       <c r="E4" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="F4" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -1946,10 +1946,10 @@
         <v>79</v>
       </c>
       <c r="E5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="F5" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -1966,10 +1966,10 @@
         <v>79</v>
       </c>
       <c r="E6" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="F6" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -1986,10 +1986,10 @@
         <v>79</v>
       </c>
       <c r="E7" t="s">
-        <v>79</v>
+        <v>159</v>
       </c>
       <c r="F7" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -2000,7 +2000,7 @@
         <v>127</v>
       </c>
       <c r="C8" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="D8" t="s">
         <v>79</v>
@@ -2017,10 +2017,10 @@
         <v>109</v>
       </c>
       <c r="B9" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C9" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D9" t="s">
         <v>79</v>
@@ -2037,10 +2037,10 @@
         <v>110</v>
       </c>
       <c r="B10" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C10" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D10" t="s">
         <v>79</v>
@@ -2049,7 +2049,7 @@
         <v>161</v>
       </c>
       <c r="F10" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -2057,10 +2057,10 @@
         <v>111</v>
       </c>
       <c r="B11" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C11" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D11" t="s">
         <v>79</v>
@@ -2069,7 +2069,7 @@
         <v>79</v>
       </c>
       <c r="F11" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -2077,10 +2077,10 @@
         <v>112</v>
       </c>
       <c r="B12" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C12" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D12" t="s">
         <v>79</v>
@@ -2089,7 +2089,7 @@
         <v>162</v>
       </c>
       <c r="F12" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -2100,7 +2100,7 @@
         <v>129</v>
       </c>
       <c r="C13" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D13" t="s">
         <v>79</v>
@@ -2109,7 +2109,7 @@
         <v>163</v>
       </c>
       <c r="F13" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -2117,19 +2117,19 @@
         <v>114</v>
       </c>
       <c r="B14" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C14" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D14" t="s">
         <v>79</v>
       </c>
       <c r="E14" t="s">
-        <v>164</v>
+        <v>79</v>
       </c>
       <c r="F14" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -2140,16 +2140,16 @@
         <v>130</v>
       </c>
       <c r="C15" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D15" t="s">
         <v>79</v>
       </c>
       <c r="E15" t="s">
-        <v>79</v>
+        <v>164</v>
       </c>
       <c r="F15" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -2160,7 +2160,7 @@
         <v>131</v>
       </c>
       <c r="C16" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D16" t="s">
         <v>79</v>
@@ -2169,7 +2169,7 @@
         <v>165</v>
       </c>
       <c r="F16" t="s">
-        <v>170</v>
+        <v>180</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -2177,10 +2177,10 @@
         <v>117</v>
       </c>
       <c r="B17" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C17" t="s">
-        <v>139</v>
+        <v>150</v>
       </c>
       <c r="D17" t="s">
         <v>79</v>
@@ -2189,7 +2189,7 @@
         <v>166</v>
       </c>
       <c r="F17" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
     </row>
     <row r="18" spans="1:6">
@@ -2197,7 +2197,7 @@
         <v>118</v>
       </c>
       <c r="B18" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C18" t="s">
         <v>151</v>
@@ -2206,10 +2206,10 @@
         <v>79</v>
       </c>
       <c r="E18" t="s">
-        <v>167</v>
+        <v>79</v>
       </c>
       <c r="F18" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
     </row>
     <row r="19" spans="1:6">
@@ -2217,7 +2217,7 @@
         <v>119</v>
       </c>
       <c r="B19" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C19" t="s">
         <v>152</v>
@@ -2226,10 +2226,10 @@
         <v>79</v>
       </c>
       <c r="E19" t="s">
-        <v>79</v>
+        <v>167</v>
       </c>
       <c r="F19" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -2237,10 +2237,10 @@
         <v>120</v>
       </c>
       <c r="B20" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C20" t="s">
-        <v>153</v>
+        <v>140</v>
       </c>
       <c r="D20" t="s">
         <v>79</v>
@@ -2249,7 +2249,7 @@
         <v>168</v>
       </c>
       <c r="F20" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -2260,16 +2260,16 @@
         <v>135</v>
       </c>
       <c r="C21" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D21" t="s">
         <v>79</v>
       </c>
       <c r="E21" t="s">
-        <v>79</v>
+        <v>169</v>
       </c>
       <c r="F21" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
RPA datasets push 2024-09-23
</commit_message>
<xml_diff>
--- a/datasets/ib-strategy-data.xlsx
+++ b/datasets/ib-strategy-data.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="185">
   <si>
     <t>수요예측(시작일)</t>
   </si>
@@ -92,6 +92,9 @@
     <t>주요제품</t>
   </si>
   <si>
+    <t>2024-07-29</t>
+  </si>
+  <si>
     <t>2024-08-26</t>
   </si>
   <si>
@@ -107,9 +110,6 @@
     <t>2024-07-30</t>
   </si>
   <si>
-    <t>2024-07-29</t>
-  </si>
-  <si>
     <t>2024-07-23</t>
   </si>
   <si>
@@ -134,6 +134,9 @@
     <t>2024-07-10</t>
   </si>
   <si>
+    <t>2024-08-16</t>
+  </si>
+  <si>
     <t>2024-09-11</t>
   </si>
   <si>
@@ -149,9 +152,6 @@
     <t>2024-08-20</t>
   </si>
   <si>
-    <t>2024-08-16</t>
-  </si>
-  <si>
     <t>2024-08-13</t>
   </si>
   <si>
@@ -161,6 +161,9 @@
     <t>2024-07-26</t>
   </si>
   <si>
+    <t>대신</t>
+  </si>
+  <si>
     <t>미래</t>
   </si>
   <si>
@@ -170,9 +173,6 @@
     <t>한국</t>
   </si>
   <si>
-    <t>대신</t>
-  </si>
-  <si>
     <t>하나</t>
   </si>
   <si>
@@ -188,6 +188,9 @@
     <t>SK</t>
   </si>
   <si>
+    <t>아이언디바이스</t>
+  </si>
+  <si>
     <t>미래에셋비전스팩7호</t>
   </si>
   <si>
@@ -221,6 +224,9 @@
     <t>SK증권제13호스팩</t>
   </si>
   <si>
+    <t>1152.85:1</t>
+  </si>
+  <si>
     <t>1051.62 :1</t>
   </si>
   <si>
@@ -254,6 +260,9 @@
     <t>1197.45:1</t>
   </si>
   <si>
+    <t>3.34%</t>
+  </si>
+  <si>
     <t>-</t>
   </si>
   <si>
@@ -273,6 +282,9 @@
   </si>
   <si>
     <t>0.49%</t>
+  </si>
+  <si>
+    <t>스마트폰용 오디오 앰프 반도체 Soc</t>
   </si>
   <si>
     <t>기업인수합병</t>
@@ -915,7 +927,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Y12"/>
+  <dimension ref="A1:Y13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:25">
@@ -1000,7 +1012,7 @@
         <v>25</v>
       </c>
       <c r="B2" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="C2" t="s">
         <v>39</v>
@@ -1012,64 +1024,64 @@
         <v>57</v>
       </c>
       <c r="F2">
-        <v>7950000</v>
+        <v>3000000</v>
       </c>
       <c r="G2">
-        <v>7950000</v>
+        <v>3000000</v>
       </c>
       <c r="H2">
         <v>0</v>
       </c>
       <c r="I2">
-        <v>2000</v>
+        <v>4900</v>
       </c>
       <c r="J2">
-        <v>2000</v>
+        <v>5700</v>
       </c>
       <c r="K2">
-        <v>8215000</v>
+        <v>13653263</v>
       </c>
       <c r="L2">
         <v>0</v>
       </c>
       <c r="M2">
-        <v>2000</v>
+        <v>7000</v>
       </c>
       <c r="N2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="O2" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>5436813</v>
       </c>
       <c r="Q2">
-        <v>0</v>
+        <v>6232339</v>
       </c>
       <c r="R2">
-        <v>0</v>
+        <v>2471281</v>
       </c>
       <c r="S2">
-        <v>0</v>
+        <v>-1510039</v>
       </c>
       <c r="T2">
-        <v>0</v>
+        <v>-3517400</v>
       </c>
       <c r="U2">
-        <v>0</v>
+        <v>-1015682</v>
       </c>
       <c r="V2">
-        <v>0</v>
+        <v>-3268622</v>
       </c>
       <c r="W2">
-        <v>0</v>
+        <v>-3926782</v>
       </c>
       <c r="X2">
-        <v>0</v>
+        <v>-801640</v>
       </c>
       <c r="Y2" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
     </row>
     <row r="3" spans="1:25">
@@ -1077,7 +1089,7 @@
         <v>26</v>
       </c>
       <c r="B3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C3" t="s">
         <v>40</v>
@@ -1089,64 +1101,64 @@
         <v>58</v>
       </c>
       <c r="F3">
-        <v>1566800</v>
+        <v>7950000</v>
       </c>
       <c r="G3">
-        <v>1566800</v>
+        <v>7950000</v>
       </c>
       <c r="H3">
         <v>0</v>
       </c>
       <c r="I3">
-        <v>13600</v>
+        <v>2000</v>
       </c>
       <c r="J3">
-        <v>15300</v>
+        <v>2000</v>
       </c>
       <c r="K3">
-        <v>9349954</v>
+        <v>8215000</v>
       </c>
       <c r="L3">
         <v>0</v>
       </c>
       <c r="M3">
-        <v>15300</v>
+        <v>2000</v>
       </c>
       <c r="N3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="O3" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="P3">
-        <v>7367362</v>
+        <v>0</v>
       </c>
       <c r="Q3">
-        <v>10525887</v>
+        <v>0</v>
       </c>
       <c r="R3">
-        <v>1790340</v>
+        <v>0</v>
       </c>
       <c r="S3">
-        <v>-9315442</v>
+        <v>0</v>
       </c>
       <c r="T3">
-        <v>-11755057</v>
+        <v>0</v>
       </c>
       <c r="U3">
-        <v>-2929307</v>
+        <v>0</v>
       </c>
       <c r="V3">
-        <v>-45566953</v>
+        <v>0</v>
       </c>
       <c r="W3">
-        <v>-5053520</v>
+        <v>0</v>
       </c>
       <c r="X3">
-        <v>-2903334</v>
+        <v>0</v>
       </c>
       <c r="Y3" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
     </row>
     <row r="4" spans="1:25">
@@ -1154,7 +1166,7 @@
         <v>27</v>
       </c>
       <c r="B4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C4" t="s">
         <v>41</v>
@@ -1166,64 +1178,64 @@
         <v>59</v>
       </c>
       <c r="F4">
-        <v>1000000</v>
+        <v>1566800</v>
       </c>
       <c r="G4">
-        <v>500000</v>
+        <v>1566800</v>
       </c>
       <c r="H4">
-        <v>500000</v>
+        <v>0</v>
       </c>
       <c r="I4">
-        <v>9500</v>
+        <v>13600</v>
       </c>
       <c r="J4">
-        <v>10700</v>
+        <v>15300</v>
       </c>
       <c r="K4">
-        <v>5530000</v>
+        <v>9349954</v>
       </c>
       <c r="L4">
         <v>0</v>
       </c>
       <c r="M4">
-        <v>13000</v>
+        <v>15300</v>
       </c>
       <c r="N4" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="O4" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="P4">
-        <v>25588</v>
+        <v>7367362</v>
       </c>
       <c r="Q4">
-        <v>30049</v>
+        <v>10525887</v>
       </c>
       <c r="R4">
-        <v>7363</v>
+        <v>1790340</v>
       </c>
       <c r="S4">
-        <v>3780</v>
+        <v>-9315442</v>
       </c>
       <c r="T4">
-        <v>5016</v>
+        <v>-11755057</v>
       </c>
       <c r="U4">
-        <v>938</v>
+        <v>-2929307</v>
       </c>
       <c r="V4">
-        <v>3456</v>
+        <v>-45566953</v>
       </c>
       <c r="W4">
-        <v>4688</v>
+        <v>-5053520</v>
       </c>
       <c r="X4">
-        <v>809</v>
+        <v>-2903334</v>
       </c>
       <c r="Y4" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
     </row>
     <row r="5" spans="1:25">
@@ -1243,64 +1255,64 @@
         <v>60</v>
       </c>
       <c r="F5">
-        <v>6500000</v>
+        <v>1000000</v>
       </c>
       <c r="G5">
-        <v>6500000</v>
+        <v>500000</v>
       </c>
       <c r="H5">
-        <v>0</v>
+        <v>500000</v>
       </c>
       <c r="I5">
-        <v>2000</v>
+        <v>9500</v>
       </c>
       <c r="J5">
-        <v>2000</v>
+        <v>10700</v>
       </c>
       <c r="K5">
-        <v>7910000</v>
+        <v>5530000</v>
       </c>
       <c r="L5">
         <v>0</v>
       </c>
       <c r="M5">
-        <v>2000</v>
+        <v>13000</v>
       </c>
       <c r="N5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="O5" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="P5">
-        <v>0</v>
+        <v>25588</v>
       </c>
       <c r="Q5">
-        <v>0</v>
+        <v>30049</v>
       </c>
       <c r="R5">
-        <v>0</v>
+        <v>7363</v>
       </c>
       <c r="S5">
-        <v>0</v>
+        <v>3780</v>
       </c>
       <c r="T5">
-        <v>0</v>
+        <v>5016</v>
       </c>
       <c r="U5">
-        <v>0</v>
+        <v>938</v>
       </c>
       <c r="V5">
-        <v>0</v>
+        <v>3456</v>
       </c>
       <c r="W5">
-        <v>0</v>
+        <v>4688</v>
       </c>
       <c r="X5">
-        <v>0</v>
+        <v>809</v>
       </c>
       <c r="Y5" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="6" spans="1:25">
@@ -1308,76 +1320,76 @@
         <v>29</v>
       </c>
       <c r="B6" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="C6" t="s">
         <v>43</v>
       </c>
       <c r="D6" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="E6" t="s">
         <v>61</v>
       </c>
       <c r="F6">
-        <v>1400000</v>
+        <v>6500000</v>
       </c>
       <c r="G6">
-        <v>1400000</v>
+        <v>6500000</v>
       </c>
       <c r="H6">
         <v>0</v>
       </c>
       <c r="I6">
-        <v>12500</v>
+        <v>2000</v>
       </c>
       <c r="J6">
-        <v>15500</v>
+        <v>2000</v>
       </c>
       <c r="K6">
-        <v>7486442</v>
+        <v>7910000</v>
       </c>
       <c r="L6">
         <v>0</v>
       </c>
       <c r="M6">
-        <v>15500</v>
+        <v>2000</v>
       </c>
       <c r="N6" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="O6" t="s">
         <v>82</v>
       </c>
       <c r="P6">
-        <v>10740898602</v>
+        <v>0</v>
       </c>
       <c r="Q6">
-        <v>13058877126</v>
+        <v>0</v>
       </c>
       <c r="R6">
-        <v>3506428302</v>
+        <v>0</v>
       </c>
       <c r="S6">
-        <v>1748628548</v>
+        <v>0</v>
       </c>
       <c r="T6">
-        <v>1115790858</v>
+        <v>0</v>
       </c>
       <c r="U6">
-        <v>191527654</v>
+        <v>0</v>
       </c>
       <c r="V6">
-        <v>1491084554</v>
+        <v>0</v>
       </c>
       <c r="W6">
-        <v>1185231988</v>
+        <v>0</v>
       </c>
       <c r="X6">
-        <v>219774608</v>
+        <v>0</v>
       </c>
       <c r="Y6" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
     </row>
     <row r="7" spans="1:25">
@@ -1385,123 +1397,123 @@
         <v>30</v>
       </c>
       <c r="B7" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C7" t="s">
         <v>44</v>
       </c>
       <c r="D7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E7" t="s">
         <v>62</v>
       </c>
       <c r="F7">
-        <v>751000</v>
+        <v>1400000</v>
       </c>
       <c r="G7">
-        <v>203700</v>
+        <v>1400000</v>
       </c>
       <c r="H7">
-        <v>547300</v>
+        <v>0</v>
       </c>
       <c r="I7">
-        <v>18000</v>
+        <v>12500</v>
       </c>
       <c r="J7">
-        <v>21000</v>
+        <v>15500</v>
       </c>
       <c r="K7">
-        <v>4330068</v>
+        <v>7486442</v>
       </c>
       <c r="L7">
         <v>0</v>
       </c>
       <c r="M7">
-        <v>21000</v>
+        <v>15500</v>
       </c>
       <c r="N7" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="O7" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="P7">
-        <v>0</v>
+        <v>10740898602</v>
       </c>
       <c r="Q7">
-        <v>0</v>
+        <v>13058877126</v>
       </c>
       <c r="R7">
-        <v>0</v>
+        <v>3506428302</v>
       </c>
       <c r="S7">
-        <v>0</v>
+        <v>1748628548</v>
       </c>
       <c r="T7">
-        <v>0</v>
+        <v>1115790858</v>
       </c>
       <c r="U7">
-        <v>0</v>
+        <v>191527654</v>
       </c>
       <c r="V7">
-        <v>0</v>
+        <v>1491084554</v>
       </c>
       <c r="W7">
-        <v>0</v>
+        <v>1185231988</v>
       </c>
       <c r="X7">
-        <v>0</v>
+        <v>219774608</v>
       </c>
       <c r="Y7" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
     </row>
     <row r="8" spans="1:25">
       <c r="A8" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="B8" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C8" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="D8" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E8" t="s">
         <v>63</v>
       </c>
       <c r="F8">
-        <v>5800000</v>
+        <v>751000</v>
       </c>
       <c r="G8">
-        <v>5800000</v>
+        <v>203700</v>
       </c>
       <c r="H8">
-        <v>0</v>
+        <v>547300</v>
       </c>
       <c r="I8">
-        <v>2000</v>
+        <v>18000</v>
       </c>
       <c r="J8">
-        <v>2000</v>
+        <v>21000</v>
       </c>
       <c r="K8">
-        <v>6100000</v>
+        <v>4330068</v>
       </c>
       <c r="L8">
         <v>0</v>
       </c>
       <c r="M8">
-        <v>2000</v>
+        <v>21000</v>
       </c>
       <c r="N8" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="O8" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="P8">
         <v>0</v>
@@ -1531,238 +1543,238 @@
         <v>0</v>
       </c>
       <c r="Y8" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
     </row>
     <row r="9" spans="1:25">
       <c r="A9" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="B9" t="s">
         <v>30</v>
       </c>
       <c r="C9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D9" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="E9" t="s">
         <v>64</v>
       </c>
       <c r="F9">
-        <v>1400000</v>
+        <v>5800000</v>
       </c>
       <c r="G9">
-        <v>1400000</v>
+        <v>5800000</v>
       </c>
       <c r="H9">
         <v>0</v>
       </c>
       <c r="I9">
-        <v>16000</v>
+        <v>2000</v>
       </c>
       <c r="J9">
-        <v>19000</v>
+        <v>2000</v>
       </c>
       <c r="K9">
-        <v>10000988</v>
+        <v>6100000</v>
       </c>
       <c r="L9">
         <v>0</v>
       </c>
       <c r="M9">
-        <v>16000</v>
+        <v>2000</v>
       </c>
       <c r="N9" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="O9" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="P9">
-        <v>72895458363</v>
+        <v>0</v>
       </c>
       <c r="Q9">
-        <v>72913766913</v>
+        <v>0</v>
       </c>
       <c r="R9">
-        <v>11230711680</v>
+        <v>0</v>
       </c>
       <c r="S9">
-        <v>-6524077412</v>
+        <v>0</v>
       </c>
       <c r="T9">
-        <v>-4556157069</v>
+        <v>0</v>
       </c>
       <c r="U9">
-        <v>-3633759729</v>
+        <v>0</v>
       </c>
       <c r="V9">
-        <v>-11528915410</v>
+        <v>0</v>
       </c>
       <c r="W9">
-        <v>-7978634776</v>
+        <v>0</v>
       </c>
       <c r="X9">
-        <v>-3801868433</v>
+        <v>0</v>
       </c>
       <c r="Y9" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="10" spans="1:25">
       <c r="A10" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B10" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="C10" t="s">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="D10" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="E10" t="s">
         <v>65</v>
       </c>
       <c r="F10">
-        <v>2234000</v>
+        <v>1400000</v>
       </c>
       <c r="G10">
-        <v>2234000</v>
+        <v>1400000</v>
       </c>
       <c r="H10">
         <v>0</v>
       </c>
       <c r="I10">
-        <v>7300</v>
+        <v>16000</v>
       </c>
       <c r="J10">
-        <v>8500</v>
+        <v>19000</v>
       </c>
       <c r="K10">
-        <v>14965620</v>
+        <v>10000988</v>
       </c>
       <c r="L10">
         <v>0</v>
       </c>
       <c r="M10">
-        <v>10000</v>
+        <v>16000</v>
       </c>
       <c r="N10" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O10" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="P10">
-        <v>1337894447</v>
+        <v>72895458363</v>
       </c>
       <c r="Q10">
-        <v>4495088983</v>
+        <v>72913766913</v>
       </c>
       <c r="R10">
-        <v>99398351</v>
+        <v>11230711680</v>
       </c>
       <c r="S10">
-        <v>-3330678562</v>
+        <v>-6524077412</v>
       </c>
       <c r="T10">
-        <v>-2905069801</v>
+        <v>-4556157069</v>
       </c>
       <c r="U10">
-        <v>-1314068310</v>
+        <v>-3633759729</v>
       </c>
       <c r="V10">
-        <v>-9735376868</v>
+        <v>-11528915410</v>
       </c>
       <c r="W10">
-        <v>-5043515600</v>
+        <v>-7978634776</v>
       </c>
       <c r="X10">
-        <v>-1257080998</v>
+        <v>-3801868433</v>
       </c>
       <c r="Y10" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
     </row>
     <row r="11" spans="1:25">
       <c r="A11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B11" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C11" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="D11" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="E11" t="s">
         <v>66</v>
       </c>
       <c r="F11">
-        <v>6000000</v>
+        <v>2234000</v>
       </c>
       <c r="G11">
-        <v>6000000</v>
+        <v>2234000</v>
       </c>
       <c r="H11">
         <v>0</v>
       </c>
       <c r="I11">
-        <v>2000</v>
+        <v>7300</v>
       </c>
       <c r="J11">
-        <v>2000</v>
+        <v>8500</v>
       </c>
       <c r="K11">
-        <v>6345000</v>
+        <v>14965620</v>
       </c>
       <c r="L11">
         <v>0</v>
       </c>
       <c r="M11">
-        <v>2000</v>
+        <v>10000</v>
       </c>
       <c r="N11" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="O11" t="s">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="P11">
-        <v>0</v>
+        <v>1337894447</v>
       </c>
       <c r="Q11">
-        <v>0</v>
+        <v>4495088983</v>
       </c>
       <c r="R11">
-        <v>0</v>
+        <v>99398351</v>
       </c>
       <c r="S11">
-        <v>0</v>
+        <v>-3330678562</v>
       </c>
       <c r="T11">
-        <v>0</v>
+        <v>-2905069801</v>
       </c>
       <c r="U11">
-        <v>0</v>
+        <v>-1314068310</v>
       </c>
       <c r="V11">
-        <v>0</v>
+        <v>-9735376868</v>
       </c>
       <c r="W11">
-        <v>0</v>
+        <v>-5043515600</v>
       </c>
       <c r="X11">
-        <v>0</v>
+        <v>-1257080998</v>
       </c>
       <c r="Y11" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
     </row>
     <row r="12" spans="1:25">
@@ -1773,19 +1785,19 @@
         <v>38</v>
       </c>
       <c r="C12" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D12" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="E12" t="s">
         <v>67</v>
       </c>
       <c r="F12">
-        <v>4000000</v>
+        <v>6000000</v>
       </c>
       <c r="G12">
-        <v>4000000</v>
+        <v>6000000</v>
       </c>
       <c r="H12">
         <v>0</v>
@@ -1797,7 +1809,7 @@
         <v>2000</v>
       </c>
       <c r="K12">
-        <v>4420000</v>
+        <v>6345000</v>
       </c>
       <c r="L12">
         <v>0</v>
@@ -1806,10 +1818,10 @@
         <v>2000</v>
       </c>
       <c r="N12" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="O12" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="P12">
         <v>0</v>
@@ -1839,7 +1851,84 @@
         <v>0</v>
       </c>
       <c r="Y12" t="s">
-        <v>95</v>
+        <v>98</v>
+      </c>
+    </row>
+    <row r="13" spans="1:25">
+      <c r="A13" t="s">
+        <v>33</v>
+      </c>
+      <c r="B13" t="s">
+        <v>38</v>
+      </c>
+      <c r="C13" t="s">
+        <v>46</v>
+      </c>
+      <c r="D13" t="s">
+        <v>56</v>
+      </c>
+      <c r="E13" t="s">
+        <v>68</v>
+      </c>
+      <c r="F13">
+        <v>4000000</v>
+      </c>
+      <c r="G13">
+        <v>4000000</v>
+      </c>
+      <c r="H13">
+        <v>0</v>
+      </c>
+      <c r="I13">
+        <v>2000</v>
+      </c>
+      <c r="J13">
+        <v>2000</v>
+      </c>
+      <c r="K13">
+        <v>4420000</v>
+      </c>
+      <c r="L13">
+        <v>0</v>
+      </c>
+      <c r="M13">
+        <v>2000</v>
+      </c>
+      <c r="N13" t="s">
+        <v>80</v>
+      </c>
+      <c r="O13" t="s">
+        <v>82</v>
+      </c>
+      <c r="P13">
+        <v>0</v>
+      </c>
+      <c r="Q13">
+        <v>0</v>
+      </c>
+      <c r="R13">
+        <v>0</v>
+      </c>
+      <c r="S13">
+        <v>0</v>
+      </c>
+      <c r="T13">
+        <v>0</v>
+      </c>
+      <c r="U13">
+        <v>0</v>
+      </c>
+      <c r="V13">
+        <v>0</v>
+      </c>
+      <c r="W13">
+        <v>0</v>
+      </c>
+      <c r="X13">
+        <v>0</v>
+      </c>
+      <c r="Y13" t="s">
+        <v>99</v>
       </c>
     </row>
   </sheetData>
@@ -1854,422 +1943,422 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="B2" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="C2" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="D2" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="E2" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="F2" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="B3" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="C3" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="D3" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="E3" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="F3" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="B4" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="C4" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="D4" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="E4" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="F4" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="B5" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="C5" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="D5" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="E5" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="F5" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="B6" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="C6" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="D6" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="E6" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="F6" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="B7" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="C7" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="D7" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="E7" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="F7" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="B8" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="C8" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="D8" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="E8" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="F8" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="B9" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="C9" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="D9" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="E9" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="F9" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="B10" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="C10" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="D10" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="E10" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="F10" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="B11" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="C11" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="D11" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="E11" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="F11" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="B12" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="C12" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="D12" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="E12" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="F12" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="B13" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="C13" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="D13" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="E13" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="F13" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="B14" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="C14" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="D14" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="E14" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="F14" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="B15" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="C15" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="D15" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="E15" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="F15" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B16" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="C16" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="D16" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="E16" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="F16" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="B17" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="C17" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="D17" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="E17" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="F17" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="B18" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="C18" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="D18" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="E18" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="F18" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B19" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C19" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="D19" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="E19" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="F19" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
     </row>
     <row r="20" spans="1:6">
       <c r="A20" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="B20" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="C20" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="D20" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="E20" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="F20" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="B21" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="C21" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D21" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="E21" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="F21" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
RPA datasets push 2024-09-25
</commit_message>
<xml_diff>
--- a/datasets/ib-strategy-data.xlsx
+++ b/datasets/ib-strategy-data.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="167">
   <si>
     <t>수요예측(시작일)</t>
   </si>
@@ -113,9 +113,6 @@
     <t>2024-07-15</t>
   </si>
   <si>
-    <t>2024-07-09</t>
-  </si>
-  <si>
     <t>2024-08-27</t>
   </si>
   <si>
@@ -128,9 +125,6 @@
     <t>2024-07-19</t>
   </si>
   <si>
-    <t>2024-07-10</t>
-  </si>
-  <si>
     <t>2024-08-16</t>
   </si>
   <si>
@@ -152,9 +146,6 @@
     <t>2024-08-13</t>
   </si>
   <si>
-    <t>2024-07-26</t>
-  </si>
-  <si>
     <t>대신</t>
   </si>
   <si>
@@ -206,9 +197,6 @@
     <t>아이빔테크놀로지</t>
   </si>
   <si>
-    <t>엔에이치스팩31호</t>
-  </si>
-  <si>
     <t>1152.85:1</t>
   </si>
   <si>
@@ -236,9 +224,6 @@
     <t>1011.50:1</t>
   </si>
   <si>
-    <t>1123.43 :1</t>
-  </si>
-  <si>
     <t>3.34%</t>
   </si>
   <si>
@@ -284,9 +269,6 @@
     <t>생체현미경, CRO 서비스</t>
   </si>
   <si>
-    <t>금융지원서비스업</t>
-  </si>
-  <si>
     <t>종목명</t>
   </si>
   <si>
@@ -308,6 +290,9 @@
     <t>위츠</t>
   </si>
   <si>
+    <t>토모큐브</t>
+  </si>
+  <si>
     <t>엠오티</t>
   </si>
   <si>
@@ -323,6 +308,9 @@
     <t>미트박스글로벌</t>
   </si>
   <si>
+    <t>에어레인</t>
+  </si>
+  <si>
     <t>에이치이엠파마(구.에이치이엠)</t>
   </si>
   <si>
@@ -359,12 +347,6 @@
     <t>쓰리빌리언</t>
   </si>
   <si>
-    <t>루미르</t>
-  </si>
-  <si>
-    <t>신한스팩14호</t>
-  </si>
-  <si>
     <t>2024.10.28~11.01</t>
   </si>
   <si>
@@ -398,15 +380,12 @@
     <t>2024.09.27~10.04</t>
   </si>
   <si>
-    <t>2024.09.26~10.04</t>
-  </si>
-  <si>
-    <t>2024.09.26~09.27</t>
-  </si>
-  <si>
     <t>5,300~6,400</t>
   </si>
   <si>
+    <t>10,900~13,400</t>
+  </si>
+  <si>
     <t>12,000~14,000</t>
   </si>
   <si>
@@ -422,6 +401,9 @@
     <t>23,000~28,500</t>
   </si>
   <si>
+    <t>16,000~18,500</t>
+  </si>
+  <si>
     <t>16,400~19,000</t>
   </si>
   <si>
@@ -455,9 +437,6 @@
     <t>4,500~6,500</t>
   </si>
   <si>
-    <t>16,500~20,500</t>
-  </si>
-  <si>
     <t>15900</t>
   </si>
   <si>
@@ -476,6 +455,9 @@
     <t>23000</t>
   </si>
   <si>
+    <t>19200</t>
+  </si>
+  <si>
     <t>11430</t>
   </si>
   <si>
@@ -500,15 +482,12 @@
     <t>11000</t>
   </si>
   <si>
-    <t>49500</t>
-  </si>
-  <si>
-    <t>10000</t>
-  </si>
-  <si>
     <t>신한투자증권</t>
   </si>
   <si>
+    <t>대신증권</t>
+  </si>
+  <si>
     <t>한국투자증권</t>
   </si>
   <si>
@@ -524,10 +503,10 @@
     <t>미래에셋증권</t>
   </si>
   <si>
+    <t>신영증권</t>
+  </si>
+  <si>
     <t>KB증권</t>
-  </si>
-  <si>
-    <t>대신증권</t>
   </si>
   <si>
     <t>NH투자증권,KB증권,신한투자증권,키움증권</t>
@@ -894,7 +873,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Y11"/>
+  <dimension ref="A1:Y10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:25">
@@ -982,13 +961,13 @@
         <v>27</v>
       </c>
       <c r="C2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D2" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="E2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F2">
         <v>3000000</v>
@@ -1015,10 +994,10 @@
         <v>7000</v>
       </c>
       <c r="N2" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="O2" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="P2">
         <v>5436813</v>
@@ -1048,7 +1027,7 @@
         <v>-801640</v>
       </c>
       <c r="Y2" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
     </row>
     <row r="3" spans="1:25">
@@ -1056,16 +1035,16 @@
         <v>26</v>
       </c>
       <c r="B3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C3" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D3" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="E3" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="F3">
         <v>7950000</v>
@@ -1092,10 +1071,10 @@
         <v>2000</v>
       </c>
       <c r="N3" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="O3" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="P3">
         <v>0</v>
@@ -1125,7 +1104,7 @@
         <v>0</v>
       </c>
       <c r="Y3" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
     </row>
     <row r="4" spans="1:25">
@@ -1133,16 +1112,16 @@
         <v>27</v>
       </c>
       <c r="B4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D4" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="E4" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="F4">
         <v>1566800</v>
@@ -1169,10 +1148,10 @@
         <v>15300</v>
       </c>
       <c r="N4" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="O4" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="P4">
         <v>7367362</v>
@@ -1202,7 +1181,7 @@
         <v>-2903334</v>
       </c>
       <c r="Y4" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
     </row>
     <row r="5" spans="1:25">
@@ -1210,16 +1189,16 @@
         <v>28</v>
       </c>
       <c r="B5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C5" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="D5" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="E5" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="F5">
         <v>1000000</v>
@@ -1246,10 +1225,10 @@
         <v>13000</v>
       </c>
       <c r="N5" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="O5" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="P5">
         <v>25588</v>
@@ -1279,7 +1258,7 @@
         <v>809</v>
       </c>
       <c r="Y5" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
     </row>
     <row r="6" spans="1:25">
@@ -1287,16 +1266,16 @@
         <v>29</v>
       </c>
       <c r="B6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C6" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D6" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="E6" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="F6">
         <v>6500000</v>
@@ -1323,10 +1302,10 @@
         <v>2000</v>
       </c>
       <c r="N6" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="O6" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="P6">
         <v>0</v>
@@ -1356,7 +1335,7 @@
         <v>0</v>
       </c>
       <c r="Y6" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
     </row>
     <row r="7" spans="1:25">
@@ -1367,13 +1346,13 @@
         <v>29</v>
       </c>
       <c r="C7" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D7" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="E7" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="F7">
         <v>1400000</v>
@@ -1400,40 +1379,40 @@
         <v>15500</v>
       </c>
       <c r="N7" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="O7" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="P7">
-        <v>0</v>
+        <v>10740898602</v>
       </c>
       <c r="Q7">
-        <v>0</v>
+        <v>13058877126</v>
       </c>
       <c r="R7">
-        <v>0</v>
+        <v>3506428302</v>
       </c>
       <c r="S7">
-        <v>0</v>
+        <v>1748628548</v>
       </c>
       <c r="T7">
-        <v>0</v>
+        <v>1115790858</v>
       </c>
       <c r="U7">
-        <v>0</v>
+        <v>191527654</v>
       </c>
       <c r="V7">
-        <v>0</v>
+        <v>1491084554</v>
       </c>
       <c r="W7">
-        <v>0</v>
+        <v>1185231988</v>
       </c>
       <c r="X7">
-        <v>0</v>
+        <v>219774608</v>
       </c>
       <c r="Y7" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
     </row>
     <row r="8" spans="1:25">
@@ -1444,13 +1423,13 @@
         <v>27</v>
       </c>
       <c r="C8" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D8" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="E8" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="F8">
         <v>751000</v>
@@ -1477,10 +1456,10 @@
         <v>21000</v>
       </c>
       <c r="N8" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="O8" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="P8">
         <v>0</v>
@@ -1510,7 +1489,7 @@
         <v>0</v>
       </c>
       <c r="Y8" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
     </row>
     <row r="9" spans="1:25">
@@ -1521,13 +1500,13 @@
         <v>30</v>
       </c>
       <c r="C9" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D9" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="E9" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="F9">
         <v>5800000</v>
@@ -1554,10 +1533,10 @@
         <v>2000</v>
       </c>
       <c r="N9" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="O9" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="P9">
         <v>0</v>
@@ -1587,7 +1566,7 @@
         <v>0</v>
       </c>
       <c r="Y9" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
     </row>
     <row r="10" spans="1:25">
@@ -1595,16 +1574,16 @@
         <v>31</v>
       </c>
       <c r="B10" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C10" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D10" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="E10" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="F10">
         <v>2234000</v>
@@ -1631,10 +1610,10 @@
         <v>10000</v>
       </c>
       <c r="N10" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="O10" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="P10">
         <v>1337894447</v>
@@ -1664,84 +1643,7 @@
         <v>-1257080998</v>
       </c>
       <c r="Y10" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="11" spans="1:25">
-      <c r="A11" t="s">
-        <v>32</v>
-      </c>
-      <c r="B11" t="s">
-        <v>37</v>
-      </c>
-      <c r="C11" t="s">
-        <v>45</v>
-      </c>
-      <c r="D11" t="s">
-        <v>48</v>
-      </c>
-      <c r="E11" t="s">
-        <v>63</v>
-      </c>
-      <c r="F11">
-        <v>6000000</v>
-      </c>
-      <c r="G11">
-        <v>6000000</v>
-      </c>
-      <c r="H11">
-        <v>0</v>
-      </c>
-      <c r="I11">
-        <v>2000</v>
-      </c>
-      <c r="J11">
-        <v>2000</v>
-      </c>
-      <c r="K11">
-        <v>6345000</v>
-      </c>
-      <c r="L11">
-        <v>0</v>
-      </c>
-      <c r="M11">
-        <v>2000</v>
-      </c>
-      <c r="N11" t="s">
-        <v>73</v>
-      </c>
-      <c r="O11" t="s">
-        <v>75</v>
-      </c>
-      <c r="P11">
-        <v>0</v>
-      </c>
-      <c r="Q11">
-        <v>0</v>
-      </c>
-      <c r="R11">
-        <v>0</v>
-      </c>
-      <c r="S11">
-        <v>0</v>
-      </c>
-      <c r="T11">
-        <v>0</v>
-      </c>
-      <c r="U11">
-        <v>0</v>
-      </c>
-      <c r="V11">
-        <v>0</v>
-      </c>
-      <c r="W11">
-        <v>0</v>
-      </c>
-      <c r="X11">
-        <v>0</v>
-      </c>
-      <c r="Y11" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
     </row>
   </sheetData>
@@ -1756,422 +1658,422 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="B2" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="C2" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="D2" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="E2" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="F2" t="s">
-        <v>163</v>
+        <v>155</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="B3" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="C3" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
       <c r="D3" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="E3" t="s">
-        <v>148</v>
+        <v>70</v>
       </c>
       <c r="F3" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="B4" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="C4" t="s">
-        <v>131</v>
+        <v>123</v>
       </c>
       <c r="D4" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="E4" t="s">
-        <v>149</v>
+        <v>141</v>
       </c>
       <c r="F4" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="B5" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="C5" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
       <c r="D5" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="E5" t="s">
-        <v>150</v>
+        <v>142</v>
       </c>
       <c r="F5" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="B6" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="C6" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
       <c r="D6" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="E6" t="s">
-        <v>151</v>
+        <v>143</v>
       </c>
       <c r="F6" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="B7" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="C7" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="D7" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="E7" t="s">
-        <v>152</v>
+        <v>144</v>
       </c>
       <c r="F7" t="s">
-        <v>168</v>
+        <v>160</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="B8" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="C8" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="D8" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="E8" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="F8" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="B9" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="C9" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D9" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="E9" t="s">
-        <v>75</v>
+        <v>146</v>
       </c>
       <c r="F9" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="B10" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="C10" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="D10" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="E10" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="F10" t="s">
-        <v>170</v>
+        <v>155</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="B11" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="C11" t="s">
-        <v>137</v>
+        <v>123</v>
       </c>
       <c r="D11" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="E11" t="s">
-        <v>155</v>
+        <v>70</v>
       </c>
       <c r="F11" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="B12" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="C12" t="s">
-        <v>138</v>
+        <v>130</v>
       </c>
       <c r="D12" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="E12" t="s">
-        <v>75</v>
+        <v>148</v>
       </c>
       <c r="F12" t="s">
-        <v>168</v>
+        <v>156</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="B13" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="C13" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="D13" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="E13" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="F13" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="B14" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="C14" t="s">
-        <v>140</v>
+        <v>132</v>
       </c>
       <c r="D14" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="E14" t="s">
-        <v>157</v>
+        <v>70</v>
       </c>
       <c r="F14" t="s">
-        <v>171</v>
+        <v>161</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="B15" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="C15" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="D15" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="E15" t="s">
-        <v>75</v>
+        <v>150</v>
       </c>
       <c r="F15" t="s">
-        <v>170</v>
+        <v>157</v>
       </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="B16" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="C16" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
       <c r="D16" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="E16" t="s">
-        <v>158</v>
+        <v>151</v>
       </c>
       <c r="F16" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="B17" t="s">
-        <v>125</v>
+        <v>118</v>
       </c>
       <c r="C17" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="D17" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="E17" t="s">
-        <v>159</v>
+        <v>70</v>
       </c>
       <c r="F17" t="s">
-        <v>173</v>
+        <v>156</v>
       </c>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="B18" t="s">
-        <v>125</v>
+        <v>118</v>
       </c>
       <c r="C18" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
       <c r="D18" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="E18" t="s">
-        <v>160</v>
+        <v>152</v>
       </c>
       <c r="F18" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="B19" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="C19" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="D19" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="E19" t="s">
-        <v>75</v>
+        <v>153</v>
       </c>
       <c r="F19" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
     <row r="20" spans="1:6">
       <c r="A20" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="B20" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="C20" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="D20" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="E20" t="s">
+        <v>154</v>
+      </c>
+      <c r="F20" t="s">
         <v>161</v>
-      </c>
-      <c r="F20" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="B21" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="C21" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="D21" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="E21" t="s">
-        <v>162</v>
+        <v>70</v>
       </c>
       <c r="F21" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
     </row>
   </sheetData>

</xml_diff>